<commit_message>
Revise the general education writer allocation
Per the Vice Dean, 13 Sep 2026: religion to Ilag and Maglalang, PATH-FIT to
Calma and Mequiabas, ethics and mathematics to Manuel. Aquino, Agnes M. moved
out of the GE pool to write BEED/BSED major courses under item 79 instead,
leaving seven writers for the 20 courses. NSTP 1 and 2 now sit with different
writers - flagged on both cards and on items 74 and 79.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RjXH6Pg8FcbrhQUKSMaVjy
</commit_message>
<xml_diff>
--- a/CHED 3-Year Trimester Application Tracker.xlsx
+++ b/CHED 3-Year Trimester Application Tracker.xlsx
@@ -657,7 +657,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="30" customHeight="1" s="31">
       <c r="A4" s="1" t="inlineStr">
         <is>
@@ -3761,7 +3760,7 @@
       </c>
       <c r="E84" s="3" t="inlineStr">
         <is>
-          <t>General Education Syllabi Pool (Ilag, Maglalang, Calma, Manuel, Tolosa, Aquino (Agnes), Mequiabas, Jamlang); Vice Dean Ken Gie Anthony G. Cruel (GE code harmonisation, Open Item 7); all 8 Program Chairs (recipients)</t>
+          <t>General Education Syllabi Pool — 7 writers (Ilag, Maglalang, Calma, Mequiabas, Manuel, Tolosa, Jamlang); Vice Dean Ken Gie Anthony G. Cruel (GE code harmonisation); all 8 Program Chairs (recipients)</t>
         </is>
       </c>
       <c r="F84" s="4" t="n">
@@ -3777,7 +3776,7 @@
       </c>
       <c r="I84" s="7" t="inlineStr">
         <is>
-          <t>POOL LEAD NAMED 9 Sep 2026: Chair Kent E. Garcia convenes the General Education Syllabi Pool. The pool writes the 20 shared GE, PATH-FIT, NSTP and CLE courses ONCE for all 8 programmes, so its output feeds items 19-20, 25-26, 31-32, 37-38, 43-44, 49-50, 55-56 and 61-62 — sixteen rows owned by five different Chairs. THE LEAD'S SPECIFIC TASKS: (1) publish the allocation — which of the 8 writers takes which of the 20 courses; (2) issue one common syllabus template carrying the assessment scheme (midterm, final, one monthly assessment, plus quizzes) and the 14-week / 56-hour basis; (3) set internal hand-in dates ahead of the 9 Oct descriptions and 16 Oct syllabi; (4) collect the finished set and hand ONE copy to all 8 Programme Chairs; (5) report slippage to the Vice Dean weekly. BLOCKED BY OPEN ITEM 7: the GE course codes do not match across programmes — only about 13 of the 20 match cleanly — and the pool cannot write once-for-all until they are harmonised. Resolve that first or the allocation will be wrong. The Chair convenes and reports; each Programme Chair still answers for their own 7.3 and 7.4 rows.</t>
+          <t>POOL LEAD: Chair Kent E. Garcia (named 9 Sep 2026). ALLOCATION REVISED 13 Sep 2026 by direction of the Vice Dean — all 20 courses are assigned by name across SEVEN writers (Aquino, Agnes M. was moved out of the pool on the same date to write BEED/BSED major courses under item 79 instead). Ilag: REL-GEC, CLE 1, STS-GEC. Maglalang: CLE 2, HIS-GEC, RIZ-GEC. Calma: PATH-FIT 1, PATH-FIT 2, NSTP 1. Mequiabas: PATH-FIT 3, PATH-FIT 4, NSTP 2. Manuel: ETH-GEC, MAT-GEC, BL-GEC. Tolosa: ART-GEC, COM-GEC, US-GEC. Jamlang: CON-GEC, ITE-GEC — two only, on the heaviest teaching load in the pool at 27 units over 5 preps. Each writer produces the description AND the syllabus per course. THE LEAD'S TASKS: issue one common syllabus template carrying the assessment scheme and the 14-week / 56-hour basis; set internal hand-in dates ahead of 9 Oct and 16 Oct; hand one finished set to all 8 Chairs; report slippage weekly to the Vice Dean. WATCH: NSTP 1 is the prerequisite of NSTP 2 and they now sit with different writers — Calma and Mequiabas must agree the two syllabi between them. STILL BLOCKED BY OPEN ITEM 7 — the GE course codes do not match across programmes, so the allocation is not final until they are harmonised. He convenes and reports; each Programme Chair still answers for their own 7.3 and 7.4 rows.</t>
         </is>
       </c>
     </row>
@@ -3966,7 +3965,7 @@
       </c>
       <c r="E89" s="3" t="inlineStr">
         <is>
-          <t>The six Teacher Education full-time faculty not in the GE pool (Ablaya, Cajucom, Delos Reyes, Germino, Sta. Cruz, Villamayor); Vice Dean Ken Gie Anthony G. Cruel</t>
+          <t>The seven Teacher Education full-time faculty not in the GE pool (Ablaya, Aquino (Agnes), Cajucom, Delos Reyes, Germino, Sta. Cruz, Villamayor); Vice Dean Ken Gie Anthony G. Cruel</t>
         </is>
       </c>
       <c r="F89" s="4" t="n">
@@ -3982,7 +3981,7 @@
       </c>
       <c r="I89" s="7" t="inlineStr">
         <is>
-          <t>The eight Teacher Education faculty in the General Education Syllabi Pool are writing 20 courses for the whole college under item 74 and are deliberately EXCLUDED from this allocation. That leaves six writers for the BEED and BSED major courses. Sta. Cruz also carries library items 66 to 69 on top of a 27-unit load — weight her share accordingly. Internal hand-in: descriptions 9 Oct 2026, syllabi 16 Oct 2026. Feeds items 55 and 56 (BEED) and 61 and 62 (BSED).</t>
+          <t>The seven Teacher Education faculty in the General Education Syllabi Pool are writing 20 courses for the whole college under item 74 and are deliberately EXCLUDED from this allocation. SEVEN writers remain for the BEED and BSED major courses — Aquino, Agnes M. was moved out of the GE pool on 13 Sep 2026 by direction of the Vice Dean and joins this group, on the heaviest prep count in the department at 7. Sta. Cruz also carries library items 66 to 69 on top of a 27-unit load — weight her share accordingly. Internal hand-in: descriptions 9 Oct 2026, syllabi 16 Oct 2026. Feeds items 55 and 56 (BEED) and 61 and 62 (BSED).</t>
         </is>
       </c>
     </row>
@@ -4098,7 +4097,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="30" customHeight="1" s="31">
       <c r="A4" s="1" t="inlineStr">
         <is>
@@ -4940,7 +4938,7 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>General Education Syllabi Pool writer (item 74) — writes the course description AND the OBE syllabus for 2 courses: NSTP 1 Civic Welfare Training Service 1; NSTP 2 Civic Welfare Training Service 2. 4 documents, one set serving all 8 programmes. To Chair K. Garcia: descriptions 9 Oct, syllabi 16 Oct 2026. Also Curriculum &amp; Syllabi — BEED/BSED (not allocated BEED/BSED major courses under item 79 while carrying this pool load).  [FT, 24 units, 7 preps this semester]</t>
+          <t>Curriculum &amp; Syllabi — BEED/BSED. Writes the course descriptions and OBE syllabi for the BEED and BSED major courses allocated to her under item 79, due 25 Sep 2026. Moved out of the General Education Syllabi Pool on 13 Sep 2026 so the major-course load is not carried on top of the college-wide general education work.  [FT, 24 units, 7 preps this semester]</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
@@ -4950,7 +4948,7 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>17 items: #19–20, 25–26, 31–32, 37–38, 43–44, 49–50, 55–56, 61–62, 74</t>
+          <t>5 items: #55–56, 61–62, 79</t>
         </is>
       </c>
       <c r="E40" s="4">
@@ -4992,7 +4990,7 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>General Education Syllabi Pool writer (item 74) — writes the course description AND the OBE syllabus for 3 courses: US-GEC Understanding the Self; ART-GEC Art Appreciation; COM-GEC Purposive Communication. 6 documents, one set serving all 8 programmes. To Chair K. Garcia: descriptions 9 Oct, syllabi 16 Oct 2026. Also Curriculum &amp; Syllabi — BEED/BSED (not allocated BEED/BSED major courses under item 79 while carrying this pool load).  [FT, 24 units, 4 preps this semester]</t>
+          <t>General Education Syllabi Pool writer (item 74) — writes the course description AND the OBE syllabus for 3 courses, one set serving all 8 programmes: PATH-FIT 1 Movement Competency Training; PATH-FIT 2 Exercise-Based Fitness Activities; NSTP 1 Civic Welfare Training Service 1. 6 documents. To Chair K. Garcia: descriptions 9 Oct, syllabi 16 Oct 2026. Also Curriculum &amp; Syllabi — BEED/BSED (not allocated BEED/BSED major courses under item 79 while carrying this pool load).  [FT, 24 units, 4 preps this semester]</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
@@ -5070,7 +5068,7 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>General Education Syllabi Pool writer (item 74) — writes the course description AND the OBE syllabus for 3 courses: MAT-GEC Mathematics in the Modern World; BL-GEC Business Logic; STS-GEC Science, Technology and Society. 6 documents, one set serving all 8 programmes. To Chair K. Garcia: descriptions 9 Oct, syllabi 16 Oct 2026. Also Curriculum &amp; Syllabi — BEED/BSED (not allocated BEED/BSED major courses under item 79 while carrying this pool load).  [FT, 21 units, 3 preps this semester]</t>
+          <t>General Education Syllabi Pool writer (item 74) — writes the course description AND the OBE syllabus for 3 courses, one set serving all 8 programmes: REL-GEC Religion, Religious Experience and Spirituality; CLE 1 Church and Salvation History; STS-GEC Science, Technology and Society. 6 documents. To Chair K. Garcia: descriptions 9 Oct, syllabi 16 Oct 2026. Also Curriculum &amp; Syllabi — BEED/BSED (not allocated BEED/BSED major courses under item 79 while carrying this pool load).  [FT, 21 units, 3 preps this semester]</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
@@ -5096,7 +5094,7 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>General Education Syllabi Pool writer (item 74) — writes the course description AND the OBE syllabus for 2 courses: PATH-FIT 3 Dance; PATH-FIT 4 Sports. 4 documents, one set serving all 8 programmes. To Chair K. Garcia: descriptions 9 Oct, syllabi 16 Oct 2026. Also Curriculum &amp; Syllabi — BEED/BSED (not allocated BEED/BSED major courses under item 79 while carrying this pool load).  [FT, 27 units, 5 preps this semester]</t>
+          <t>General Education Syllabi Pool writer (item 74) — writes the course description AND the OBE syllabus for 2 courses, one set serving all 8 programmes: CON-GEC The Contemporary World; ITE-GEC Living in the I.T. Era. 4 documents. To Chair K. Garcia: descriptions 9 Oct, syllabi 16 Oct 2026. Also Curriculum &amp; Syllabi — BEED/BSED (not allocated BEED/BSED major courses under item 79 while carrying this pool load).  [FT, 27 units, 5 preps this semester]</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
@@ -5122,7 +5120,7 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>General Education Syllabi Pool writer (item 74) — writes the course description AND the OBE syllabus for 3 courses: HIS-GEC Readings in Philippine History; RIZ-GEC Rizal's Life and Works; CON-GEC The Contemporary World. 6 documents, one set serving all 8 programmes. To Chair K. Garcia: descriptions 9 Oct, syllabi 16 Oct 2026. Also Curriculum &amp; Syllabi — BEED/BSED (not allocated BEED/BSED major courses under item 79 while carrying this pool load).  [FT, 24 units, 3 preps this semester]</t>
+          <t>General Education Syllabi Pool writer (item 74) — writes the course description AND the OBE syllabus for 3 courses, one set serving all 8 programmes: CLE 2 Evangelism and Discipleship; HIS-GEC Readings in Philippine History; RIZ-GEC Rizal's Life and Works. 6 documents. To Chair K. Garcia: descriptions 9 Oct, syllabi 16 Oct 2026. Also Curriculum &amp; Syllabi — BEED/BSED (not allocated BEED/BSED major courses under item 79 while carrying this pool load).  [FT, 24 units, 3 preps this semester]</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
@@ -5148,7 +5146,7 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>General Education Syllabi Pool writer (item 74) — writes the course description AND the OBE syllabus for 3 courses: REL-GEC Religion, Religious Experience and Spirituality; CLE 1 Church and Salvation History; CLE 2 Evangelism and Discipleship. 6 documents, one set serving all 8 programmes. To Chair K. Garcia: descriptions 9 Oct, syllabi 16 Oct 2026. Also Curriculum &amp; Syllabi — BEED/BSED (not allocated BEED/BSED major courses under item 79 while carrying this pool load).  [FT, 24 units, 4 preps this semester]</t>
+          <t>General Education Syllabi Pool writer (item 74) — writes the course description AND the OBE syllabus for 3 courses, one set serving all 8 programmes: ETH-GEC Ethics; MAT-GEC Mathematics in the Modern World; BL-GEC Business Logic. 6 documents. To Chair K. Garcia: descriptions 9 Oct, syllabi 16 Oct 2026. Also Curriculum &amp; Syllabi — BEED/BSED (not allocated BEED/BSED major courses under item 79 while carrying this pool load).  [FT, 24 units, 4 preps this semester]</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
@@ -5174,7 +5172,7 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>General Education Syllabi Pool writer (item 74) — writes the course description AND the OBE syllabus for 2 courses: ETH-GEC Ethics; ITE-GEC Living in the I.T. Era. 4 documents, one set serving all 8 programmes. To Chair K. Garcia: descriptions 9 Oct, syllabi 16 Oct 2026. Also Curriculum &amp; Syllabi — BEED/BSED (not allocated BEED/BSED major courses under item 79 while carrying this pool load).  [FT, 26 units, 4 preps this semester]</t>
+          <t>General Education Syllabi Pool writer (item 74) — writes the course description AND the OBE syllabus for 3 courses, one set serving all 8 programmes: PATH-FIT 3 Dance; PATH-FIT 4 Sports; NSTP 2 Civic Welfare Training Service 2. 6 documents. To Chair K. Garcia: descriptions 9 Oct, syllabi 16 Oct 2026. Also Curriculum &amp; Syllabi — BEED/BSED (not allocated BEED/BSED major courses under item 79 while carrying this pool load).  [FT, 26 units, 4 preps this semester]</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
@@ -5226,7 +5224,7 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>General Education Syllabi Pool writer (item 74) — writes the course description AND the OBE syllabus for 2 courses: PATH-FIT 1 Movement Competency Training; PATH-FIT 2 Exercise-Based Fitness Activities. 4 documents, one set serving all 8 programmes. To Chair K. Garcia: descriptions 9 Oct, syllabi 16 Oct 2026. Also Curriculum &amp; Syllabi — BEED/BSED (not allocated BEED/BSED major courses under item 79 while carrying this pool load).  [FT, 24 units, 5 preps this semester]</t>
+          <t>General Education Syllabi Pool writer (item 74) — writes the course description AND the OBE syllabus for 3 courses, one set serving all 8 programmes: ART-GEC Art Appreciation; COM-GEC Purposive Communication; US-GEC Understanding the Self. 6 documents. To Chair K. Garcia: descriptions 9 Oct, syllabi 16 Oct 2026. Also Curriculum &amp; Syllabi — BEED/BSED (not allocated BEED/BSED major courses under item 79 while carrying this pool load).  [FT, 24 units, 5 preps this semester]</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
@@ -5309,7 +5307,6 @@
         </is>
       </c>
     </row>
-    <row r="56"/>
     <row r="57" ht="15" customHeight="1" s="31">
       <c r="A57" s="35" t="inlineStr">
         <is>
@@ -5367,7 +5364,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="24" customHeight="1" s="31">
       <c r="A4" s="16" t="inlineStr">
         <is>
@@ -6131,7 +6127,7 @@
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>THE MAIN BORROWING. LEAD: Programme Chair Kent E. Garcia (named 9 Sep 2026). The 20 general education, PATH-FIT, NSTP and CLE courses are common to all 8 programmes, so they are written ONCE for the whole college instead of eight times — removing roughly 140 duplicated syllabi. Drawn from Teacher Education, the only department with surplus full-time capacity. WRITER ALLOCATION, issued 13 Sep 2026 — each writer produces the course description AND the OBE syllabus for every course listed: Ilag, Ferdinand T. — MAT-GEC Mathematics in the Modern World, BL-GEC Business Logic, STS-GEC Science, Technology and Society. Maglalang, Danica — HIS-GEC Readings in Philippine History, RIZ-GEC Rizal's Life and Works, CON-GEC The Contemporary World. Calma, Shiela Mae C. — US-GEC Understanding the Self, ART-GEC Art Appreciation, COM-GEC Purposive Communication. Manuel, Consuelo V., Dr. — REL-GEC Religion, Religious Experience and Spirituality, CLE 1 Church and Salvation History, CLE 2 Evangelism and Discipleship. Mequiabas, Meah — ETH-GEC Ethics, ITE-GEC Living in the I.T. Era. Tolosa, Nenita — PATH-FIT 1 Movement Competency Training, PATH-FIT 2 Exercise-Based Fitness Activities. Jamlang, Jamie A. — PATH-FIT 3 Dance, PATH-FIT 4 Sports. Aquino, Agnes M., Dr. — NSTP 1 and NSTP 2 Civic Welfare Training Service. Three courses each to the four lightest teaching loads, two each to the four heaviest. Internal hand-in to the lead: descriptions 9 Oct 2026, syllabi 16 Oct 2026. CAVEAT: the codes above are the BSA and BSAIS spellings taken from the prospectus in hand. Open Item 7 — general education course codes do not match across programmes — must be closed before this allocation is final, and it blocks item 74. The eight pool writers are deliberately EXCLUDED from the BEED and BSED specialised allocation in item 79.</t>
+          <t>THE MAIN BORROWING. LEAD: Programme Chair Kent E. Garcia (named 9 Sep 2026). The 20 general education, PATH-FIT, NSTP and CLE courses are common to all 8 programmes, so they are written ONCE for the whole college instead of eight times — removing roughly 140 duplicated syllabi. Drawn from Teacher Education, the only department with surplus full-time capacity. WRITER ALLOCATION, revised 13 Sep 2026 — each writer produces the course description AND the OBE syllabus for every course listed: Ilag, Ferdinand T. — REL-GEC Religion, Religious Experience and Spirituality, CLE 1 Church and Salvation History, STS-GEC Science, Technology and Society. Maglalang, Danica — CLE 2 Evangelism and Discipleship, HIS-GEC Readings in Philippine History, RIZ-GEC Rizal's Life and Works. Calma, Shiela Mae C. — PATH-FIT 1 Movement Competency Training, PATH-FIT 2 Exercise-Based Fitness Activities, NSTP 1. Mequiabas, Meah — PATH-FIT 3 Dance, PATH-FIT 4 Sports, NSTP 2. Manuel, Consuelo V., Dr. — ETH-GEC Ethics, MAT-GEC Mathematics in the Modern World, BL-GEC Business Logic. Tolosa, Nenita — ART-GEC Art Appreciation, COM-GEC Purposive Communication, US-GEC Understanding the Self. Jamlang, Jamie A. — CON-GEC The Contemporary World, ITE-GEC Living in the I.T. Era (two only, on the heaviest teaching load in the pool). AQUINO, AGNES M., Dr. WAS MOVED OUT OF THIS POOL on 13 Sep 2026 by direction of the Vice Dean — she writes BEED/BSED major courses under item 79 instead, and the pool went from eight writers to seven. Internal hand-in to the lead: descriptions 9 Oct 2026, syllabi 16 Oct 2026. CAVEATS: the codes above are the BSA and BSAIS spellings and Open Item 7 must close before the allocation is final — it blocks item 74; and NSTP 1 is the prerequisite of NSTP 2, now with different writers, so Calma and Mequiabas must agree the pair.</t>
         </is>
       </c>
     </row>
@@ -6460,7 +6456,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="30" customHeight="1" s="31">
       <c r="A4" s="1" t="inlineStr">
         <is>
@@ -8242,20 +8237,24 @@
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
-          <t>Curriculum &amp; Syllabi — BEED/BSED; General Education Syllabi Pool (college-wide)</t>
+          <t>Curriculum &amp; Syllabi — BEED/BSED</t>
         </is>
       </c>
       <c r="I41" s="3" t="inlineStr">
         <is>
-          <t>GENERAL EDUCATION SYLLABI POOL (tracker item 74) — write the COURSE DESCRIPTION and the OBE SYLLABUS for 2 allocated courses, one set serving all 8 programmes: NSTP 1 Civic Welfare Training Service 1; NSTP 2 Civic Welfare Training Service 2. 4 documents in total. Common syllabus template: 14-week trimester, 56 hours per 3-unit course, two examinations (midterm and final) plus one required monthly assessment and regular quizzes. Hand in to Chair Kent E. Garcia: descriptions 9 Oct 2026, syllabi 16 Oct 2026. Course codes are the BSA/BSAIS spellings — reconcile with your own programme's codes once Open Item 7 is closed. Not included in the BEED/BSED specialised allocation (item 79) while carrying this pool load. Records obligation on top, compulsory for all faculty: certified true copy of Transcript of Records and signed contract to HR by 30 Oct 2026 (items 12–13).</t>
+          <t>PROGRAMME-SPECIALISED COURSES — BEED and BSED. Write the COURSE DESCRIPTION and the OBE SYLLABUS for the BEED and BSED major courses allocated to you by Chair K. Garcia. The allocation naming your specific courses is tracked as item 79, due 25 Sep 2026. Common syllabus template: 14-week trimester, 56 hours per 3-unit course, two examinations (midterm and final) plus one required monthly assessment and regular quizzes. Hand in to your Chair: descriptions 9 Oct 2026, syllabi 16 Oct 2026. Feeds tracker items 55 and 56 (BEED) and 61 and 62 (BSED). MOVED OUT OF THE GENERAL EDUCATION SYLLABI POOL on 13 Sep 2026 by direction of the Vice Dean, so that this major-course load is not carried on top of the college-wide general education work — you hold the heaviest prep count in the department at 7. Records obligation on top, compulsory for all faculty: certified true copy of Transcript of Records and signed contract to HR by 30 Oct 2026 (items 12–13).</t>
         </is>
       </c>
       <c r="J41" s="21" t="inlineStr">
         <is>
-          <t>#19–20, 25–26, 31–32, 37–38, 43–44, 49–50, 55–56, 61–62</t>
-        </is>
-      </c>
-      <c r="K41" s="3" t="n"/>
+          <t>#55–56, 61–62, 79</t>
+        </is>
+      </c>
+      <c r="K41" s="3" t="inlineStr">
+        <is>
+          <t>Moved out of the General Education Syllabi Pool 13 Sep 2026 by direction of the Vice Dean — she writes BEED/BSED major courses instead. The pool now has 7 writers.</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="23.75" customHeight="1" s="31">
       <c r="A42" s="2" t="n">
@@ -8333,7 +8332,7 @@
       </c>
       <c r="I43" s="3" t="inlineStr">
         <is>
-          <t>GENERAL EDUCATION SYLLABI POOL (tracker item 74) — write the COURSE DESCRIPTION and the OBE SYLLABUS for 3 allocated courses, one set serving all 8 programmes: US-GEC Understanding the Self; ART-GEC Art Appreciation; COM-GEC Purposive Communication. 6 documents in total. Common syllabus template: 14-week trimester, 56 hours per 3-unit course, two examinations (midterm and final) plus one required monthly assessment and regular quizzes. Hand in to Chair Kent E. Garcia: descriptions 9 Oct 2026, syllabi 16 Oct 2026. Course codes are the BSA/BSAIS spellings — reconcile with your own programme's codes once Open Item 7 is closed. Not included in the BEED/BSED specialised allocation (item 79) while carrying this pool load. Records obligation on top, compulsory for all faculty: certified true copy of Transcript of Records and signed contract to HR by 30 Oct 2026 (items 12–13).</t>
+          <t>GENERAL EDUCATION SYLLABI POOL (tracker item 74) — write the COURSE DESCRIPTION and the OBE SYLLABUS for 3 allocated courses, one set serving all 8 programmes: PATH-FIT 1 Movement Competency Training; PATH-FIT 2 Exercise-Based Fitness Activities; NSTP 1 Civic Welfare Training Service 1. 6 documents in total. Common syllabus template: 14-week trimester, 56 hours per 3-unit course, two examinations (midterm and final) plus one required monthly assessment and regular quizzes. Hand in to Chair Kent E. Garcia: descriptions 9 Oct 2026, syllabi 16 Oct 2026. Course codes are the BSA/BSAIS spellings — reconcile with your own programme's codes once Open Item 7 is closed. Not included in the BEED/BSED specialised allocation (item 79) while carrying this pool load. NSTP 1 is the prerequisite of NSTP 2 and the two are split between Calma and Mequiabas — agree the two syllabi between you so the sequence holds. Records obligation on top, compulsory for all faculty: certified true copy of Transcript of Records and signed contract to HR by 30 Oct 2026 (items 12–13).</t>
         </is>
       </c>
       <c r="J43" s="21" t="inlineStr">
@@ -8560,7 +8559,7 @@
       </c>
       <c r="I48" s="3" t="inlineStr">
         <is>
-          <t>GENERAL EDUCATION SYLLABI POOL (tracker item 74) — write the COURSE DESCRIPTION and the OBE SYLLABUS for 3 allocated courses, one set serving all 8 programmes: MAT-GEC Mathematics in the Modern World; BL-GEC Business Logic; STS-GEC Science, Technology and Society. 6 documents in total. Common syllabus template: 14-week trimester, 56 hours per 3-unit course, two examinations (midterm and final) plus one required monthly assessment and regular quizzes. Hand in to Chair Kent E. Garcia: descriptions 9 Oct 2026, syllabi 16 Oct 2026. Course codes are the BSA/BSAIS spellings — reconcile with your own programme's codes once Open Item 7 is closed. Not included in the BEED/BSED specialised allocation (item 79) while carrying this pool load. Records obligation on top, compulsory for all faculty: certified true copy of Transcript of Records and signed contract to HR by 30 Oct 2026 (items 12–13).</t>
+          <t>GENERAL EDUCATION SYLLABI POOL (tracker item 74) — write the COURSE DESCRIPTION and the OBE SYLLABUS for 3 allocated courses, one set serving all 8 programmes: REL-GEC Religion, Religious Experience and Spirituality; CLE 1 Church and Salvation History; STS-GEC Science, Technology and Society. 6 documents in total. Common syllabus template: 14-week trimester, 56 hours per 3-unit course, two examinations (midterm and final) plus one required monthly assessment and regular quizzes. Hand in to Chair Kent E. Garcia: descriptions 9 Oct 2026, syllabi 16 Oct 2026. Course codes are the BSA/BSAIS spellings — reconcile with your own programme's codes once Open Item 7 is closed. Not included in the BEED/BSED specialised allocation (item 79) while carrying this pool load. Records obligation on top, compulsory for all faculty: certified true copy of Transcript of Records and signed contract to HR by 30 Oct 2026 (items 12–13).</t>
         </is>
       </c>
       <c r="J48" s="21" t="inlineStr">
@@ -8603,7 +8602,7 @@
       </c>
       <c r="I49" s="3" t="inlineStr">
         <is>
-          <t>GENERAL EDUCATION SYLLABI POOL (tracker item 74) — write the COURSE DESCRIPTION and the OBE SYLLABUS for 2 allocated courses, one set serving all 8 programmes: PATH-FIT 3 Dance; PATH-FIT 4 Sports. 4 documents in total. Common syllabus template: 14-week trimester, 56 hours per 3-unit course, two examinations (midterm and final) plus one required monthly assessment and regular quizzes. Hand in to Chair Kent E. Garcia: descriptions 9 Oct 2026, syllabi 16 Oct 2026. Course codes are the BSA/BSAIS spellings — reconcile with your own programme's codes once Open Item 7 is closed. Not included in the BEED/BSED specialised allocation (item 79) while carrying this pool load. Records obligation on top, compulsory for all faculty: certified true copy of Transcript of Records and signed contract to HR by 30 Oct 2026 (items 12–13).</t>
+          <t>GENERAL EDUCATION SYLLABI POOL (tracker item 74) — write the COURSE DESCRIPTION and the OBE SYLLABUS for 2 allocated courses, one set serving all 8 programmes: CON-GEC The Contemporary World; ITE-GEC Living in the I.T. Era. 4 documents in total. Common syllabus template: 14-week trimester, 56 hours per 3-unit course, two examinations (midterm and final) plus one required monthly assessment and regular quizzes. Hand in to Chair Kent E. Garcia: descriptions 9 Oct 2026, syllabi 16 Oct 2026. Course codes are the BSA/BSAIS spellings — reconcile with your own programme's codes once Open Item 7 is closed. Not included in the BEED/BSED specialised allocation (item 79) while carrying this pool load. Records obligation on top, compulsory for all faculty: certified true copy of Transcript of Records and signed contract to HR by 30 Oct 2026 (items 12–13).</t>
         </is>
       </c>
       <c r="J49" s="21" t="inlineStr">
@@ -8646,7 +8645,7 @@
       </c>
       <c r="I50" s="3" t="inlineStr">
         <is>
-          <t>GENERAL EDUCATION SYLLABI POOL (tracker item 74) — write the COURSE DESCRIPTION and the OBE SYLLABUS for 3 allocated courses, one set serving all 8 programmes: HIS-GEC Readings in Philippine History; RIZ-GEC Rizal's Life and Works; CON-GEC The Contemporary World. 6 documents in total. Common syllabus template: 14-week trimester, 56 hours per 3-unit course, two examinations (midterm and final) plus one required monthly assessment and regular quizzes. Hand in to Chair Kent E. Garcia: descriptions 9 Oct 2026, syllabi 16 Oct 2026. Course codes are the BSA/BSAIS spellings — reconcile with your own programme's codes once Open Item 7 is closed. Not included in the BEED/BSED specialised allocation (item 79) while carrying this pool load. Records obligation on top, compulsory for all faculty: certified true copy of Transcript of Records and signed contract to HR by 30 Oct 2026 (items 12–13).</t>
+          <t>GENERAL EDUCATION SYLLABI POOL (tracker item 74) — write the COURSE DESCRIPTION and the OBE SYLLABUS for 3 allocated courses, one set serving all 8 programmes: CLE 2 Evangelism and Discipleship; HIS-GEC Readings in Philippine History; RIZ-GEC Rizal's Life and Works. 6 documents in total. Common syllabus template: 14-week trimester, 56 hours per 3-unit course, two examinations (midterm and final) plus one required monthly assessment and regular quizzes. Hand in to Chair Kent E. Garcia: descriptions 9 Oct 2026, syllabi 16 Oct 2026. Course codes are the BSA/BSAIS spellings — reconcile with your own programme's codes once Open Item 7 is closed. Not included in the BEED/BSED specialised allocation (item 79) while carrying this pool load. Records obligation on top, compulsory for all faculty: certified true copy of Transcript of Records and signed contract to HR by 30 Oct 2026 (items 12–13).</t>
         </is>
       </c>
       <c r="J50" s="21" t="inlineStr">
@@ -8693,7 +8692,7 @@
       </c>
       <c r="I51" s="3" t="inlineStr">
         <is>
-          <t>GENERAL EDUCATION SYLLABI POOL (tracker item 74) — write the COURSE DESCRIPTION and the OBE SYLLABUS for 3 allocated courses, one set serving all 8 programmes: REL-GEC Religion, Religious Experience and Spirituality; CLE 1 Church and Salvation History; CLE 2 Evangelism and Discipleship. 6 documents in total. Common syllabus template: 14-week trimester, 56 hours per 3-unit course, two examinations (midterm and final) plus one required monthly assessment and regular quizzes. Hand in to Chair Kent E. Garcia: descriptions 9 Oct 2026, syllabi 16 Oct 2026. Course codes are the BSA/BSAIS spellings — reconcile with your own programme's codes once Open Item 7 is closed. Not included in the BEED/BSED specialised allocation (item 79) while carrying this pool load. Records obligation on top, compulsory for all faculty: certified true copy of Transcript of Records and signed contract to HR by 30 Oct 2026 (items 12–13).</t>
+          <t>GENERAL EDUCATION SYLLABI POOL (tracker item 74) — write the COURSE DESCRIPTION and the OBE SYLLABUS for 3 allocated courses, one set serving all 8 programmes: ETH-GEC Ethics; MAT-GEC Mathematics in the Modern World; BL-GEC Business Logic. 6 documents in total. Common syllabus template: 14-week trimester, 56 hours per 3-unit course, two examinations (midterm and final) plus one required monthly assessment and regular quizzes. Hand in to Chair Kent E. Garcia: descriptions 9 Oct 2026, syllabi 16 Oct 2026. Course codes are the BSA/BSAIS spellings — reconcile with your own programme's codes once Open Item 7 is closed. Not included in the BEED/BSED specialised allocation (item 79) while carrying this pool load. Records obligation on top, compulsory for all faculty: certified true copy of Transcript of Records and signed contract to HR by 30 Oct 2026 (items 12–13).</t>
         </is>
       </c>
       <c r="J51" s="21" t="inlineStr">
@@ -8736,7 +8735,7 @@
       </c>
       <c r="I52" s="3" t="inlineStr">
         <is>
-          <t>GENERAL EDUCATION SYLLABI POOL (tracker item 74) — write the COURSE DESCRIPTION and the OBE SYLLABUS for 2 allocated courses, one set serving all 8 programmes: ETH-GEC Ethics; ITE-GEC Living in the I.T. Era. 4 documents in total. Common syllabus template: 14-week trimester, 56 hours per 3-unit course, two examinations (midterm and final) plus one required monthly assessment and regular quizzes. Hand in to Chair Kent E. Garcia: descriptions 9 Oct 2026, syllabi 16 Oct 2026. Course codes are the BSA/BSAIS spellings — reconcile with your own programme's codes once Open Item 7 is closed. Not included in the BEED/BSED specialised allocation (item 79) while carrying this pool load. Records obligation on top, compulsory for all faculty: certified true copy of Transcript of Records and signed contract to HR by 30 Oct 2026 (items 12–13).</t>
+          <t>GENERAL EDUCATION SYLLABI POOL (tracker item 74) — write the COURSE DESCRIPTION and the OBE SYLLABUS for 3 allocated courses, one set serving all 8 programmes: PATH-FIT 3 Dance; PATH-FIT 4 Sports; NSTP 2 Civic Welfare Training Service 2. 6 documents in total. Common syllabus template: 14-week trimester, 56 hours per 3-unit course, two examinations (midterm and final) plus one required monthly assessment and regular quizzes. Hand in to Chair Kent E. Garcia: descriptions 9 Oct 2026, syllabi 16 Oct 2026. Course codes are the BSA/BSAIS spellings — reconcile with your own programme's codes once Open Item 7 is closed. Not included in the BEED/BSED specialised allocation (item 79) while carrying this pool load. NSTP 1 is the prerequisite of NSTP 2 and the two are split between Calma and Mequiabas — agree the two syllabi between you so the sequence holds. Records obligation on top, compulsory for all faculty: certified true copy of Transcript of Records and signed contract to HR by 30 Oct 2026 (items 12–13).</t>
         </is>
       </c>
       <c r="J52" s="21" t="inlineStr">
@@ -8826,7 +8825,7 @@
       </c>
       <c r="I54" s="3" t="inlineStr">
         <is>
-          <t>GENERAL EDUCATION SYLLABI POOL (tracker item 74) — write the COURSE DESCRIPTION and the OBE SYLLABUS for 2 allocated courses, one set serving all 8 programmes: PATH-FIT 1 Movement Competency Training; PATH-FIT 2 Exercise-Based Fitness Activities. 4 documents in total. Common syllabus template: 14-week trimester, 56 hours per 3-unit course, two examinations (midterm and final) plus one required monthly assessment and regular quizzes. Hand in to Chair Kent E. Garcia: descriptions 9 Oct 2026, syllabi 16 Oct 2026. Course codes are the BSA/BSAIS spellings — reconcile with your own programme's codes once Open Item 7 is closed. Not included in the BEED/BSED specialised allocation (item 79) while carrying this pool load. Records obligation on top, compulsory for all faculty: certified true copy of Transcript of Records and signed contract to HR by 30 Oct 2026 (items 12–13).</t>
+          <t>GENERAL EDUCATION SYLLABI POOL (tracker item 74) — write the COURSE DESCRIPTION and the OBE SYLLABUS for 3 allocated courses, one set serving all 8 programmes: ART-GEC Art Appreciation; COM-GEC Purposive Communication; US-GEC Understanding the Self. 6 documents in total. Common syllabus template: 14-week trimester, 56 hours per 3-unit course, two examinations (midterm and final) plus one required monthly assessment and regular quizzes. Hand in to Chair Kent E. Garcia: descriptions 9 Oct 2026, syllabi 16 Oct 2026. Course codes are the BSA/BSAIS spellings — reconcile with your own programme's codes once Open Item 7 is closed. Not included in the BEED/BSED specialised allocation (item 79) while carrying this pool load. Records obligation on top, compulsory for all faculty: certified true copy of Transcript of Records and signed contract to HR by 30 Oct 2026 (items 12–13).</t>
         </is>
       </c>
       <c r="J54" s="21" t="inlineStr">
@@ -9067,7 +9066,6 @@
         </is>
       </c>
     </row>
-    <row r="60"/>
     <row r="61" ht="15" customHeight="1" s="31">
       <c r="A61" s="35" t="inlineStr">
         <is>
@@ -9181,7 +9179,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="30" customHeight="1" s="31">
       <c r="A4" s="1" t="inlineStr">
         <is>
@@ -9424,7 +9421,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13" ht="15" customHeight="1" s="31">
       <c r="A13" s="35" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
First Year schedule and faculty loading for review; adopt 'First Year - Trimester 1' naming
Items 18 and 24 move to For review. Notes on items 2, 11, 15 and 21 record
the naming convention and the faculty loading. Three rows added to My Outputs.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MfWrZ4Zkh7zsRiGVP1SDYc
</commit_message>
<xml_diff>
--- a/CHED 3-Year Trimester Application Tracker.xlsx
+++ b/CHED 3-Year Trimester Application Tracker.xlsx
@@ -24,8 +24,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="dd\-mmm\-yyyy"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -797,7 +798,7 @@
       </c>
       <c r="I7" s="7" t="inlineStr">
         <is>
-          <t>RESOLVED 3 Sep 2026: there is no prescribed CHED form. It is a compilation the college prepares against each programme's PSG. Corroborated by the CHED Region III Citizen's Charter, which requires a duly accomplished self-evaluation form per programme on submission. Each of the 8 Chairs supplies their own programme's PSG comparison; the Vice Dean consolidates.</t>
+          <t>RESOLVED 3 Sep 2026: there is no prescribed CHED form. It is a compilation the college prepares against each programme's PSG. Corroborated by the CHED Region III Citizen's Charter, which requires a duly accomplished self-evaluation form per programme on submission. Each of the 8 Chairs supplies their own programme's PSG comparison; the Vice Dean consolidates. 21 Sep 2026: BSA and BSAIS self-evaluations (Official and generated copies) now use the "First Year - Trimester 1" naming convention; the builder was updated to write it.</t>
         </is>
       </c>
     </row>
@@ -1176,7 +1177,7 @@
       </c>
       <c r="I18" s="7" t="inlineStr">
         <is>
-          <t>Phase 1 of the project plan has HR issuing the call-out for faculty certified true copy Transcripts of Record.</t>
+          <t>Phase 1 of the project plan has HR issuing the call-out for faculty certified true copy Transcripts of Record. 21 Sep 2026: BSA and BSAIS course assignments for First Year - Trimester 1 to 3 are available from the Proposed Faculty Loading (BSA &amp; BSAIS Outputs/Faculty Matrix &amp; Loading).</t>
         </is>
       </c>
     </row>
@@ -1347,7 +1348,7 @@
       </c>
       <c r="I23" s="7" t="inlineStr">
         <is>
-          <t>Draft 9-trimester prospectus prepared by the Vice Dean — 191 total units across 9 terms. Must be recast onto the agreed template (see Reference): Course Code, Course Title, Lec Hrs, Lab Hrs, Total Hrs, Credit Units, Prerequisite(s), with a sub-total per trimester and the programme's own PSG cited in the header. TERM LENGTH DECIDED, 9 Sep 2026: 14 weeks per trimester, by the Council of Programme Chairs. The contact-hour standard moves with it from 54 to 56 hours per 3-unit subject, so a 3-unit subject runs 240 minutes a week and divides into whole periods (2 x 120, 3 x 80 or 4 x 60 minutes). MEETING DATE AND RESOLUTION NUMBER STILL TO BE SUPPLIED for the dossier.</t>
+          <t>Draft 9-trimester prospectus prepared by the Vice Dean — 191 total units across 9 terms. Must be recast onto the agreed template (see Reference): Course Code, Course Title, Lec Hrs, Lab Hrs, Total Hrs, Credit Units, Prerequisite(s), with a sub-total per trimester and the programme's own PSG cited in the header. TERM LENGTH DECIDED, 9 Sep 2026: 14 weeks per trimester, by the Council of Programme Chairs. The contact-hour standard moves with it from 54 to 56 hours per 3-unit subject, so a 3-unit subject runs 240 minutes a week and divides into whole periods (2 x 120, 3 x 80 or 4 x 60 minutes). MEETING DATE AND RESOLUTION NUMBER STILL TO BE SUPPLIED for the dossier. 21 Sep 2026: term headings renamed to the college convention "First Year - Trimester 1", "First Year - Trimester 2" … "Third Year - Trimester 3"; prerequisites now read "Completed Second Year" / "Completed Third Year - Trimester 1".</t>
         </is>
       </c>
     </row>
@@ -1462,15 +1463,15 @@
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>For review</t>
         </is>
       </c>
       <c r="H26" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I26" s="7" t="inlineStr">
         <is>
-          <t>The 14-week term and the 56-hour contact-hour standard are settled, so this grid can now be built. A 3-unit subject runs 240 minutes a week, which divides into 2 x 120, 3 x 80 or 4 x 60 minute periods. The grid must leave room for two examinations (midterm and final) and one monthly assessment per term. CALENDAR CONFLICT: the proposed AY 2027-2028 academic calendar was drawn on three terms of FIFTEEN academic weeks and must be redrawn to 14 before any grid is finalised — this also moves the enrolment, grade-processing and graduation dates. DAILY LOAD at 56 hours over four teaching days: 8.00 hours on a 24-unit term, 7.67 on 23 units, and 8.33 on the two 25-unit trimesters in BSCRIM (see item 45). TERM LENGTH DECIDED, 9 Sep 2026: 14 weeks per trimester, by the Council of Programme Chairs. The contact-hour standard moves with it from 54 to 56 hours per 3-unit subject, so a 3-unit subject runs 240 minutes a week and divides into whole periods (2 x 120, 3 x 80 or 4 x 60 minutes). MEETING DATE AND RESOLUTION NUMBER STILL TO BE SUPPLIED for the dossier.</t>
+          <t>21 Sep 2026: PROPOSED SCHEDULE OF CLASSES built for First Year - Trimester 1, 2 and 3 (BSA and BSAIS share one First Year section, 1-BSA-A / 1-BSAIS-A), with the matching PROPOSED FACULTY LOADING. Each trimester carries 31 contact hours a week and 23 units, Monday to Thursday only; Friday is kept free for consultation, make-up classes and student activities. A 3-unit course meets 4 hours a week (2 x 2-hour meetings, MW or TTH), which gives the settled 56 hours over 14 weeks, examination weeks included. Signatories: prepared by the Program Chair, reviewed by the College Dean, approved by the VPAA. Files: BSA &amp; BSAIS Outputs/Sample Schedule/Proposed Schedule of Classes - First Year, Trimesters 1-3 (BSA-BSAIS) and BSA &amp; BSAIS Outputs/Faculty Matrix &amp; Loading/Proposed Faculty Loading - First Year, Trimesters 1-3 (BSA-BSAIS), Word and PDF. NOT YET BUILT: Second Year and Third Year schedules — raise with the Vice Dean if CHED expects all nine trimesters rather than one year's Trimesters 1, 2 and 3. Rooms are provisional (ML 401 for lecture, ML 211 for PATH-FIT).</t>
         </is>
       </c>
     </row>
@@ -1593,7 +1594,7 @@
       </c>
       <c r="I29" s="7" t="inlineStr">
         <is>
-          <t>Draft 9-trimester prospectus prepared by the Vice Dean — 185 total units across 9 terms. Must be recast onto the agreed template (see Reference): Course Code, Course Title, Lec Hrs, Lab Hrs, Total Hrs, Credit Units, Prerequisite(s), with a sub-total per trimester and the programme's own PSG cited in the header. TERM LENGTH DECIDED, 9 Sep 2026: 14 weeks per trimester, by the Council of Programme Chairs. The contact-hour standard moves with it from 54 to 56 hours per 3-unit subject, so a 3-unit subject runs 240 minutes a week and divides into whole periods (2 x 120, 3 x 80 or 4 x 60 minutes). MEETING DATE AND RESOLUTION NUMBER STILL TO BE SUPPLIED for the dossier.</t>
+          <t>Draft 9-trimester prospectus prepared by the Vice Dean — 185 total units across 9 terms. Must be recast onto the agreed template (see Reference): Course Code, Course Title, Lec Hrs, Lab Hrs, Total Hrs, Credit Units, Prerequisite(s), with a sub-total per trimester and the programme's own PSG cited in the header. TERM LENGTH DECIDED, 9 Sep 2026: 14 weeks per trimester, by the Council of Programme Chairs. The contact-hour standard moves with it from 54 to 56 hours per 3-unit subject, so a 3-unit subject runs 240 minutes a week and divides into whole periods (2 x 120, 3 x 80 or 4 x 60 minutes). MEETING DATE AND RESOLUTION NUMBER STILL TO BE SUPPLIED for the dossier. 21 Sep 2026: term headings renamed to the college convention "First Year - Trimester 1", "First Year - Trimester 2" … "Third Year - Trimester 3"; prerequisites now read "Completed Second Year" / "Completed Third Year - Trimester 1".</t>
         </is>
       </c>
     </row>
@@ -1708,15 +1709,15 @@
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>For review</t>
         </is>
       </c>
       <c r="H32" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I32" s="7" t="inlineStr">
         <is>
-          <t>The 14-week term and the 56-hour contact-hour standard are settled, so this grid can now be built. A 3-unit subject runs 240 minutes a week, which divides into 2 x 120, 3 x 80 or 4 x 60 minute periods. The grid must leave room for two examinations (midterm and final) and one monthly assessment per term. CALENDAR CONFLICT: the proposed AY 2027-2028 academic calendar was drawn on three terms of FIFTEEN academic weeks and must be redrawn to 14 before any grid is finalised — this also moves the enrolment, grade-processing and graduation dates. DAILY LOAD at 56 hours over four teaching days: 8.00 hours on a 24-unit term, 7.67 on 23 units, and 8.33 on the two 25-unit trimesters in BSCRIM (see item 45). TERM LENGTH DECIDED, 9 Sep 2026: 14 weeks per trimester, by the Council of Programme Chairs. The contact-hour standard moves with it from 54 to 56 hours per 3-unit subject, so a 3-unit subject runs 240 minutes a week and divides into whole periods (2 x 120, 3 x 80 or 4 x 60 minutes). MEETING DATE AND RESOLUTION NUMBER STILL TO BE SUPPLIED for the dossier.</t>
+          <t>21 Sep 2026: PROPOSED SCHEDULE OF CLASSES built for First Year - Trimester 1, 2 and 3 (BSA and BSAIS share one First Year section, 1-BSA-A / 1-BSAIS-A), with the matching PROPOSED FACULTY LOADING. Each trimester carries 31 contact hours a week and 23 units, Monday to Thursday only; Friday is kept free for consultation, make-up classes and student activities. A 3-unit course meets 4 hours a week (2 x 2-hour meetings, MW or TTH), which gives the settled 56 hours over 14 weeks, examination weeks included. Signatories: prepared by the Program Chair, reviewed by the College Dean, approved by the VPAA. Files: BSA &amp; BSAIS Outputs/Sample Schedule/Proposed Schedule of Classes - First Year, Trimesters 1-3 (BSA-BSAIS) and BSA &amp; BSAIS Outputs/Faculty Matrix &amp; Loading/Proposed Faculty Loading - First Year, Trimesters 1-3 (BSA-BSAIS), Word and PDF. NOT YET BUILT: Second Year and Third Year schedules — raise with the Vice Dean if CHED expects all nine trimesters rather than one year's Trimesters 1, 2 and 3. Rooms are provisional (ML 401 for lecture, ML 211 for PATH-FIT).</t>
         </is>
       </c>
     </row>
@@ -5268,7 +5269,6 @@
         <v/>
       </c>
     </row>
-    <row r="53"/>
     <row r="54" ht="15" customHeight="1" s="31">
       <c r="A54" s="33" t="inlineStr">
         <is>
@@ -5468,7 +5468,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14" ht="15" customHeight="1" s="31">
       <c r="A14" s="27" t="inlineStr">
         <is>
@@ -5513,7 +5512,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19" ht="15" customHeight="1" s="31">
       <c r="A19" s="27" t="inlineStr">
         <is>
@@ -5558,7 +5556,6 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
     <row r="24" ht="15" customHeight="1" s="31">
       <c r="A24" s="27" t="inlineStr">
         <is>
@@ -5651,7 +5648,6 @@
         </is>
       </c>
     </row>
-    <row r="32"/>
     <row r="33" ht="15" customHeight="1" s="31">
       <c r="A33" s="27" t="inlineStr">
         <is>
@@ -5768,7 +5764,6 @@
         </is>
       </c>
     </row>
-    <row r="43"/>
     <row r="44" ht="15" customHeight="1" s="31">
       <c r="A44" s="27" t="inlineStr">
         <is>
@@ -9155,7 +9150,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" style="31" min="1" max="1"/>
@@ -9179,6 +9174,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1" s="31">
       <c r="A4" s="1" t="inlineStr">
         <is>
@@ -9421,21 +9417,112 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="15" customHeight="1" s="31">
-      <c r="A13" s="35" t="inlineStr">
+    <row r="12" ht="35" customHeight="1" s="31">
+      <c r="A12" s="4" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Proposed Schedule of Classes, First Year - Trimester 1 to 3, combined 1-BSA / 1-BSAIS section — 31 contact hours and 23 units per trimester, Monday to Thursday, Friday kept free</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Program Chair, BSA &amp; BSAIS</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Items 18, 24</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>For review</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>BSA &amp; BSAIS Outputs/Sample Schedule — Word and PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="35" customHeight="1" s="31">
+      <c r="A13" s="4" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Proposed Faculty Loading, First Year - Trimester 1 to 3 — one full-time and 13 part-time faculty, units per instructor per trimester</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Program Chair, BSA &amp; BSAIS</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Items 18, 24; supports item 11</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>For review</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>BSA &amp; BSAIS Outputs/Faculty Matrix &amp; Loading — Word and PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="35" customHeight="1" s="31">
+      <c r="A14" s="4" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Naming convention "First Year - Trimester 1" applied to the BSA and BSAIS curricula, Sample Curriculum.xlsx, the sample schedule workbook, CHED Form 1 and 2, and both self-evaluations (builder updated)</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Program Chair, BSA &amp; BSAIS</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Items 2, 15, 21</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>BSA &amp; BSAIS Outputs (all subfolders); Self-Evaluation Builder</t>
+        </is>
+      </c>
+    </row>
+    <row r="15"/>
+    <row r="16">
+      <c r="A16" s="35" t="inlineStr">
         <is>
           <t>Outputs recorded</t>
         </is>
       </c>
-      <c r="B13" s="15">
-        <f>COUNTA($B$5:$B$11)</f>
+      <c r="B16" s="15">
+        <f>COUNTA($B$5:$B$14)</f>
         <v/>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1" s="31">
-      <c r="A14" s="26" t="inlineStr">
-        <is>
-          <t>Add new rows directly beneath row 11; the count above uses a fixed range, so extend it if you add rows below.</t>
+    <row r="17">
+      <c r="A17" s="26" t="inlineStr">
+        <is>
+          <t>Add new rows directly beneath row 14; the count above uses a fixed range, so extend it if you add rows below.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Feasibility studies for BSA and BSAIS, tuition computation workbooks, tracker notes
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MfWrZ4Zkh7zsRiGVP1SDYc
</commit_message>
<xml_diff>
--- a/CHED 3-Year Trimester Application Tracker.xlsx
+++ b/CHED 3-Year Trimester Application Tracker.xlsx
@@ -846,13 +846,17 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="H9" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" s="7" t="n"/>
+        <v>0.5</v>
+      </c>
+      <c r="I9" s="7" t="inlineStr">
+        <is>
+          <t>23 Sep 2026: the description and goals of each programme are drafted in Section I of the BSA and BSAIS feasibility studies (BSA &amp; BSAIS Outputs/Feasibility Study). The remaining six programmes still need theirs.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="35" customHeight="1" s="31">
       <c r="A10" s="2" t="n">
@@ -891,7 +895,7 @@
       </c>
       <c r="I10" s="7" t="inlineStr">
         <is>
-          <t>Phase 2 of the project plan assigns market demand data gathering to MIS with the Chairs.</t>
+          <t>Phase 2 of the project plan assigns market demand data gathering to MIS with the Chairs. 23 Sep 2026: Section III of the BSA and BSAIS feasibility studies carries the College's rationale on demand, flagged in the document itself as rationale and not survey findings. The market demand study supersedes it when available.</t>
         </is>
       </c>
     </row>
@@ -930,7 +934,11 @@
       <c r="H11" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="I11" s="7" t="n"/>
+      <c r="I11" s="7" t="inlineStr">
+        <is>
+          <t>23 Sep 2026: the feasibility studies project first-year intake at 30 (BSA) and 25 (BSAIS) growing ten per cent a year, and ask the Registrar for six years of historical freshmen enrolment to confirm or revise it.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="35" customHeight="1" s="31">
       <c r="A12" s="2" t="n">
@@ -967,7 +975,11 @@
       <c r="H12" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="I12" s="7" t="n"/>
+      <c r="I12" s="7" t="inlineStr">
+        <is>
+          <t>23 Sep 2026: the feasibility studies state that no other institution in the immediate area offers these programmes on a trimester calendar. This needs the competing-schools study behind it.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="23.75" customHeight="1" s="31">
       <c r="A13" s="2" t="n">
@@ -1006,7 +1018,7 @@
       </c>
       <c r="I13" s="7" t="inlineStr">
         <is>
-          <t>The VPAA also serves as VP for Administration and Finance, so this sits with her office.</t>
+          <t>The VPAA also serves as VP for Administration and Finance, so this sits with her office. 23 Sep 2026: the location narrative (Central Luzon, Maharlika Highway, Clark Economic Zone, the Bulacan airport terminal) is drafted in Section III of both feasibility studies.</t>
         </is>
       </c>
     </row>
@@ -1047,7 +1059,7 @@
       </c>
       <c r="I14" s="7" t="inlineStr">
         <is>
-          <t>Phase 1 of the project plan calls for the trimestral fee distribution model to be initiated.</t>
+          <t>Phase 1 of the project plan calls for the trimestral fee distribution model to be initiated. 23 Sep 2026: a computation workbook is ready for the Finance Office — “BSA/BSAIS 3-Year Trimester — Tuition Computation.xlsx”. Enter the rate per unit, the miscellaneous fee per term, the expense ratios and the tax rate, and tuition, collections, expenses and net income compute for five years. Two decisions are still Finance's: the rates themselves, and whether miscellaneous fees are charged at the same amount per term under a three-term year or annualised across three terms.</t>
         </is>
       </c>
     </row>
@@ -9150,7 +9162,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" style="31" min="1" max="1"/>
@@ -9174,7 +9186,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="30" customHeight="1" s="31">
       <c r="A4" s="1" t="inlineStr">
         <is>
@@ -9507,22 +9518,112 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
-    <row r="16">
-      <c r="A16" s="35" t="inlineStr">
+    <row r="15" ht="35" customHeight="1" s="31">
+      <c r="A15" s="4" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Feasibility study for the conversion of the BSA to a 3-year trimester delivery — description, management viability (administrator matrix), market viability (five-year enrolment projection from 30 first-year enrollees growing 10% a year), financial viability, matters to be supplied, conclusion and recommendation</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Program Chair, BSA</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Items 3, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>For review</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>BSA &amp; BSAIS Outputs/Feasibility Study — Word and PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="35" customHeight="1" s="31">
+      <c r="A16" s="4" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Feasibility study for the conversion of the BSAIS to a 3-year trimester delivery — same structure, projected from 25 first-year enrollees growing 10% a year</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Program Chair, BSAIS</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Items 3, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>For review</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>BSA &amp; BSAIS Outputs/Feasibility Study — Word and PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="35" customHeight="1" s="31">
+      <c r="A17" s="4" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Tuition computation workbook, one per programme — Finance enters the rate per unit, the miscellaneous fee per term, the expense ratios and the tax rate on the Inputs sheet; enrolment, units billed, student-terms, collections, expenses, net income and the per-student comparison against the present four-year delivery all compute</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Program Chair, BSA &amp; BSAIS</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Item 8; supports items 3–7</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>For review</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>BSA &amp; BSAIS Outputs/Feasibility Study — Excel</t>
+        </is>
+      </c>
+    </row>
+    <row r="18"/>
+    <row r="19">
+      <c r="A19" s="35" t="inlineStr">
         <is>
           <t>Outputs recorded</t>
         </is>
       </c>
-      <c r="B16" s="15">
-        <f>COUNTA($B$5:$B$14)</f>
+      <c r="B19" s="15">
+        <f>COUNTA($B$5:$B$17)</f>
         <v/>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="26" t="inlineStr">
-        <is>
-          <t>Add new rows directly beneath row 14; the count above uses a fixed range, so extend it if you add rows below.</t>
+    <row r="20">
+      <c r="A20" s="26" t="inlineStr">
+        <is>
+          <t>Add new rows directly beneath row 17; the count above uses a fixed range, so widen it when you do.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add graduate employment survey and first CPALE batch results to the feasibility studies
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MfWrZ4Zkh7zsRiGVP1SDYc
</commit_message>
<xml_diff>
--- a/CHED 3-Year Trimester Application Tracker.xlsx
+++ b/CHED 3-Year Trimester Application Tracker.xlsx
@@ -24,9 +24,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd\-mmm\-yyyy"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -895,7 +894,7 @@
       </c>
       <c r="I10" s="7" t="inlineStr">
         <is>
-          <t>Phase 2 of the project plan assigns market demand data gathering to MIS with the Chairs. 23 Sep 2026: Section III of the BSA and BSAIS feasibility studies carries the College's rationale on demand, flagged in the document itself as rationale and not survey findings. The market demand study supersedes it when available.</t>
+          <t>Phase 2 of the project plan assigns market demand data gathering to MIS with the Chairs. 23 Sep 2026: Section III of the BSA and BSAIS feasibility studies carries the College's rationale on demand, flagged in the document itself as rationale and not survey findings. The market demand study supersedes it when available. Evidence now in Section III of both studies: 95% of BSA and BSAIS graduates are gainfully employed in work related to their field, on the College's own graduate survey; the first batch of CPALE examinees returned 4 passers out of 6. The survey instrument, period, population and respondents, and the PRC report of rating, must be attached as annexes.</t>
         </is>
       </c>
     </row>
@@ -936,7 +935,7 @@
       </c>
       <c r="I11" s="7" t="inlineStr">
         <is>
-          <t>23 Sep 2026: the feasibility studies project first-year intake at 30 (BSA) and 25 (BSAIS) growing ten per cent a year, and ask the Registrar for six years of historical freshmen enrolment to confirm or revise it.</t>
+          <t>23 Sep 2026: the feasibility studies project first-year intake at 30 (BSA) and 25 (BSAIS) growing ten per cent a year, and ask the Registrar for six years of historical freshmen enrolment to confirm or revise it. The 95% employment result strengthens the prospective-student case and is cited in Section III of both studies.</t>
         </is>
       </c>
     </row>
@@ -9524,7 +9523,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Feasibility study for the conversion of the BSA to a 3-year trimester delivery — description, management viability (administrator matrix), market viability (five-year enrolment projection from 30 first-year enrollees growing 10% a year), financial viability, matters to be supplied, conclusion and recommendation</t>
+          <t>Feasibility study for the conversion of the BSA to a 3-year trimester delivery — description, management viability (administrator matrix), market viability (five-year enrolment projection from 30 first-year enrollees growing 10% a year), financial viability, matters to be supplied, conclusion and recommendation; cites the College's graduate survey (95% of BSA and BSAIS graduates gainfully employed in their field) and, for BSA, the first CPALE batch (4 passers of 6)</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -9554,7 +9553,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Feasibility study for the conversion of the BSAIS to a 3-year trimester delivery — same structure, projected from 25 first-year enrollees growing 10% a year</t>
+          <t>Feasibility study for the conversion of the BSAIS to a 3-year trimester delivery — same structure, projected from 25 first-year enrollees growing 10% a year; cites the College's graduate survey (95% of BSA and BSAIS graduates gainfully employed in their field) and, for BSA, the first CPALE batch (4 passers of 6)</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
@@ -9608,7 +9607,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19">
       <c r="A19" s="35" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Acceptability survey instrument and tabulation workbook
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MfWrZ4Zkh7zsRiGVP1SDYc
</commit_message>
<xml_diff>
--- a/CHED 3-Year Trimester Application Tracker.xlsx
+++ b/CHED 3-Year Trimester Application Tracker.xlsx
@@ -24,8 +24,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="dd\-mmm\-yyyy"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -894,7 +895,7 @@
       </c>
       <c r="I10" s="7" t="inlineStr">
         <is>
-          <t>Phase 2 of the project plan assigns market demand data gathering to MIS with the Chairs. 23 Sep 2026: Section III of the BSA and BSAIS feasibility studies carries the College's rationale on demand, flagged in the document itself as rationale and not survey findings. The market demand study supersedes it when available. Evidence now in Section III of both studies: 95% of BSA and BSAIS graduates are gainfully employed in work related to their field, on the College's own graduate survey; the first batch of CPALE examinees returned 4 passers out of 6. The survey instrument, period, population and respondents, and the PRC report of rating, must be attached as annexes.</t>
+          <t>Phase 2 of the project plan assigns market demand data gathering to MIS with the Chairs. 23 Sep 2026: Section III of the BSA and BSAIS feasibility studies carries the College's rationale on demand, flagged in the document itself as rationale and not survey findings. The market demand study supersedes it when available. Evidence now in Section III of both studies: 95% of BSA and BSAIS graduates are gainfully employed in work related to their field, on the College's own graduate survey; the first batch of CPALE examinees returned 4 passers out of 6. The survey instrument, period, population and respondents, and the PRC report of rating, must be attached as annexes. 23 Sep 2026: an acceptability survey on the proposed change is ready to run — questionnaire (form ref. HCC-VD-TRI-ACC-01, 23 Likert items in four parts plus preference and open questions) and a tabulation workbook that computes weighted means, verbal interpretations and an acceptability index as responses are encoded. In BSA &amp; BSAIS Outputs/Acceptability Survey. Still to decide: who is asked and how they are chosen — CHED will ask.</t>
         </is>
       </c>
     </row>
@@ -935,7 +936,7 @@
       </c>
       <c r="I11" s="7" t="inlineStr">
         <is>
-          <t>23 Sep 2026: the feasibility studies project first-year intake at 30 (BSA) and 25 (BSAIS) growing ten per cent a year, and ask the Registrar for six years of historical freshmen enrolment to confirm or revise it. The 95% employment result strengthens the prospective-student case and is cited in Section III of both studies.</t>
+          <t>23 Sep 2026: the feasibility studies project first-year intake at 30 (BSA) and 25 (BSAIS) growing ten per cent a year, and ask the Registrar for six years of historical freshmen enrolment to confirm or revise it. The 95% employment result strengthens the prospective-student case and is cited in Section III of both studies. 23 Sep 2026: an acceptability survey on the proposed change is ready to run — questionnaire (form ref. HCC-VD-TRI-ACC-01, 23 Likert items in four parts plus preference and open questions) and a tabulation workbook that computes weighted means, verbal interpretations and an acceptability index as responses are encoded. In BSA &amp; BSAIS Outputs/Acceptability Survey. Still to decide: who is asked and how they are chosen — CHED will ask.</t>
         </is>
       </c>
     </row>
@@ -9161,7 +9162,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" style="31" min="1" max="1"/>
@@ -9607,21 +9608,52 @@
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="35" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="4" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Acceptability survey on the proposed 3-year trimester delivery — questionnaire on HCC letterhead (respondent profile, Part A acceptability, Part B benefits, Part C concerns, Part D readiness of the College, Part E preference and intention, Part F open questions, data privacy notice under RA 10173) and a tabulation workbook with dropdown encoding, weighted means, verbal interpretation bands and an acceptability index that recompute as forms are entered</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Program Chair, BSA &amp; BSAIS</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Supports items 4, 5, 6</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>For review</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>BSA &amp; BSAIS Outputs/Acceptability Survey — Word, PDF and Excel</t>
+        </is>
+      </c>
+    </row>
+    <row r="19"/>
+    <row r="20">
+      <c r="A20" s="35" t="inlineStr">
         <is>
           <t>Outputs recorded</t>
         </is>
       </c>
-      <c r="B19" s="15">
-        <f>COUNTA($B$5:$B$17)</f>
+      <c r="B20" s="15">
+        <f>COUNTA($B$5:$B$18)</f>
         <v/>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="26" t="inlineStr">
-        <is>
-          <t>Add new rows directly beneath row 17; the count above uses a fixed range, so widen it when you do.</t>
+    <row r="21">
+      <c r="A21" s="26" t="inlineStr">
+        <is>
+          <t>Add new rows directly beneath row 18; the count above uses a fixed range, so widen it when you do.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Official letterhead across all documents; survey sampling plan
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MfWrZ4Zkh7zsRiGVP1SDYc
</commit_message>
<xml_diff>
--- a/CHED 3-Year Trimester Application Tracker.xlsx
+++ b/CHED 3-Year Trimester Application Tracker.xlsx
@@ -895,7 +895,7 @@
       </c>
       <c r="I10" s="7" t="inlineStr">
         <is>
-          <t>Phase 2 of the project plan assigns market demand data gathering to MIS with the Chairs. 23 Sep 2026: Section III of the BSA and BSAIS feasibility studies carries the College's rationale on demand, flagged in the document itself as rationale and not survey findings. The market demand study supersedes it when available. Evidence now in Section III of both studies: 95% of BSA and BSAIS graduates are gainfully employed in work related to their field, on the College's own graduate survey; the first batch of CPALE examinees returned 4 passers out of 6. The survey instrument, period, population and respondents, and the PRC report of rating, must be attached as annexes. 23 Sep 2026: an acceptability survey on the proposed change is ready to run — questionnaire (form ref. HCC-VD-TRI-ACC-01, 23 Likert items in four parts plus preference and open questions) and a tabulation workbook that computes weighted means, verbal interpretations and an acceptability index as responses are encoded. In BSA &amp; BSAIS Outputs/Acceptability Survey. Still to decide: who is asked and how they are chosen — CHED will ask.</t>
+          <t>Phase 2 of the project plan assigns market demand data gathering to MIS with the Chairs. 23 Sep 2026: Section III of the BSA and BSAIS feasibility studies carries the College's rationale on demand, flagged in the document itself as rationale and not survey findings. The market demand study supersedes it when available. Evidence now in Section III of both studies: 95% of BSA and BSAIS graduates are gainfully employed in work related to their field, on the College's own graduate survey; the first batch of CPALE examinees returned 4 passers out of 6. The survey instrument, period, population and respondents, and the PRC report of rating, must be attached as annexes. 23 Sep 2026: an acceptability survey on the proposed change is ready to run — questionnaire (form ref. HCC-VD-TRI-ACC-01, 23 Likert items in four parts plus preference and open questions) and a tabulation workbook that computes weighted means, verbal interpretations and an acceptability index as responses are encoded. In BSA &amp; BSAIS Outputs/Acceptability Survey. Still to decide: who is asked and how they are chosen — CHED will ask. 23 Sep 2026: house standard set for this application — every document is built on the College's official letterhead template (HEADER-PORTRAIT-SHORT-LONG.docx) on short bond, 8.5 x 11. The feasibility studies and the acceptability survey are already on it. The sampling plan for the survey is in the tabulation workbook: whole-population for the small groups, Slovin at a 5% margin for the large ones.</t>
         </is>
       </c>
     </row>
@@ -9162,7 +9162,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" style="31" min="1" max="1"/>
@@ -9638,22 +9638,52 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
-    <row r="20">
-      <c r="A20" s="35" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="4" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Sampling plan for the acceptability survey — eight respondent groups with who is asked and how they are chosen, populations entered by office, target respondents computed (whole population for small groups, Slovin at 5% margin for large ones, floors for alumni and employers), and forms-out against forms-back with response rate. Plus all feasibility and survey documents rebuilt on the official HCC letterhead, short bond</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Program Chair, BSA &amp; BSAIS</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Supports items 3–8</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>For review</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>BSA &amp; BSAIS Outputs/Acceptability Survey and /Feasibility Study</t>
+        </is>
+      </c>
+    </row>
+    <row r="20"/>
+    <row r="21">
+      <c r="A21" s="35" t="inlineStr">
         <is>
           <t>Outputs recorded</t>
         </is>
       </c>
-      <c r="B20" s="15">
-        <f>COUNTA($B$5:$B$18)</f>
+      <c r="B21" s="15">
+        <f>COUNTA($B$5:$B$19)</f>
         <v/>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="26" t="inlineStr">
-        <is>
-          <t>Add new rows directly beneath row 18; the count above uses a fixed range, so widen it when you do.</t>
+    <row r="22">
+      <c r="A22" s="26" t="inlineStr">
+        <is>
+          <t>Add new rows directly beneath row 19; the count above uses a fixed range, so widen it when you do.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracer study figures, faculty tasked from the proposed loading, Maglalang removed
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MfWrZ4Zkh7zsRiGVP1SDYc
</commit_message>
<xml_diff>
--- a/CHED 3-Year Trimester Application Tracker.xlsx
+++ b/CHED 3-Year Trimester Application Tracker.xlsx
@@ -24,9 +24,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd\-mmm\-yyyy"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -790,15 +789,15 @@
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="H7" s="6" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I7" s="7" t="inlineStr">
         <is>
-          <t>RESOLVED 3 Sep 2026: there is no prescribed CHED form. It is a compilation the college prepares against each programme's PSG. Corroborated by the CHED Region III Citizen's Charter, which requires a duly accomplished self-evaluation form per programme on submission. Each of the 8 Chairs supplies their own programme's PSG comparison; the Vice Dean consolidates. 21 Sep 2026: BSA and BSAIS self-evaluations (Official and generated copies) now use the "First Year - Trimester 1" naming convention; the builder was updated to write it.</t>
+          <t>RESOLVED 3 Sep 2026: there is no prescribed CHED form. It is a compilation the college prepares against each programme's PSG. Corroborated by the CHED Region III Citizen's Charter, which requires a duly accomplished self-evaluation form per programme on submission. Each of the 8 Chairs supplies their own programme's PSG comparison; the Vice Dean consolidates. 21 Sep 2026: BSA and BSAIS self-evaluations (Official and generated copies) now use the "First Year - Trimester 1" naming convention; the builder was updated to write it. 13 Oct 2026: BSA and BSAIS drafts regenerated as v1.1 (curricular finding complete; 40 programme-outcome mappings and the Year 1 teaching-load rows filled). 11 of 17 institutional requirements per programme still outstanding: faculty roster, library, facilities, internship, admission and retention, and the Sec. 20, 22 and 23 systems. 26 Oct 2026: the BSA and BSAIS Year 1 course syllabi that the self-evaluation cites are now drafted (see item 20 and 26).</t>
         </is>
       </c>
     </row>
@@ -854,7 +853,7 @@
       </c>
       <c r="I9" s="7" t="inlineStr">
         <is>
-          <t>23 Sep 2026: the description and goals of each programme are drafted in Section I of the BSA and BSAIS feasibility studies (BSA &amp; BSAIS Outputs/Feasibility Study). The remaining six programmes still need theirs.</t>
+          <t>23 Sep 2026: the description and goals of each programme are drafted in Section I of the BSA and BSAIS feasibility studies (BSA &amp; BSAIS Outputs/Feasibility Study). The remaining six programmes still need theirs. 26 Oct 2026: v2 drafts of the BSA and BSAIS feasibility studies now replace the earlier versions (acceptability survey results added; Table 9 mean to be corrected at source).</t>
         </is>
       </c>
     </row>
@@ -895,7 +894,7 @@
       </c>
       <c r="I10" s="7" t="inlineStr">
         <is>
-          <t>Phase 2 of the project plan assigns market demand data gathering to MIS with the Chairs. 23 Sep 2026: Section III of the BSA and BSAIS feasibility studies carries the College's rationale on demand, flagged in the document itself as rationale and not survey findings. The market demand study supersedes it when available. Evidence now in Section III of both studies: 95% of BSA and BSAIS graduates are gainfully employed in work related to their field, on the College's own graduate survey; the first batch of CPALE examinees returned 4 passers out of 6. The survey instrument, period, population and respondents, and the PRC report of rating, must be attached as annexes. 23 Sep 2026: an acceptability survey on the proposed change is ready to run — questionnaire (form ref. HCC-VD-TRI-ACC-01, 23 Likert items in four parts plus preference and open questions) and a tabulation workbook that computes weighted means, verbal interpretations and an acceptability index as responses are encoded. In BSA &amp; BSAIS Outputs/Acceptability Survey. Still to decide: who is asked and how they are chosen — CHED will ask. 23 Sep 2026: house standard set for this application — every document is built on the College's official letterhead template (HEADER-PORTRAIT-SHORT-LONG.docx) on short bond, 8.5 x 11. The feasibility studies and the acceptability survey are already on it. The sampling plan for the survey is in the tabulation workbook: whole-population for the small groups, Slovin at a 5% margin for the large ones.</t>
+          <t>Phase 2 of the project plan assigns market demand data gathering to MIS with the Chairs. 23 Sep 2026: Section III of the BSA and BSAIS feasibility studies carries the College's rationale on demand, flagged in the document itself as rationale and not survey findings. The market demand study supersedes it when available. Evidence now in Section III of both studies: 95% of BSA and BSAIS graduates are gainfully employed in work related to their field, on the College's own graduate survey; the first batch of CPALE examinees returned 4 passers out of 6. The survey instrument, period, population and respondents, and the PRC report of rating, must be attached as annexes. 23 Sep 2026: an acceptability survey on the proposed change is ready to run — questionnaire (form ref. HCC-VD-TRI-ACC-01, 23 Likert items in four parts plus preference and open questions) and a tabulation workbook that computes weighted means, verbal interpretations and an acceptability index as responses are encoded. In BSA &amp; BSAIS Outputs/Acceptability Survey. Still to decide: who is asked and how they are chosen — CHED will ask. 23 Sep 2026: house standard set for this application — every document is built on the College's official letterhead template (HEADER-PORTRAIT-SHORT-LONG.docx) on short bond, 8.5 x 11. The feasibility studies and the acceptability survey are already on it. The sampling plan for the survey is in the tabulation workbook: whole-population for the small groups, Slovin at a 5% margin for the large ones. 26 Oct 2026: the Graduate Tracer Study for the Batch of May 2025 is in and replaces the earlier 95% figure. Thirty graduates, twenty-eight employed in work related to their field — 93% overall, BSA 19 of 20 (95%), BSAIS 9 of 10 (90%). Ten were hired within a month of graduating and fifteen within three months; all within eight. One entry marked not employed was confirmed employed by the Vice Dean. Both feasibility studies now carry these figures and the workbook is filed with them.</t>
         </is>
       </c>
     </row>
@@ -936,7 +935,7 @@
       </c>
       <c r="I11" s="7" t="inlineStr">
         <is>
-          <t>23 Sep 2026: the feasibility studies project first-year intake at 30 (BSA) and 25 (BSAIS) growing ten per cent a year, and ask the Registrar for six years of historical freshmen enrolment to confirm or revise it. The 95% employment result strengthens the prospective-student case and is cited in Section III of both studies. 23 Sep 2026: an acceptability survey on the proposed change is ready to run — questionnaire (form ref. HCC-VD-TRI-ACC-01, 23 Likert items in four parts plus preference and open questions) and a tabulation workbook that computes weighted means, verbal interpretations and an acceptability index as responses are encoded. In BSA &amp; BSAIS Outputs/Acceptability Survey. Still to decide: who is asked and how they are chosen — CHED will ask.</t>
+          <t>23 Sep 2026: the feasibility studies project first-year intake at 30 (BSA) and 25 (BSAIS) growing ten per cent a year, and ask the Registrar for six years of historical freshmen enrolment to confirm or revise it. The 93% employment result from the May 2025 tracer study (BSA 95%) strengthens the prospective-student case and is cited in Section III of both studies. 23 Sep 2026: an acceptability survey on the proposed change is ready to run — questionnaire (form ref. HCC-VD-TRI-ACC-01, 23 Likert items in four parts plus preference and open questions) and a tabulation workbook that computes weighted means, verbal interpretations and an acceptability index as responses are encoded. In BSA &amp; BSAIS Outputs/Acceptability Survey. Still to decide: who is asked and how they are chosen — CHED will ask.</t>
         </is>
       </c>
     </row>
@@ -1508,7 +1507,7 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>Vice Dean Ken Gie Anthony G. Cruel (compliance audit); MIS Head Jayson R. Francisco (repository); General Education Syllabi Pool (20 shared GE, PATH-FIT, NSTP and CLE courses, written once for all 8 programs); Business Cluster Pool (shared business, economics and law courses); NO full-time BSA faculty besides the Chair — see Open Item 9</t>
+          <t>Vice Dean Ken Gie Anthony G. Cruel (compliance audit); MIS Head Jayson R. Francisco (repository); General Education Syllabi Pool (20 shared GE, PATH-FIT, NSTP and CLE courses, written once for all 8 programs); Business Cluster Pool (shared business, economics and law courses); Course teachers named in the Proposed Faculty Loading, First Year Trimesters 1–3 — J.R. Francisco, CPA; J.R. Empay, CPA; D.N. Santiago, CPA; R. Cruz, CPA (professional courses), each writing the description and syllabus for the courses that loading gives them; M. Germino, N. Tolosa, S.M. Calma, L. Ramos, M. Mequiabas, X. Villamayor, F. Ilag, J. Jamlang (GE, PATH-FIT, NSTP and CLE). Still no full-time faculty besides the Chair — see Open Item 9</t>
         </is>
       </c>
       <c r="F27" s="4" t="n">
@@ -1549,7 +1548,7 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>Vice Dean Ken Gie Anthony G. Cruel (compliance audit); MIS Head Jayson R. Francisco (repository); General Education Syllabi Pool (20 shared GE, PATH-FIT, NSTP and CLE courses, written once for all 8 programs); Business Cluster Pool (shared business, economics and law courses); NO full-time BSA faculty besides the Chair — see Open Item 9</t>
+          <t>Vice Dean Ken Gie Anthony G. Cruel (compliance audit); MIS Head Jayson R. Francisco (repository); General Education Syllabi Pool (20 shared GE, PATH-FIT, NSTP and CLE courses, written once for all 8 programs); Business Cluster Pool (shared business, economics and law courses); Course teachers named in the Proposed Faculty Loading, First Year Trimesters 1–3 — J.R. Francisco, CPA; J.R. Empay, CPA; D.N. Santiago, CPA; R. Cruz, CPA (professional courses), each writing the description and syllabus for the courses that loading gives them; M. Germino, N. Tolosa, S.M. Calma, L. Ramos, M. Mequiabas, X. Villamayor, F. Ilag, J. Jamlang (GE, PATH-FIT, NSTP and CLE). Still no full-time faculty besides the Chair — see Open Item 9</t>
         </is>
       </c>
       <c r="F28" s="4" t="n">
@@ -1557,15 +1556,15 @@
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>For review</t>
         </is>
       </c>
       <c r="H28" s="6" t="n">
-        <v>0.05</v>
+        <v>1</v>
       </c>
       <c r="I28" s="7" t="inlineStr">
         <is>
-          <t>ASSESSMENT SCHEME confirmed by the Vice Dean, 3 Sep 2026: two examinations per term (midterm and final), one required monthly assessment, plus regular quizzes and activities. Every syllabus must carry this scheme. CAPACITY RISK: the programme-specialised courses here have no full-time author other than the Chair.</t>
+          <t>ASSESSMENT SCHEME confirmed by the Vice Dean, 3 Sep 2026: two examinations per term (midterm and final), one required monthly assessment, plus regular quizzes and activities. Every syllabus must carry this scheme. CAPACITY RISK: the programme-specialised courses here have no full-time author other than the Chair. 26 Oct 2026: all BSA course syllabi drafted on the OBE template (14-week / 56-hour basis, midterm Week 7, final Week 14) in BSA &amp; BSAIS Outputs/Sample Syllabus/Drafts for Review; references left blank; subject-expert review pending. AE7-INT 400-hour deployment still to be confirmed.</t>
         </is>
       </c>
     </row>
@@ -1754,7 +1753,7 @@
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>Vice Dean Ken Gie Anthony G. Cruel (compliance audit); MIS Head Jayson R. Francisco (repository); General Education Syllabi Pool (20 shared GE, PATH-FIT, NSTP and CLE courses, written once for all 8 programs); Business Cluster Pool (shared business, economics and law courses); NO full-time BSAIS faculty besides the Chair — see Open Item 9</t>
+          <t>Vice Dean Ken Gie Anthony G. Cruel (compliance audit); MIS Head Jayson R. Francisco (repository); General Education Syllabi Pool (20 shared GE, PATH-FIT, NSTP and CLE courses, written once for all 8 programs); Business Cluster Pool (shared business, economics and law courses); Course teachers named in the Proposed Faculty Loading, First Year Trimesters 1–3 — J.R. Francisco, CPA; J.R. Empay, CPA; D.N. Santiago, CPA; R. Cruz, CPA (professional courses), each writing the description and syllabus for the courses that loading gives them; M. Germino, N. Tolosa, S.M. Calma, L. Ramos, M. Mequiabas, X. Villamayor, F. Ilag, J. Jamlang (GE, PATH-FIT, NSTP and CLE). Still no full-time faculty besides the Chair — see Open Item 9</t>
         </is>
       </c>
       <c r="F33" s="4" t="n">
@@ -1795,7 +1794,7 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>Vice Dean Ken Gie Anthony G. Cruel (compliance audit); MIS Head Jayson R. Francisco (repository); General Education Syllabi Pool (20 shared GE, PATH-FIT, NSTP and CLE courses, written once for all 8 programs); Business Cluster Pool (shared business, economics and law courses); NO full-time BSAIS faculty besides the Chair — see Open Item 9</t>
+          <t>Vice Dean Ken Gie Anthony G. Cruel (compliance audit); MIS Head Jayson R. Francisco (repository); General Education Syllabi Pool (20 shared GE, PATH-FIT, NSTP and CLE courses, written once for all 8 programs); Business Cluster Pool (shared business, economics and law courses); Course teachers named in the Proposed Faculty Loading, First Year Trimesters 1–3 — J.R. Francisco, CPA; J.R. Empay, CPA; D.N. Santiago, CPA; R. Cruz, CPA (professional courses), each writing the description and syllabus for the courses that loading gives them; M. Germino, N. Tolosa, S.M. Calma, L. Ramos, M. Mequiabas, X. Villamayor, F. Ilag, J. Jamlang (GE, PATH-FIT, NSTP and CLE). Still no full-time faculty besides the Chair — see Open Item 9</t>
         </is>
       </c>
       <c r="F34" s="4" t="n">
@@ -1803,15 +1802,15 @@
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>For review</t>
         </is>
       </c>
       <c r="H34" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I34" s="7" t="inlineStr">
         <is>
-          <t>ASSESSMENT SCHEME confirmed by the Vice Dean, 3 Sep 2026: two examinations per term (midterm and final), one required monthly assessment, plus regular quizzes and activities. Every syllabus must carry this scheme. CAPACITY RISK: the programme-specialised courses here have no full-time author other than the Chair.</t>
+          <t>ASSESSMENT SCHEME confirmed by the Vice Dean, 3 Sep 2026: two examinations per term (midterm and final), one required monthly assessment, plus regular quizzes and activities. Every syllabus must carry this scheme. CAPACITY RISK: the programme-specialised courses here have no full-time author other than the Chair. 26 Oct 2026: all BSAIS course syllabi drafted on the OBE template (14-week / 56-hour basis, midterm Week 7, final Week 14) in BSA &amp; BSAIS Outputs/Sample Syllabus/Drafts for Review; references left blank; subject-expert review pending. AE7-INT 400-hour deployment still to be confirmed.</t>
         </is>
       </c>
     </row>
@@ -3773,7 +3772,7 @@
       </c>
       <c r="E84" s="3" t="inlineStr">
         <is>
-          <t>General Education Syllabi Pool — 7 writers (Ilag, Maglalang, Calma, Mequiabas, Manuel, Tolosa, Jamlang); Vice Dean Ken Gie Anthony G. Cruel (GE code harmonisation); all 8 Program Chairs (recipients)</t>
+          <t>General Education Syllabi Pool — 7 writers (Ilag, Germino, Calma, Mequiabas, Manuel, Tolosa, Jamlang); Vice Dean Ken Gie Anthony G. Cruel (GE code harmonisation); all 8 Program Chairs (recipients)</t>
         </is>
       </c>
       <c r="F84" s="4" t="n">
@@ -3789,7 +3788,7 @@
       </c>
       <c r="I84" s="7" t="inlineStr">
         <is>
-          <t>POOL LEAD: Chair Kent E. Garcia (named 9 Sep 2026). ALLOCATION REVISED 13 Sep 2026 by direction of the Vice Dean — all 20 courses are assigned by name across SEVEN writers (Aquino, Agnes M. was moved out of the pool on the same date to write BEED/BSED major courses under item 79 instead). Ilag: REL-GEC, CLE 1, STS-GEC. Maglalang: CLE 2, HIS-GEC, RIZ-GEC. Calma: PATH-FIT 1, PATH-FIT 2, NSTP 1. Mequiabas: PATH-FIT 3, PATH-FIT 4, NSTP 2. Manuel: ETH-GEC, MAT-GEC, BL-GEC. Tolosa: ART-GEC, COM-GEC, US-GEC. Jamlang: CON-GEC, ITE-GEC — two only, on the heaviest teaching load in the pool at 27 units over 5 preps. Each writer produces the description AND the syllabus per course. THE LEAD'S TASKS: issue one common syllabus template carrying the assessment scheme and the 14-week / 56-hour basis; set internal hand-in dates ahead of 9 Oct and 16 Oct; hand one finished set to all 8 Chairs; report slippage weekly to the Vice Dean. WATCH: NSTP 1 is the prerequisite of NSTP 2 and they now sit with different writers — Calma and Mequiabas must agree the two syllabi between them. STILL BLOCKED BY OPEN ITEM 7 — the GE course codes do not match across programmes, so the allocation is not final until they are harmonised. He convenes and reports; each Programme Chair still answers for their own 7.3 and 7.4 rows.</t>
+          <t>POOL LEAD: Chair Kent E. Garcia (named 9 Sep 2026). ALLOCATION REVISED 13 Sep 2026 by direction of the Vice Dean — all 20 courses are assigned by name across SEVEN writers (Aquino, Agnes M. was moved out of the pool on the same date to write BEED/BSED major courses under item 79 instead). Ilag: REL-GEC, CLE 1, CLE 2, STS-GEC. Germino: HIS-GEC. Calma: PATH-FIT 1, PATH-FIT 2, NSTP 1. Mequiabas: PATH-FIT 3, PATH-FIT 4, NSTP 2. Manuel: ETH-GEC, MAT-GEC, BL-GEC. Tolosa: ART-GEC, COM-GEC, US-GEC. Jamlang: CON-GEC, ITE-GEC, RIZ-GEC — two only, on the heaviest teaching load in the pool at 27 units over 5 preps. Each writer produces the description AND the syllabus per course. THE LEAD'S TASKS: issue one common syllabus template carrying the assessment scheme and the 14-week / 56-hour basis; set internal hand-in dates ahead of 9 Oct and 16 Oct; hand one finished set to all 8 Chairs; report slippage weekly to the Vice Dean. WATCH: NSTP 1 is the prerequisite of NSTP 2 and they now sit with different writers — Calma and Mequiabas must agree the two syllabi between them. STILL BLOCKED BY OPEN ITEM 7 — the GE course codes do not match across programmes, so the allocation is not final until they are harmonised. He convenes and reports; each Programme Chair still answers for their own 7.3 and 7.4 rows. 26 Oct 2026: the Vice Dean has drafted syllabi for all 20 GE, PATH-FIT, NSTP and CLE courses (Drafts for Review) for the writers to adopt, check and finalise. Open Item 7 (code mismatch) still applies. REALLOCATED 26 Oct 2026 — D. Maglalang resigned. Her three courses went to the faculty who teach them in the Proposed Faculty Loading: CLE 2 to Ilag (who already has CLE 1), HIS-GEC to Germino (who teaches it in First Year - Trimester 1, and joins the pool for it), RIZ-GEC to Jamlang (who teaches it in First Year - Trimester 3). Still seven writers.</t>
         </is>
       </c>
     </row>
@@ -3830,7 +3829,7 @@
       </c>
       <c r="I85" s="7" t="inlineStr">
         <is>
-          <t>POOL LEAD NAMED 9 Sep 2026: Chair Ranilo S. Castillo II convenes the Business Cluster Pool. The pool writes the shared business, economics and law courses ONCE for BSA, BSAIS, BSBA and BSHM, so its output feeds items 19-20, 25-26, 31-32 and 43-44. THE LEAD'S SPECIFIC TASKS: (1) FIX THE DEFINITIVE COURSE LIST — it is still recorded only as 'about 12 to 13 courses' and no exact list exists, so this comes first; (2) publish the allocation across the 4 writers; (3) use the same common syllabus template as the GE pool; (4) set internal hand-in dates ahead of 9 Oct and 16 Oct; (5) hand ONE copy to the Chairs of BSA, BSAIS, BSBA and BSHM; (6) report slippage to the Vice Dean. BSA and BSAIS have no full-time faculty of their own, so this pool is the only source of these courses for two of the four programmes. The Chair convenes and reports; each Programme Chair still answers for their own 7.3 and 7.4 rows.</t>
+          <t>POOL LEAD NAMED 9 Sep 2026: Chair Ranilo S. Castillo II convenes the Business Cluster Pool. The pool writes the shared business, economics and law courses ONCE for BSA, BSAIS, BSBA and BSHM, so its output feeds items 19-20, 25-26, 31-32 and 43-44. THE LEAD'S SPECIFIC TASKS: (1) FIX THE DEFINITIVE COURSE LIST — it is still recorded only as 'about 12 to 13 courses' and no exact list exists, so this comes first; (2) publish the allocation across the 4 writers; (3) use the same common syllabus template as the GE pool; (4) set internal hand-in dates ahead of 9 Oct and 16 Oct; (5) hand ONE copy to the Chairs of BSA, BSAIS, BSBA and BSHM; (6) report slippage to the Vice Dean. BSA and BSAIS have no full-time faculty of their own, so this pool is the only source of these courses for two of the four programmes. The Chair convenes and reports; each Programme Chair still answers for their own 7.3 and 7.4 rows. 26 Oct 2026: the Vice Dean has drafted syllabi for the business, economics and law courses (Drafts for Review) for the writers to adopt, check and finalise.</t>
         </is>
       </c>
     </row>
@@ -4086,7 +4085,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E57"/>
+  <dimension ref="A1:E60"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" style="31" min="1" max="1"/>
@@ -4500,416 +4499,415 @@
     <row r="20" ht="57.5" customHeight="1" s="31">
       <c r="A20" s="10" t="inlineStr">
         <is>
-          <t>— no full-time faculty —</t>
+          <t>Francisco, Josephine Rose, CPA</t>
         </is>
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>All programme-specialised course descriptions and syllabi for this department fall to the Chair alone. General education courses are covered by the General Education Syllabi Pool and, where applicable, the Business Cluster Pool. See Open Item 9.</t>
+          <t>Named in the Proposed Faculty Loading, First Year Trimesters 1–3 — teaches AE13-FAR Financial Accounting and Reporting (T1), AE14-CFAS Conceptual Framework and Accounting Standards (T2). Writes the course description and outcomes-based syllabus for those courses.</t>
         </is>
       </c>
       <c r="C20" s="10" t="inlineStr">
         <is>
+          <t>None — support role only</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>4 items: #19–20, 25–26</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D20" s="10" t="inlineStr">
+    </row>
+    <row r="21" ht="15" customHeight="1" s="31">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>Empay, Jan Rhommer, CPA</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>Named in the Proposed Faculty Loading, First Year Trimesters 1–3 — teaches CBME 1 Operations Management and TQM (T1), AE1-BL1 Law on Obligations and Contracts (T3). Writes the course description and outcomes-based syllabus for those courses.</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="inlineStr">
+        <is>
+          <t>None — support role only</t>
+        </is>
+      </c>
+      <c r="D21" s="10" t="inlineStr">
+        <is>
+          <t>4 items: #19–20, 25–26</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="35" customHeight="1" s="31">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>Santiago, Decirae Nicole, CPA</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>Named in the Proposed Faculty Loading, First Year Trimesters 1–3 — teaches AE4-MGT1 Management Science (T3). Writes the course description and outcomes-based syllabus for those courses.</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="inlineStr">
+        <is>
+          <t>None — support role only</t>
+        </is>
+      </c>
+      <c r="D22" s="10" t="inlineStr">
+        <is>
+          <t>4 items: #19–20, 25–26</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="35" customHeight="1" s="31">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>Cruz, Rommel, CPA</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>Named in the Proposed Faculty Loading, First Year Trimesters 1–3 — teaches AE19-FINMGT Financial Management (T3). Writes the course description and outcomes-based syllabus for those courses.</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>None — support role only</t>
+        </is>
+      </c>
+      <c r="D23" s="10" t="inlineStr">
+        <is>
+          <t>4 items: #19–20, 25–26</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="35" customHeight="1" s="31">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>— still no full-time faculty besides the Chair —</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>The four above are part-time. The General Education, PE, NSTP and CLE courses of the First Year loading are written by the pool writers listed under Teacher Education and Criminal Justice Education. The Article VI full-time faculty requirement is still open — see Open Item 9.</t>
+        </is>
+      </c>
+      <c r="C24" s="10" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E20" s="11" t="inlineStr">
+      <c r="D24" s="10" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1" s="31">
-      <c r="A21" s="27" t="inlineStr">
+    <row r="25" ht="35" customHeight="1" s="31">
+      <c r="A25" s="27" t="inlineStr">
         <is>
           <t>BUSINESS ADMINISTRATION — Curriculum &amp; Syllabi Committee for BSBA (chaired by Chair Castillo)  (4 full-time faculty tasked; 1 part-time not tasked)</t>
         </is>
       </c>
-      <c r="B21" s="28" t="n"/>
-      <c r="C21" s="28" t="n"/>
-      <c r="D21" s="28" t="n"/>
-      <c r="E21" s="29" t="n"/>
-    </row>
-    <row r="22" ht="35" customHeight="1" s="31">
-      <c r="A22" s="3" t="inlineStr">
+      <c r="B25" s="28" t="n"/>
+      <c r="C25" s="28" t="n"/>
+      <c r="D25" s="28" t="n"/>
+      <c r="E25" s="29" t="n"/>
+    </row>
+    <row r="26" ht="15" customHeight="1" s="31">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>Aquino, Ann Jellie B.</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>Business Cluster Pool writer (item 75) — writes the course description AND the OBE syllabus for 3 courses: AE11-ECO1 Managerial Economics; AE12-ECO2 Economic Development; AE5-IBT International Business and Trade. 6 documents, one set serving BSA, BSAIS, BSBA and BSHM. Candidate list, to be confirmed by Chair Castillo against the BSBA and BSHM prospectuses. To Chair Castillo: descriptions 9 Oct, syllabi 16 Oct 2026. Also Curriculum &amp; Syllabi — BSBA, and a share of the BSBA major courses under item 80.  [FT, 24 units, 6 preps this semester]</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr">
+      <c r="C26" s="3" t="inlineStr">
         <is>
           <t>None — support role only</t>
         </is>
       </c>
-      <c r="D22" s="3" t="inlineStr">
+      <c r="D26" s="3" t="inlineStr">
         <is>
           <t>13 items: #4–6, 19–20, 25–26, 31–32, 43–44, 75, 80</t>
         </is>
       </c>
-      <c r="E22" s="4">
+      <c r="E26" s="4">
         <f>IF(MIN(IF(Tracker!$G$10="Done",99999,Tracker!$F$10),IF(Tracker!$G$11="Done",99999,Tracker!$F$11),IF(Tracker!$G$12="Done",99999,Tracker!$F$12),IF(Tracker!$G$27="Done",99999,Tracker!$F$27),IF(Tracker!$G$28="Done",99999,Tracker!$F$28),IF(Tracker!$G$33="Done",99999,Tracker!$F$33),IF(Tracker!$G$34="Done",99999,Tracker!$F$34),IF(Tracker!$G$39="Done",99999,Tracker!$F$39),IF(Tracker!$G$40="Done",99999,Tracker!$F$40),IF(Tracker!$G$51="Done",99999,Tracker!$F$51),IF(Tracker!$G$52="Done",99999,Tracker!$F$52))=99999,"—",MIN(IF(Tracker!$G$10="Done",99999,Tracker!$F$10),IF(Tracker!$G$11="Done",99999,Tracker!$F$11),IF(Tracker!$G$12="Done",99999,Tracker!$F$12),IF(Tracker!$G$27="Done",99999,Tracker!$F$27),IF(Tracker!$G$28="Done",99999,Tracker!$F$28),IF(Tracker!$G$33="Done",99999,Tracker!$F$33),IF(Tracker!$G$34="Done",99999,Tracker!$F$34),IF(Tracker!$G$39="Done",99999,Tracker!$F$39),IF(Tracker!$G$40="Done",99999,Tracker!$F$40),IF(Tracker!$G$51="Done",99999,Tracker!$F$51),IF(Tracker!$G$52="Done",99999,Tracker!$F$52)))</f>
         <v/>
       </c>
     </row>
-    <row r="23" ht="35" customHeight="1" s="31">
-      <c r="A23" s="3" t="inlineStr">
+    <row r="27" ht="23.75" customHeight="1" s="31">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>Bauat, Jhosalyn</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>Business Cluster Pool writer (item 75) — writes the course description AND the OBE syllabus for 4 courses: CBME 1 Operations Management and TQM; CBME 2 Strategic Management; AE4-MGT1 Management Science; PE1-HBO Human Behavior in Organizations. 8 documents, one set serving BSA, BSAIS, BSBA and BSHM. Candidate list, to be confirmed by Chair Castillo against the BSBA and BSHM prospectuses. To Chair Castillo: descriptions 9 Oct, syllabi 16 Oct 2026. Also Curriculum &amp; Syllabi — BSBA, and a share of the BSBA major courses under item 80.  [FT, 24 units, 6 preps this semester]</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="C27" s="3" t="inlineStr">
         <is>
           <t>None — support role only</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr">
+      <c r="D27" s="3" t="inlineStr">
         <is>
           <t>10 items: #19–20, 25–26, 31–32, 43–44, 75, 80</t>
         </is>
       </c>
-      <c r="E23" s="4">
+      <c r="E27" s="4">
         <f>IF(MIN(IF(Tracker!$G$27="Done",99999,Tracker!$F$27),IF(Tracker!$G$28="Done",99999,Tracker!$F$28),IF(Tracker!$G$33="Done",99999,Tracker!$F$33),IF(Tracker!$G$34="Done",99999,Tracker!$F$34),IF(Tracker!$G$39="Done",99999,Tracker!$F$39),IF(Tracker!$G$40="Done",99999,Tracker!$F$40),IF(Tracker!$G$51="Done",99999,Tracker!$F$51),IF(Tracker!$G$52="Done",99999,Tracker!$F$52))=99999,"—",MIN(IF(Tracker!$G$27="Done",99999,Tracker!$F$27),IF(Tracker!$G$28="Done",99999,Tracker!$F$28),IF(Tracker!$G$33="Done",99999,Tracker!$F$33),IF(Tracker!$G$34="Done",99999,Tracker!$F$34),IF(Tracker!$G$39="Done",99999,Tracker!$F$39),IF(Tracker!$G$40="Done",99999,Tracker!$F$40),IF(Tracker!$G$51="Done",99999,Tracker!$F$51),IF(Tracker!$G$52="Done",99999,Tracker!$F$52)))</f>
         <v/>
       </c>
     </row>
-    <row r="24" ht="35" customHeight="1" s="31">
-      <c r="A24" s="3" t="inlineStr">
+    <row r="28" ht="23.75" customHeight="1" s="31">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>Dela Cruz, Jacqueline</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B28" s="3" t="inlineStr">
         <is>
           <t>Business Cluster Pool writer (item 75) — writes the course description AND the OBE syllabus for 3 courses: AE19-FINMGT Financial Management; AE18-FINMKT Financial Markets; AE10-GOV Governance, Business Ethics, Risk Management and Internal Control. 6 documents, one set serving BSA, BSAIS, BSBA and BSHM. Candidate list, to be confirmed by Chair Castillo against the BSBA and BSHM prospectuses. To Chair Castillo: descriptions 9 Oct, syllabi 16 Oct 2026. Also Curriculum &amp; Syllabi — BSBA, and a share of the BSBA major courses under item 80.  [FT, 24 units, 5 preps this semester]</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr">
+      <c r="C28" s="3" t="inlineStr">
         <is>
           <t>None — support role only</t>
         </is>
       </c>
-      <c r="D24" s="3" t="inlineStr">
+      <c r="D28" s="3" t="inlineStr">
         <is>
           <t>12 items: #19–20, 25–26, 31–32, 43–44, 66–67, 75, 80</t>
         </is>
       </c>
-      <c r="E24" s="4">
+      <c r="E28" s="4">
         <f>IF(MIN(IF(Tracker!$G$27="Done",99999,Tracker!$F$27),IF(Tracker!$G$28="Done",99999,Tracker!$F$28),IF(Tracker!$G$33="Done",99999,Tracker!$F$33),IF(Tracker!$G$34="Done",99999,Tracker!$F$34),IF(Tracker!$G$39="Done",99999,Tracker!$F$39),IF(Tracker!$G$40="Done",99999,Tracker!$F$40),IF(Tracker!$G$51="Done",99999,Tracker!$F$51),IF(Tracker!$G$52="Done",99999,Tracker!$F$52),IF(Tracker!$G$75="Done",99999,Tracker!$F$75),IF(Tracker!$G$76="Done",99999,Tracker!$F$76))=99999,"—",MIN(IF(Tracker!$G$27="Done",99999,Tracker!$F$27),IF(Tracker!$G$28="Done",99999,Tracker!$F$28),IF(Tracker!$G$33="Done",99999,Tracker!$F$33),IF(Tracker!$G$34="Done",99999,Tracker!$F$34),IF(Tracker!$G$39="Done",99999,Tracker!$F$39),IF(Tracker!$G$40="Done",99999,Tracker!$F$40),IF(Tracker!$G$51="Done",99999,Tracker!$F$51),IF(Tracker!$G$52="Done",99999,Tracker!$F$52),IF(Tracker!$G$75="Done",99999,Tracker!$F$75),IF(Tracker!$G$76="Done",99999,Tracker!$F$76)))</f>
         <v/>
       </c>
     </row>
-    <row r="25" ht="35" customHeight="1" s="31">
-      <c r="A25" s="3" t="inlineStr">
+    <row r="29" ht="23.75" customHeight="1" s="31">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>Salas, Kristine Joy</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>Business Cluster Pool writer (item 75) — writes the course description AND the OBE syllabus for 3 courses: AE1-BL1 Law on Obligations and Contracts; AE2-BL2 Business Laws and Regulations; AE3-BL3 Regulatory Framework and Legal Issues in Business. 6 documents, one set serving BSA, BSAIS, BSBA and BSHM. Candidate list, to be confirmed by Chair Castillo against the BSBA and BSHM prospectuses. To Chair Castillo: descriptions 9 Oct, syllabi 16 Oct 2026. Also Curriculum &amp; Syllabi — BSBA, and a share of the BSBA major courses under item 80.  [FT, 24 units, 6 preps this semester]</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr">
         <is>
           <t>None — support role only</t>
         </is>
       </c>
-      <c r="D25" s="3" t="inlineStr">
+      <c r="D29" s="3" t="inlineStr">
         <is>
           <t>10 items: #19–20, 25–26, 31–32, 43–44, 75, 80</t>
         </is>
       </c>
-      <c r="E25" s="4">
+      <c r="E29" s="4">
         <f>IF(MIN(IF(Tracker!$G$27="Done",99999,Tracker!$F$27),IF(Tracker!$G$28="Done",99999,Tracker!$F$28),IF(Tracker!$G$33="Done",99999,Tracker!$F$33),IF(Tracker!$G$34="Done",99999,Tracker!$F$34),IF(Tracker!$G$39="Done",99999,Tracker!$F$39),IF(Tracker!$G$40="Done",99999,Tracker!$F$40),IF(Tracker!$G$51="Done",99999,Tracker!$F$51),IF(Tracker!$G$52="Done",99999,Tracker!$F$52))=99999,"—",MIN(IF(Tracker!$G$27="Done",99999,Tracker!$F$27),IF(Tracker!$G$28="Done",99999,Tracker!$F$28),IF(Tracker!$G$33="Done",99999,Tracker!$F$33),IF(Tracker!$G$34="Done",99999,Tracker!$F$34),IF(Tracker!$G$39="Done",99999,Tracker!$F$39),IF(Tracker!$G$40="Done",99999,Tracker!$F$40),IF(Tracker!$G$51="Done",99999,Tracker!$F$51),IF(Tracker!$G$52="Done",99999,Tracker!$F$52)))</f>
         <v/>
       </c>
     </row>
-    <row r="26" ht="15" customHeight="1" s="31">
-      <c r="A26" s="27" t="inlineStr">
+    <row r="30" ht="23.75" customHeight="1" s="31">
+      <c r="A30" s="27" t="inlineStr">
         <is>
           <t>CRIMINAL JUSTICE EDUCATION — Curriculum &amp; Syllabi Committee for BSCRIM (chaired by Chair Pisto)  (5 full-time faculty tasked; 1 part-time not tasked)</t>
         </is>
       </c>
-      <c r="B26" s="28" t="n"/>
-      <c r="C26" s="28" t="n"/>
-      <c r="D26" s="28" t="n"/>
-      <c r="E26" s="29" t="n"/>
-    </row>
-    <row r="27" ht="23.75" customHeight="1" s="31">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="B30" s="28" t="n"/>
+      <c r="C30" s="28" t="n"/>
+      <c r="D30" s="28" t="n"/>
+      <c r="E30" s="29" t="n"/>
+    </row>
+    <row r="31" ht="23.75" customHeight="1" s="31">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>Arimbuyutan, Jazzele M.</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>Curriculum &amp; Syllabi — BSCRIM; Feasibility &amp; Market Study  [FT, 21 units, 4 preps this semester]</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr">
+      <c r="C31" s="3" t="inlineStr">
         <is>
           <t>None — support role only</t>
         </is>
       </c>
-      <c r="D27" s="3" t="inlineStr">
+      <c r="D31" s="3" t="inlineStr">
         <is>
           <t>6 items: #4–6, 49–50, 76</t>
         </is>
       </c>
-      <c r="E27" s="4">
+      <c r="E31" s="4">
         <f>IF(MIN(IF(Tracker!$G$10="Done",99999,Tracker!$F$10),IF(Tracker!$G$11="Done",99999,Tracker!$F$11),IF(Tracker!$G$12="Done",99999,Tracker!$F$12),IF(Tracker!$G$57="Done",99999,Tracker!$F$57),IF(Tracker!$G$58="Done",99999,Tracker!$F$58))=99999,"—",MIN(IF(Tracker!$G$10="Done",99999,Tracker!$F$10),IF(Tracker!$G$11="Done",99999,Tracker!$F$11),IF(Tracker!$G$12="Done",99999,Tracker!$F$12),IF(Tracker!$G$57="Done",99999,Tracker!$F$57),IF(Tracker!$G$58="Done",99999,Tracker!$F$58)))</f>
         <v/>
       </c>
     </row>
-    <row r="28" ht="23.75" customHeight="1" s="31">
-      <c r="A28" s="3" t="inlineStr">
+    <row r="32" ht="15" customHeight="1" s="31">
+      <c r="A32" s="3" t="inlineStr">
         <is>
           <t>Dela Cruz, Jhon Allen R.</t>
         </is>
       </c>
-      <c r="B28" s="3" t="inlineStr">
+      <c r="B32" s="3" t="inlineStr">
         <is>
           <t>Curriculum &amp; Syllabi — BSCRIM  [FT, 22 units, 5 preps this semester]</t>
         </is>
       </c>
-      <c r="C28" s="3" t="inlineStr">
+      <c r="C32" s="3" t="inlineStr">
         <is>
           <t>None — support role only</t>
         </is>
       </c>
-      <c r="D28" s="3" t="inlineStr">
+      <c r="D32" s="3" t="inlineStr">
         <is>
           <t>3 items: #49–50, 76</t>
         </is>
       </c>
-      <c r="E28" s="4">
+      <c r="E32" s="4">
         <f>IF(MIN(IF(Tracker!$G$57="Done",99999,Tracker!$F$57),IF(Tracker!$G$58="Done",99999,Tracker!$F$58))=99999,"—",MIN(IF(Tracker!$G$57="Done",99999,Tracker!$F$57),IF(Tracker!$G$58="Done",99999,Tracker!$F$58)))</f>
         <v/>
       </c>
     </row>
-    <row r="29" ht="23.75" customHeight="1" s="31">
-      <c r="A29" s="3" t="inlineStr">
+    <row r="33" ht="23.75" customHeight="1" s="31">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>Diaz, Pamela B.</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B33" s="3" t="inlineStr">
         <is>
           <t>Curriculum &amp; Syllabi — BSCRIM  [FT, 22 units, 5 preps this semester]</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr">
+      <c r="C33" s="3" t="inlineStr">
         <is>
           <t>None — support role only</t>
         </is>
       </c>
-      <c r="D29" s="3" t="inlineStr">
+      <c r="D33" s="3" t="inlineStr">
         <is>
           <t>3 items: #49–50, 76</t>
         </is>
       </c>
-      <c r="E29" s="4">
+      <c r="E33" s="4">
         <f>IF(MIN(IF(Tracker!$G$57="Done",99999,Tracker!$F$57),IF(Tracker!$G$58="Done",99999,Tracker!$F$58))=99999,"—",MIN(IF(Tracker!$G$57="Done",99999,Tracker!$F$57),IF(Tracker!$G$58="Done",99999,Tracker!$F$58)))</f>
         <v/>
       </c>
     </row>
-    <row r="30" ht="23.75" customHeight="1" s="31">
-      <c r="A30" s="3" t="inlineStr">
+    <row r="34" ht="15" customHeight="1" s="31">
+      <c r="A34" s="3" t="inlineStr">
         <is>
           <t>Pamiloza, Honey Mica R.</t>
         </is>
       </c>
-      <c r="B30" s="3" t="inlineStr">
+      <c r="B34" s="3" t="inlineStr">
         <is>
           <t>Curriculum &amp; Syllabi — BSCRIM  [FT, 21 units, 4 preps this semester]</t>
         </is>
       </c>
-      <c r="C30" s="3" t="inlineStr">
+      <c r="C34" s="3" t="inlineStr">
         <is>
           <t>None — support role only</t>
         </is>
       </c>
-      <c r="D30" s="3" t="inlineStr">
+      <c r="D34" s="3" t="inlineStr">
         <is>
           <t>3 items: #49–50, 76</t>
         </is>
       </c>
-      <c r="E30" s="4">
+      <c r="E34" s="4">
         <f>IF(MIN(IF(Tracker!$G$57="Done",99999,Tracker!$F$57),IF(Tracker!$G$58="Done",99999,Tracker!$F$58))=99999,"—",MIN(IF(Tracker!$G$57="Done",99999,Tracker!$F$57),IF(Tracker!$G$58="Done",99999,Tracker!$F$58)))</f>
         <v/>
       </c>
     </row>
-    <row r="31" ht="23.75" customHeight="1" s="31">
-      <c r="A31" s="3" t="inlineStr">
+    <row r="35" ht="23.75" customHeight="1" s="31">
+      <c r="A35" s="3" t="inlineStr">
         <is>
           <t>Ramos, Leandro M.</t>
         </is>
       </c>
-      <c r="B31" s="3" t="inlineStr">
+      <c r="B35" s="3" t="inlineStr">
         <is>
           <t>Curriculum &amp; Syllabi — BSCRIM; Library Collection  [FT, 18 units, 4 preps this semester]</t>
         </is>
       </c>
-      <c r="C31" s="3" t="inlineStr">
+      <c r="C35" s="3" t="inlineStr">
         <is>
           <t>None — support role only</t>
         </is>
       </c>
-      <c r="D31" s="3" t="inlineStr">
+      <c r="D35" s="3" t="inlineStr">
         <is>
           <t>5 items: #49–50, 66–67, 76</t>
         </is>
       </c>
-      <c r="E31" s="4">
+      <c r="E35" s="4">
         <f>IF(MIN(IF(Tracker!$G$57="Done",99999,Tracker!$F$57),IF(Tracker!$G$58="Done",99999,Tracker!$F$58),IF(Tracker!$G$75="Done",99999,Tracker!$F$75),IF(Tracker!$G$76="Done",99999,Tracker!$F$76))=99999,"—",MIN(IF(Tracker!$G$57="Done",99999,Tracker!$F$57),IF(Tracker!$G$58="Done",99999,Tracker!$F$58),IF(Tracker!$G$75="Done",99999,Tracker!$F$75),IF(Tracker!$G$76="Done",99999,Tracker!$F$76)))</f>
         <v/>
       </c>
     </row>
-    <row r="32" ht="15" customHeight="1" s="31">
-      <c r="A32" s="27" t="inlineStr">
+    <row r="36" ht="23.75" customHeight="1" s="31">
+      <c r="A36" s="27" t="inlineStr">
         <is>
           <t>COMPUTER SCIENCE — Curriculum &amp; Syllabi Committee for BSCS (chaired by Chair Diamat)  (1 full-time faculty tasked; 5 part-time not tasked)</t>
         </is>
       </c>
-      <c r="B32" s="28" t="n"/>
-      <c r="C32" s="28" t="n"/>
-      <c r="D32" s="28" t="n"/>
-      <c r="E32" s="29" t="n"/>
-    </row>
-    <row r="33" ht="23.75" customHeight="1" s="31">
-      <c r="A33" s="3" t="inlineStr">
+      <c r="B36" s="28" t="n"/>
+      <c r="C36" s="28" t="n"/>
+      <c r="D36" s="28" t="n"/>
+      <c r="E36" s="29" t="n"/>
+    </row>
+    <row r="37" ht="23.75" customHeight="1" s="31">
+      <c r="A37" s="3" t="inlineStr">
         <is>
           <t>Cristobal, Teofilo G.</t>
         </is>
       </c>
-      <c r="B33" s="3" t="inlineStr">
+      <c r="B37" s="3" t="inlineStr">
         <is>
           <t>Curriculum &amp; Syllabi — BSCS  [FT, 24 units, 3 preps this semester]</t>
         </is>
       </c>
-      <c r="C33" s="3" t="inlineStr">
+      <c r="C37" s="3" t="inlineStr">
         <is>
           <t>None — support role only</t>
         </is>
       </c>
-      <c r="D33" s="3" t="inlineStr">
+      <c r="D37" s="3" t="inlineStr">
         <is>
           <t>3 items: #37–38, 78</t>
         </is>
       </c>
-      <c r="E33" s="4">
+      <c r="E37" s="4">
         <f>IF(MIN(IF(Tracker!$G$45="Done",99999,Tracker!$F$45),IF(Tracker!$G$46="Done",99999,Tracker!$F$46))=99999,"—",MIN(IF(Tracker!$G$45="Done",99999,Tracker!$F$45),IF(Tracker!$G$46="Done",99999,Tracker!$F$46)))</f>
         <v/>
       </c>
     </row>
-    <row r="34" ht="15" customHeight="1" s="31">
-      <c r="A34" s="27" t="inlineStr">
-        <is>
-          <t>HOSPITALITY MANAGEMENT — Curriculum &amp; Syllabi Committee for BSHM (chaired by Chair Ciasico)  (3 full-time faculty tasked; 5 part-time not tasked)</t>
-        </is>
-      </c>
-      <c r="B34" s="28" t="n"/>
-      <c r="C34" s="28" t="n"/>
-      <c r="D34" s="28" t="n"/>
-      <c r="E34" s="29" t="n"/>
-    </row>
-    <row r="35" ht="23.75" customHeight="1" s="31">
-      <c r="A35" s="3" t="inlineStr">
-        <is>
-          <t>Bernardo, Romeo DG</t>
-        </is>
-      </c>
-      <c r="B35" s="3" t="inlineStr">
-        <is>
-          <t>Curriculum &amp; Syllabi — BSHM; Library Collection  [FT, 21 units, 4 preps this semester]</t>
-        </is>
-      </c>
-      <c r="C35" s="3" t="inlineStr">
-        <is>
-          <t>None — support role only</t>
-        </is>
-      </c>
-      <c r="D35" s="3" t="inlineStr">
-        <is>
-          <t>7 items: #43–44, 66–69, 77</t>
-        </is>
-      </c>
-      <c r="E35" s="4">
-        <f>IF(MIN(IF(Tracker!$G$51="Done",99999,Tracker!$F$51),IF(Tracker!$G$52="Done",99999,Tracker!$F$52),IF(Tracker!$G$75="Done",99999,Tracker!$F$75),IF(Tracker!$G$76="Done",99999,Tracker!$F$76),IF(Tracker!$G$77="Done",99999,Tracker!$F$77),IF(Tracker!$G$78="Done",99999,Tracker!$F$78))=99999,"—",MIN(IF(Tracker!$G$51="Done",99999,Tracker!$F$51),IF(Tracker!$G$52="Done",99999,Tracker!$F$52),IF(Tracker!$G$75="Done",99999,Tracker!$F$75),IF(Tracker!$G$76="Done",99999,Tracker!$F$76),IF(Tracker!$G$77="Done",99999,Tracker!$F$77),IF(Tracker!$G$78="Done",99999,Tracker!$F$78)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36" ht="23.75" customHeight="1" s="31">
-      <c r="A36" s="3" t="inlineStr">
-        <is>
-          <t>Dela Cruz, Jonathan</t>
-        </is>
-      </c>
-      <c r="B36" s="3" t="inlineStr">
-        <is>
-          <t>Curriculum &amp; Syllabi — BSHM; Feasibility &amp; Market Study  [FT, 18 units, 4 preps this semester]</t>
-        </is>
-      </c>
-      <c r="C36" s="3" t="inlineStr">
-        <is>
-          <t>None — support role only</t>
-        </is>
-      </c>
-      <c r="D36" s="3" t="inlineStr">
-        <is>
-          <t>6 items: #4–6, 43–44, 77</t>
-        </is>
-      </c>
-      <c r="E36" s="4">
-        <f>IF(MIN(IF(Tracker!$G$10="Done",99999,Tracker!$F$10),IF(Tracker!$G$11="Done",99999,Tracker!$F$11),IF(Tracker!$G$12="Done",99999,Tracker!$F$12),IF(Tracker!$G$51="Done",99999,Tracker!$F$51),IF(Tracker!$G$52="Done",99999,Tracker!$F$52))=99999,"—",MIN(IF(Tracker!$G$10="Done",99999,Tracker!$F$10),IF(Tracker!$G$11="Done",99999,Tracker!$F$11),IF(Tracker!$G$12="Done",99999,Tracker!$F$12),IF(Tracker!$G$51="Done",99999,Tracker!$F$51),IF(Tracker!$G$52="Done",99999,Tracker!$F$52)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37" ht="23.75" customHeight="1" s="31">
-      <c r="A37" s="3" t="inlineStr">
-        <is>
-          <t>Geronimo, Jing Feng A., LPT</t>
-        </is>
-      </c>
-      <c r="B37" s="3" t="inlineStr">
-        <is>
-          <t>Curriculum &amp; Syllabi — BSHM  [FT, 24 units, 4 preps this semester]</t>
-        </is>
-      </c>
-      <c r="C37" s="3" t="inlineStr">
-        <is>
-          <t>None — support role only</t>
-        </is>
-      </c>
-      <c r="D37" s="3" t="inlineStr">
-        <is>
-          <t>3 items: #43–44, 77</t>
-        </is>
-      </c>
-      <c r="E37" s="4">
-        <f>IF(MIN(IF(Tracker!$G$51="Done",99999,Tracker!$F$51),IF(Tracker!$G$52="Done",99999,Tracker!$F$52))=99999,"—",MIN(IF(Tracker!$G$51="Done",99999,Tracker!$F$51),IF(Tracker!$G$52="Done",99999,Tracker!$F$52)))</f>
-        <v/>
-      </c>
-    </row>
     <row r="38" ht="15" customHeight="1" s="31">
       <c r="A38" s="27" t="inlineStr">
         <is>
-          <t>TEACHER EDUCATION — Curriculum &amp; Syllabi Committee for BEED and BSED (chaired by Chair K. Garcia)  (14 full-time faculty tasked; 4 part-time not tasked)</t>
+          <t>HOSPITALITY MANAGEMENT — Curriculum &amp; Syllabi Committee for BSHM (chaired by Chair Ciasico)  (3 full-time faculty tasked; 5 part-time not tasked)</t>
         </is>
       </c>
       <c r="B38" s="28" t="n"/>
@@ -4920,194 +4918,179 @@
     <row r="39" ht="23.75" customHeight="1" s="31">
       <c r="A39" s="3" t="inlineStr">
         <is>
+          <t>Bernardo, Romeo DG</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Curriculum &amp; Syllabi — BSHM; Library Collection  [FT, 21 units, 4 preps this semester]</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>None — support role only</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>7 items: #43–44, 66–69, 77</t>
+        </is>
+      </c>
+      <c r="E39" s="4">
+        <f>IF(MIN(IF(Tracker!$G$51="Done",99999,Tracker!$F$51),IF(Tracker!$G$52="Done",99999,Tracker!$F$52),IF(Tracker!$G$75="Done",99999,Tracker!$F$75),IF(Tracker!$G$76="Done",99999,Tracker!$F$76),IF(Tracker!$G$77="Done",99999,Tracker!$F$77),IF(Tracker!$G$78="Done",99999,Tracker!$F$78))=99999,"—",MIN(IF(Tracker!$G$51="Done",99999,Tracker!$F$51),IF(Tracker!$G$52="Done",99999,Tracker!$F$52),IF(Tracker!$G$75="Done",99999,Tracker!$F$75),IF(Tracker!$G$76="Done",99999,Tracker!$F$76),IF(Tracker!$G$77="Done",99999,Tracker!$F$77),IF(Tracker!$G$78="Done",99999,Tracker!$F$78)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40" ht="35" customHeight="1" s="31">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>Dela Cruz, Jonathan</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Curriculum &amp; Syllabi — BSHM; Feasibility &amp; Market Study  [FT, 18 units, 4 preps this semester]</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>None — support role only</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>6 items: #4–6, 43–44, 77</t>
+        </is>
+      </c>
+      <c r="E40" s="4">
+        <f>IF(MIN(IF(Tracker!$G$10="Done",99999,Tracker!$F$10),IF(Tracker!$G$11="Done",99999,Tracker!$F$11),IF(Tracker!$G$12="Done",99999,Tracker!$F$12),IF(Tracker!$G$51="Done",99999,Tracker!$F$51),IF(Tracker!$G$52="Done",99999,Tracker!$F$52))=99999,"—",MIN(IF(Tracker!$G$10="Done",99999,Tracker!$F$10),IF(Tracker!$G$11="Done",99999,Tracker!$F$11),IF(Tracker!$G$12="Done",99999,Tracker!$F$12),IF(Tracker!$G$51="Done",99999,Tracker!$F$51),IF(Tracker!$G$52="Done",99999,Tracker!$F$52)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" ht="23.75" customHeight="1" s="31">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>Geronimo, Jing Feng A., LPT</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Curriculum &amp; Syllabi — BSHM  [FT, 24 units, 4 preps this semester]</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>None — support role only</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>3 items: #43–44, 77</t>
+        </is>
+      </c>
+      <c r="E41" s="4">
+        <f>IF(MIN(IF(Tracker!$G$51="Done",99999,Tracker!$F$51),IF(Tracker!$G$52="Done",99999,Tracker!$F$52))=99999,"—",MIN(IF(Tracker!$G$51="Done",99999,Tracker!$F$51),IF(Tracker!$G$52="Done",99999,Tracker!$F$52)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42" ht="35" customHeight="1" s="31">
+      <c r="A42" s="27" t="inlineStr">
+        <is>
+          <t>TEACHER EDUCATION — Curriculum &amp; Syllabi Committee for BEED and BSED (chaired by Chair K. Garcia)  (14 full-time faculty tasked; 4 part-time not tasked)</t>
+        </is>
+      </c>
+      <c r="B42" s="28" t="n"/>
+      <c r="C42" s="28" t="n"/>
+      <c r="D42" s="28" t="n"/>
+      <c r="E42" s="29" t="n"/>
+    </row>
+    <row r="43" ht="23.75" customHeight="1" s="31">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
           <t>Ablaya, Stephanie</t>
         </is>
       </c>
-      <c r="B39" s="3" t="inlineStr">
+      <c r="B43" s="3" t="inlineStr">
         <is>
           <t>Curriculum &amp; Syllabi — BEED/BSED; Feasibility &amp; Market Study  [FT, 27 units, 6 preps this semester]</t>
         </is>
       </c>
-      <c r="C39" s="3" t="inlineStr">
+      <c r="C43" s="3" t="inlineStr">
         <is>
           <t>None — support role only</t>
         </is>
       </c>
-      <c r="D39" s="3" t="inlineStr">
+      <c r="D43" s="3" t="inlineStr">
         <is>
           <t>8 items: #4–6, 55–56, 61–62, 79</t>
         </is>
       </c>
-      <c r="E39" s="4">
+      <c r="E43" s="4">
         <f>IF(MIN(IF(Tracker!$G$10="Done",99999,Tracker!$F$10),IF(Tracker!$G$11="Done",99999,Tracker!$F$11),IF(Tracker!$G$12="Done",99999,Tracker!$F$12),IF(Tracker!$G$63="Done",99999,Tracker!$F$63),IF(Tracker!$G$64="Done",99999,Tracker!$F$64),IF(Tracker!$G$69="Done",99999,Tracker!$F$69),IF(Tracker!$G$70="Done",99999,Tracker!$F$70))=99999,"—",MIN(IF(Tracker!$G$10="Done",99999,Tracker!$F$10),IF(Tracker!$G$11="Done",99999,Tracker!$F$11),IF(Tracker!$G$12="Done",99999,Tracker!$F$12),IF(Tracker!$G$63="Done",99999,Tracker!$F$63),IF(Tracker!$G$64="Done",99999,Tracker!$F$64),IF(Tracker!$G$69="Done",99999,Tracker!$F$69),IF(Tracker!$G$70="Done",99999,Tracker!$F$70)))</f>
         <v/>
       </c>
     </row>
-    <row r="40" ht="35" customHeight="1" s="31">
-      <c r="A40" s="3" t="inlineStr">
+    <row r="44" ht="23.75" customHeight="1" s="31">
+      <c r="A44" s="3" t="inlineStr">
         <is>
           <t>Aquino, Agnes M., Dr.</t>
         </is>
       </c>
-      <c r="B40" s="3" t="inlineStr">
+      <c r="B44" s="3" t="inlineStr">
         <is>
           <t>Curriculum &amp; Syllabi — BEED/BSED. Writes the course descriptions and OBE syllabi for the BEED and BSED major courses allocated to her under item 79, due 25 Sep 2026. Moved out of the General Education Syllabi Pool on 13 Sep 2026 so the major-course load is not carried on top of the college-wide general education work.  [FT, 24 units, 7 preps this semester]</t>
         </is>
       </c>
-      <c r="C40" s="3" t="inlineStr">
+      <c r="C44" s="3" t="inlineStr">
         <is>
           <t>None — support role only</t>
         </is>
       </c>
-      <c r="D40" s="3" t="inlineStr">
+      <c r="D44" s="3" t="inlineStr">
         <is>
           <t>5 items: #55–56, 61–62, 79</t>
         </is>
       </c>
-      <c r="E40" s="4">
+      <c r="E44" s="4">
         <f>IF(MIN(IF(Tracker!$G$27="Done",99999,Tracker!$F$27),IF(Tracker!$G$28="Done",99999,Tracker!$F$28),IF(Tracker!$G$33="Done",99999,Tracker!$F$33),IF(Tracker!$G$34="Done",99999,Tracker!$F$34),IF(Tracker!$G$39="Done",99999,Tracker!$F$39),IF(Tracker!$G$40="Done",99999,Tracker!$F$40),IF(Tracker!$G$45="Done",99999,Tracker!$F$45),IF(Tracker!$G$46="Done",99999,Tracker!$F$46),IF(Tracker!$G$51="Done",99999,Tracker!$F$51),IF(Tracker!$G$52="Done",99999,Tracker!$F$52),IF(Tracker!$G$57="Done",99999,Tracker!$F$57),IF(Tracker!$G$58="Done",99999,Tracker!$F$58),IF(Tracker!$G$63="Done",99999,Tracker!$F$63),IF(Tracker!$G$64="Done",99999,Tracker!$F$64),IF(Tracker!$G$69="Done",99999,Tracker!$F$69),IF(Tracker!$G$70="Done",99999,Tracker!$F$70))=99999,"—",MIN(IF(Tracker!$G$27="Done",99999,Tracker!$F$27),IF(Tracker!$G$28="Done",99999,Tracker!$F$28),IF(Tracker!$G$33="Done",99999,Tracker!$F$33),IF(Tracker!$G$34="Done",99999,Tracker!$F$34),IF(Tracker!$G$39="Done",99999,Tracker!$F$39),IF(Tracker!$G$40="Done",99999,Tracker!$F$40),IF(Tracker!$G$45="Done",99999,Tracker!$F$45),IF(Tracker!$G$46="Done",99999,Tracker!$F$46),IF(Tracker!$G$51="Done",99999,Tracker!$F$51),IF(Tracker!$G$52="Done",99999,Tracker!$F$52),IF(Tracker!$G$57="Done",99999,Tracker!$F$57),IF(Tracker!$G$58="Done",99999,Tracker!$F$58),IF(Tracker!$G$63="Done",99999,Tracker!$F$63),IF(Tracker!$G$64="Done",99999,Tracker!$F$64),IF(Tracker!$G$69="Done",99999,Tracker!$F$69),IF(Tracker!$G$70="Done",99999,Tracker!$F$70)))</f>
         <v/>
       </c>
     </row>
-    <row r="41" ht="23.75" customHeight="1" s="31">
-      <c r="A41" s="3" t="inlineStr">
+    <row r="45" ht="35" customHeight="1" s="31">
+      <c r="A45" s="3" t="inlineStr">
         <is>
           <t>Cajucom, Ryan Neil</t>
         </is>
       </c>
-      <c r="B41" s="3" t="inlineStr">
+      <c r="B45" s="3" t="inlineStr">
         <is>
           <t>Curriculum &amp; Syllabi — BEED/BSED  [FT, 27 units, 6 preps this semester]</t>
         </is>
       </c>
-      <c r="C41" s="3" t="inlineStr">
+      <c r="C45" s="3" t="inlineStr">
         <is>
           <t>None — support role only</t>
         </is>
       </c>
-      <c r="D41" s="3" t="inlineStr">
+      <c r="D45" s="3" t="inlineStr">
         <is>
           <t>5 items: #55–56, 61–62, 79</t>
         </is>
       </c>
-      <c r="E41" s="4">
+      <c r="E45" s="4">
         <f>IF(MIN(IF(Tracker!$G$63="Done",99999,Tracker!$F$63),IF(Tracker!$G$64="Done",99999,Tracker!$F$64),IF(Tracker!$G$69="Done",99999,Tracker!$F$69),IF(Tracker!$G$70="Done",99999,Tracker!$F$70))=99999,"—",MIN(IF(Tracker!$G$63="Done",99999,Tracker!$F$63),IF(Tracker!$G$64="Done",99999,Tracker!$F$64),IF(Tracker!$G$69="Done",99999,Tracker!$F$69),IF(Tracker!$G$70="Done",99999,Tracker!$F$70)))</f>
         <v/>
       </c>
     </row>
-    <row r="42" ht="35" customHeight="1" s="31">
-      <c r="A42" s="3" t="inlineStr">
-        <is>
-          <t>Calma, Shiela Mae C.</t>
-        </is>
-      </c>
-      <c r="B42" s="3" t="inlineStr">
-        <is>
-          <t>General Education Syllabi Pool writer (item 74) — writes the course description AND the OBE syllabus for 3 courses, one set serving all 8 programmes: PATH-FIT 1 Movement Competency Training; PATH-FIT 2 Exercise-Based Fitness Activities; NSTP 1 Civic Welfare Training Service 1. 6 documents. To Chair K. Garcia: descriptions 9 Oct, syllabi 16 Oct 2026. Also Curriculum &amp; Syllabi — BEED/BSED (not allocated BEED/BSED major courses under item 79 while carrying this pool load).  [FT, 24 units, 4 preps this semester]</t>
-        </is>
-      </c>
-      <c r="C42" s="3" t="inlineStr">
-        <is>
-          <t>None — support role only</t>
-        </is>
-      </c>
-      <c r="D42" s="3" t="inlineStr">
-        <is>
-          <t>17 items: #19–20, 25–26, 31–32, 37–38, 43–44, 49–50, 55–56, 61–62, 74</t>
-        </is>
-      </c>
-      <c r="E42" s="4">
-        <f>IF(MIN(IF(Tracker!$G$27="Done",99999,Tracker!$F$27),IF(Tracker!$G$28="Done",99999,Tracker!$F$28),IF(Tracker!$G$33="Done",99999,Tracker!$F$33),IF(Tracker!$G$34="Done",99999,Tracker!$F$34),IF(Tracker!$G$39="Done",99999,Tracker!$F$39),IF(Tracker!$G$40="Done",99999,Tracker!$F$40),IF(Tracker!$G$45="Done",99999,Tracker!$F$45),IF(Tracker!$G$46="Done",99999,Tracker!$F$46),IF(Tracker!$G$51="Done",99999,Tracker!$F$51),IF(Tracker!$G$52="Done",99999,Tracker!$F$52),IF(Tracker!$G$57="Done",99999,Tracker!$F$57),IF(Tracker!$G$58="Done",99999,Tracker!$F$58),IF(Tracker!$G$63="Done",99999,Tracker!$F$63),IF(Tracker!$G$64="Done",99999,Tracker!$F$64),IF(Tracker!$G$69="Done",99999,Tracker!$F$69),IF(Tracker!$G$70="Done",99999,Tracker!$F$70))=99999,"—",MIN(IF(Tracker!$G$27="Done",99999,Tracker!$F$27),IF(Tracker!$G$28="Done",99999,Tracker!$F$28),IF(Tracker!$G$33="Done",99999,Tracker!$F$33),IF(Tracker!$G$34="Done",99999,Tracker!$F$34),IF(Tracker!$G$39="Done",99999,Tracker!$F$39),IF(Tracker!$G$40="Done",99999,Tracker!$F$40),IF(Tracker!$G$45="Done",99999,Tracker!$F$45),IF(Tracker!$G$46="Done",99999,Tracker!$F$46),IF(Tracker!$G$51="Done",99999,Tracker!$F$51),IF(Tracker!$G$52="Done",99999,Tracker!$F$52),IF(Tracker!$G$57="Done",99999,Tracker!$F$57),IF(Tracker!$G$58="Done",99999,Tracker!$F$58),IF(Tracker!$G$63="Done",99999,Tracker!$F$63),IF(Tracker!$G$64="Done",99999,Tracker!$F$64),IF(Tracker!$G$69="Done",99999,Tracker!$F$69),IF(Tracker!$G$70="Done",99999,Tracker!$F$70)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43" ht="23.75" customHeight="1" s="31">
-      <c r="A43" s="3" t="inlineStr">
-        <is>
-          <t>Delos Reyes, Diana Maris</t>
-        </is>
-      </c>
-      <c r="B43" s="3" t="inlineStr">
-        <is>
-          <t>Curriculum &amp; Syllabi — BEED/BSED  [FT, 27 units, 7 preps this semester]</t>
-        </is>
-      </c>
-      <c r="C43" s="3" t="inlineStr">
-        <is>
-          <t>None — support role only</t>
-        </is>
-      </c>
-      <c r="D43" s="3" t="inlineStr">
-        <is>
-          <t>5 items: #55–56, 61–62, 79</t>
-        </is>
-      </c>
-      <c r="E43" s="4">
-        <f>IF(MIN(IF(Tracker!$G$63="Done",99999,Tracker!$F$63),IF(Tracker!$G$64="Done",99999,Tracker!$F$64),IF(Tracker!$G$69="Done",99999,Tracker!$F$69),IF(Tracker!$G$70="Done",99999,Tracker!$F$70))=99999,"—",MIN(IF(Tracker!$G$63="Done",99999,Tracker!$F$63),IF(Tracker!$G$64="Done",99999,Tracker!$F$64),IF(Tracker!$G$69="Done",99999,Tracker!$F$69),IF(Tracker!$G$70="Done",99999,Tracker!$F$70)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44" ht="23.75" customHeight="1" s="31">
-      <c r="A44" s="3" t="inlineStr">
-        <is>
-          <t>Germino, Melanie</t>
-        </is>
-      </c>
-      <c r="B44" s="3" t="inlineStr">
-        <is>
-          <t>Curriculum &amp; Syllabi — BEED/BSED  [FT, 27 units, 7 preps this semester]</t>
-        </is>
-      </c>
-      <c r="C44" s="3" t="inlineStr">
-        <is>
-          <t>None — support role only</t>
-        </is>
-      </c>
-      <c r="D44" s="3" t="inlineStr">
-        <is>
-          <t>5 items: #55–56, 61–62, 79</t>
-        </is>
-      </c>
-      <c r="E44" s="4">
-        <f>IF(MIN(IF(Tracker!$G$63="Done",99999,Tracker!$F$63),IF(Tracker!$G$64="Done",99999,Tracker!$F$64),IF(Tracker!$G$69="Done",99999,Tracker!$F$69),IF(Tracker!$G$70="Done",99999,Tracker!$F$70))=99999,"—",MIN(IF(Tracker!$G$63="Done",99999,Tracker!$F$63),IF(Tracker!$G$64="Done",99999,Tracker!$F$64),IF(Tracker!$G$69="Done",99999,Tracker!$F$69),IF(Tracker!$G$70="Done",99999,Tracker!$F$70)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45" ht="35" customHeight="1" s="31">
-      <c r="A45" s="3" t="inlineStr">
-        <is>
-          <t>Ilag, Ferdinand T.</t>
-        </is>
-      </c>
-      <c r="B45" s="3" t="inlineStr">
-        <is>
-          <t>General Education Syllabi Pool writer (item 74) — writes the course description AND the OBE syllabus for 3 courses, one set serving all 8 programmes: REL-GEC Religion, Religious Experience and Spirituality; CLE 1 Church and Salvation History; STS-GEC Science, Technology and Society. 6 documents. To Chair K. Garcia: descriptions 9 Oct, syllabi 16 Oct 2026. Also Curriculum &amp; Syllabi — BEED/BSED (not allocated BEED/BSED major courses under item 79 while carrying this pool load).  [FT, 21 units, 3 preps this semester]</t>
-        </is>
-      </c>
-      <c r="C45" s="3" t="inlineStr">
-        <is>
-          <t>None — support role only</t>
-        </is>
-      </c>
-      <c r="D45" s="3" t="inlineStr">
-        <is>
-          <t>17 items: #19–20, 25–26, 31–32, 37–38, 43–44, 49–50, 55–56, 61–62, 74</t>
-        </is>
-      </c>
-      <c r="E45" s="4">
-        <f>IF(MIN(IF(Tracker!$G$27="Done",99999,Tracker!$F$27),IF(Tracker!$G$28="Done",99999,Tracker!$F$28),IF(Tracker!$G$33="Done",99999,Tracker!$F$33),IF(Tracker!$G$34="Done",99999,Tracker!$F$34),IF(Tracker!$G$39="Done",99999,Tracker!$F$39),IF(Tracker!$G$40="Done",99999,Tracker!$F$40),IF(Tracker!$G$45="Done",99999,Tracker!$F$45),IF(Tracker!$G$46="Done",99999,Tracker!$F$46),IF(Tracker!$G$51="Done",99999,Tracker!$F$51),IF(Tracker!$G$52="Done",99999,Tracker!$F$52),IF(Tracker!$G$57="Done",99999,Tracker!$F$57),IF(Tracker!$G$58="Done",99999,Tracker!$F$58),IF(Tracker!$G$63="Done",99999,Tracker!$F$63),IF(Tracker!$G$64="Done",99999,Tracker!$F$64),IF(Tracker!$G$69="Done",99999,Tracker!$F$69),IF(Tracker!$G$70="Done",99999,Tracker!$F$70))=99999,"—",MIN(IF(Tracker!$G$27="Done",99999,Tracker!$F$27),IF(Tracker!$G$28="Done",99999,Tracker!$F$28),IF(Tracker!$G$33="Done",99999,Tracker!$F$33),IF(Tracker!$G$34="Done",99999,Tracker!$F$34),IF(Tracker!$G$39="Done",99999,Tracker!$F$39),IF(Tracker!$G$40="Done",99999,Tracker!$F$40),IF(Tracker!$G$45="Done",99999,Tracker!$F$45),IF(Tracker!$G$46="Done",99999,Tracker!$F$46),IF(Tracker!$G$51="Done",99999,Tracker!$F$51),IF(Tracker!$G$52="Done",99999,Tracker!$F$52),IF(Tracker!$G$57="Done",99999,Tracker!$F$57),IF(Tracker!$G$58="Done",99999,Tracker!$F$58),IF(Tracker!$G$63="Done",99999,Tracker!$F$63),IF(Tracker!$G$64="Done",99999,Tracker!$F$64),IF(Tracker!$G$69="Done",99999,Tracker!$F$69),IF(Tracker!$G$70="Done",99999,Tracker!$F$70)))</f>
-        <v/>
-      </c>
-    </row>
     <row r="46" ht="35" customHeight="1" s="31">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>Jamlang, Jamie A.</t>
+          <t>Calma, Shiela Mae C.</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>General Education Syllabi Pool writer (item 74) — writes the course description AND the OBE syllabus for 2 courses, one set serving all 8 programmes: CON-GEC The Contemporary World; ITE-GEC Living in the I.T. Era. 4 documents. To Chair K. Garcia: descriptions 9 Oct, syllabi 16 Oct 2026. Also Curriculum &amp; Syllabi — BEED/BSED (not allocated BEED/BSED major courses under item 79 while carrying this pool load).  [FT, 27 units, 5 preps this semester]</t>
+          <t>General Education Syllabi Pool writer (item 74) — writes the course description AND the OBE syllabus for 3 courses, one set serving all 8 programmes: PATH-FIT 1 Movement Competency Training; PATH-FIT 2 Exercise-Based Fitness Activities; NSTP 1 Civic Welfare Training Service 1. 6 documents. To Chair K. Garcia: descriptions 9 Oct, syllabi 16 Oct 2026. Also Curriculum &amp; Syllabi — BEED/BSED (not allocated BEED/BSED major courses under item 79 while carrying this pool load).  [FT, 24 units, 4 preps this semester]</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
@@ -5128,12 +5111,12 @@
     <row r="47" ht="35" customHeight="1" s="31">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>Maglalang, Danica</t>
+          <t>Delos Reyes, Diana Maris</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>General Education Syllabi Pool writer (item 74) — writes the course description AND the OBE syllabus for 3 courses, one set serving all 8 programmes: CLE 2 Evangelism and Discipleship; HIS-GEC Readings in Philippine History; RIZ-GEC Rizal's Life and Works. 6 documents. To Chair K. Garcia: descriptions 9 Oct, syllabi 16 Oct 2026. Also Curriculum &amp; Syllabi — BEED/BSED (not allocated BEED/BSED major courses under item 79 while carrying this pool load).  [FT, 24 units, 3 preps this semester]</t>
+          <t>Curriculum &amp; Syllabi — BEED/BSED  [FT, 27 units, 7 preps this semester]</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
@@ -5143,23 +5126,23 @@
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>17 items: #19–20, 25–26, 31–32, 37–38, 43–44, 49–50, 55–56, 61–62, 74</t>
+          <t>5 items: #55–56, 61–62, 79</t>
         </is>
       </c>
       <c r="E47" s="4">
-        <f>IF(MIN(IF(Tracker!$G$27="Done",99999,Tracker!$F$27),IF(Tracker!$G$28="Done",99999,Tracker!$F$28),IF(Tracker!$G$33="Done",99999,Tracker!$F$33),IF(Tracker!$G$34="Done",99999,Tracker!$F$34),IF(Tracker!$G$39="Done",99999,Tracker!$F$39),IF(Tracker!$G$40="Done",99999,Tracker!$F$40),IF(Tracker!$G$45="Done",99999,Tracker!$F$45),IF(Tracker!$G$46="Done",99999,Tracker!$F$46),IF(Tracker!$G$51="Done",99999,Tracker!$F$51),IF(Tracker!$G$52="Done",99999,Tracker!$F$52),IF(Tracker!$G$57="Done",99999,Tracker!$F$57),IF(Tracker!$G$58="Done",99999,Tracker!$F$58),IF(Tracker!$G$63="Done",99999,Tracker!$F$63),IF(Tracker!$G$64="Done",99999,Tracker!$F$64),IF(Tracker!$G$69="Done",99999,Tracker!$F$69),IF(Tracker!$G$70="Done",99999,Tracker!$F$70))=99999,"—",MIN(IF(Tracker!$G$27="Done",99999,Tracker!$F$27),IF(Tracker!$G$28="Done",99999,Tracker!$F$28),IF(Tracker!$G$33="Done",99999,Tracker!$F$33),IF(Tracker!$G$34="Done",99999,Tracker!$F$34),IF(Tracker!$G$39="Done",99999,Tracker!$F$39),IF(Tracker!$G$40="Done",99999,Tracker!$F$40),IF(Tracker!$G$45="Done",99999,Tracker!$F$45),IF(Tracker!$G$46="Done",99999,Tracker!$F$46),IF(Tracker!$G$51="Done",99999,Tracker!$F$51),IF(Tracker!$G$52="Done",99999,Tracker!$F$52),IF(Tracker!$G$57="Done",99999,Tracker!$F$57),IF(Tracker!$G$58="Done",99999,Tracker!$F$58),IF(Tracker!$G$63="Done",99999,Tracker!$F$63),IF(Tracker!$G$64="Done",99999,Tracker!$F$64),IF(Tracker!$G$69="Done",99999,Tracker!$F$69),IF(Tracker!$G$70="Done",99999,Tracker!$F$70)))</f>
+        <f>IF(MIN(IF(Tracker!$G$63="Done",99999,Tracker!$F$63),IF(Tracker!$G$64="Done",99999,Tracker!$F$64),IF(Tracker!$G$69="Done",99999,Tracker!$F$69),IF(Tracker!$G$70="Done",99999,Tracker!$F$70))=99999,"—",MIN(IF(Tracker!$G$63="Done",99999,Tracker!$F$63),IF(Tracker!$G$64="Done",99999,Tracker!$F$64),IF(Tracker!$G$69="Done",99999,Tracker!$F$69),IF(Tracker!$G$70="Done",99999,Tracker!$F$70)))</f>
         <v/>
       </c>
     </row>
     <row r="48" ht="35" customHeight="1" s="31">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>Manuel, Consuelo V., Dr.</t>
+          <t>Germino, Melanie</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>General Education Syllabi Pool writer (item 74) — writes the course description AND the OBE syllabus for 3 courses, one set serving all 8 programmes: ETH-GEC Ethics; MAT-GEC Mathematics in the Modern World; BL-GEC Business Logic. 6 documents. To Chair K. Garcia: descriptions 9 Oct, syllabi 16 Oct 2026. Also Curriculum &amp; Syllabi — BEED/BSED (not allocated BEED/BSED major courses under item 79 while carrying this pool load).  [FT, 24 units, 4 preps this semester]</t>
+          <t>Curriculum &amp; Syllabi — BEED/BSED  [FT, 27 units, 7 preps this semester] Joins the General Education Syllabi Pool for HIS-GEC (item 74), reallocated from D. Maglalang on her resignation.</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
@@ -5169,23 +5152,23 @@
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>17 items: #19–20, 25–26, 31–32, 37–38, 43–44, 49–50, 55–56, 61–62, 74</t>
+          <t>5 items: #55–56, 61–62, 79, 74</t>
         </is>
       </c>
       <c r="E48" s="4">
-        <f>IF(MIN(IF(Tracker!$G$27="Done",99999,Tracker!$F$27),IF(Tracker!$G$28="Done",99999,Tracker!$F$28),IF(Tracker!$G$33="Done",99999,Tracker!$F$33),IF(Tracker!$G$34="Done",99999,Tracker!$F$34),IF(Tracker!$G$39="Done",99999,Tracker!$F$39),IF(Tracker!$G$40="Done",99999,Tracker!$F$40),IF(Tracker!$G$45="Done",99999,Tracker!$F$45),IF(Tracker!$G$46="Done",99999,Tracker!$F$46),IF(Tracker!$G$51="Done",99999,Tracker!$F$51),IF(Tracker!$G$52="Done",99999,Tracker!$F$52),IF(Tracker!$G$57="Done",99999,Tracker!$F$57),IF(Tracker!$G$58="Done",99999,Tracker!$F$58),IF(Tracker!$G$63="Done",99999,Tracker!$F$63),IF(Tracker!$G$64="Done",99999,Tracker!$F$64),IF(Tracker!$G$69="Done",99999,Tracker!$F$69),IF(Tracker!$G$70="Done",99999,Tracker!$F$70))=99999,"—",MIN(IF(Tracker!$G$27="Done",99999,Tracker!$F$27),IF(Tracker!$G$28="Done",99999,Tracker!$F$28),IF(Tracker!$G$33="Done",99999,Tracker!$F$33),IF(Tracker!$G$34="Done",99999,Tracker!$F$34),IF(Tracker!$G$39="Done",99999,Tracker!$F$39),IF(Tracker!$G$40="Done",99999,Tracker!$F$40),IF(Tracker!$G$45="Done",99999,Tracker!$F$45),IF(Tracker!$G$46="Done",99999,Tracker!$F$46),IF(Tracker!$G$51="Done",99999,Tracker!$F$51),IF(Tracker!$G$52="Done",99999,Tracker!$F$52),IF(Tracker!$G$57="Done",99999,Tracker!$F$57),IF(Tracker!$G$58="Done",99999,Tracker!$F$58),IF(Tracker!$G$63="Done",99999,Tracker!$F$63),IF(Tracker!$G$64="Done",99999,Tracker!$F$64),IF(Tracker!$G$69="Done",99999,Tracker!$F$69),IF(Tracker!$G$70="Done",99999,Tracker!$F$70)))</f>
+        <f>IF(MIN(IF(Tracker!$G$63="Done",99999,Tracker!$F$63),IF(Tracker!$G$64="Done",99999,Tracker!$F$64),IF(Tracker!$G$69="Done",99999,Tracker!$F$69),IF(Tracker!$G$70="Done",99999,Tracker!$F$70))=99999,"—",MIN(IF(Tracker!$G$63="Done",99999,Tracker!$F$63),IF(Tracker!$G$64="Done",99999,Tracker!$F$64),IF(Tracker!$G$69="Done",99999,Tracker!$F$69),IF(Tracker!$G$70="Done",99999,Tracker!$F$70)))</f>
         <v/>
       </c>
     </row>
     <row r="49" ht="35" customHeight="1" s="31">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>Mequiabas, Meah</t>
+          <t>Ilag, Ferdinand T.</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>General Education Syllabi Pool writer (item 74) — writes the course description AND the OBE syllabus for 3 courses, one set serving all 8 programmes: PATH-FIT 3 Dance; PATH-FIT 4 Sports; NSTP 2 Civic Welfare Training Service 2. 6 documents. To Chair K. Garcia: descriptions 9 Oct, syllabi 16 Oct 2026. Also Curriculum &amp; Syllabi — BEED/BSED (not allocated BEED/BSED major courses under item 79 while carrying this pool load).  [FT, 26 units, 4 preps this semester]</t>
+          <t>General Education Syllabi Pool writer (item 74) — writes the course description AND the OBE syllabus for 3 courses, one set serving all 8 programmes: REL-GEC Religion, Religious Experience and Spirituality; CLE 1 Church and Salvation History; STS-GEC Science, Technology and Society. 6 documents. To Chair K. Garcia: descriptions 9 Oct, syllabi 16 Oct 2026. Also Curriculum &amp; Syllabi — BEED/BSED (not allocated BEED/BSED major courses under item 79 while carrying this pool load).  [FT, 21 units, 3 preps this semester] Also CLE 2 (item 74), reallocated from D. Maglalang.</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
@@ -5206,12 +5189,12 @@
     <row r="50" ht="23.75" customHeight="1" s="31">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>Sta. Cruz, Ma. Patricia</t>
+          <t>Jamlang, Jamie A.</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>Curriculum &amp; Syllabi — BEED/BSED; Library Collection  [FT, 27 units, 3 preps this semester]</t>
+          <t>General Education Syllabi Pool writer (item 74) — writes the course description AND the OBE syllabus for 2 courses, one set serving all 8 programmes: CON-GEC The Contemporary World; ITE-GEC Living in the I.T. Era. 4 documents. To Chair K. Garcia: descriptions 9 Oct, syllabi 16 Oct 2026. Also Curriculum &amp; Syllabi — BEED/BSED (not allocated BEED/BSED major courses under item 79 while carrying this pool load).  [FT, 27 units, 5 preps this semester] Also RIZ-GEC (item 74), reallocated from D. Maglalang.</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
@@ -5221,23 +5204,23 @@
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>9 items: #55–56, 61–62, 66–69, 79</t>
+          <t>17 items: #19–20, 25–26, 31–32, 37–38, 43–44, 49–50, 55–56, 61–62, 74</t>
         </is>
       </c>
       <c r="E50" s="4">
-        <f>IF(MIN(IF(Tracker!$G$63="Done",99999,Tracker!$F$63),IF(Tracker!$G$64="Done",99999,Tracker!$F$64),IF(Tracker!$G$69="Done",99999,Tracker!$F$69),IF(Tracker!$G$70="Done",99999,Tracker!$F$70),IF(Tracker!$G$75="Done",99999,Tracker!$F$75),IF(Tracker!$G$76="Done",99999,Tracker!$F$76),IF(Tracker!$G$77="Done",99999,Tracker!$F$77),IF(Tracker!$G$78="Done",99999,Tracker!$F$78))=99999,"—",MIN(IF(Tracker!$G$63="Done",99999,Tracker!$F$63),IF(Tracker!$G$64="Done",99999,Tracker!$F$64),IF(Tracker!$G$69="Done",99999,Tracker!$F$69),IF(Tracker!$G$70="Done",99999,Tracker!$F$70),IF(Tracker!$G$75="Done",99999,Tracker!$F$75),IF(Tracker!$G$76="Done",99999,Tracker!$F$76),IF(Tracker!$G$77="Done",99999,Tracker!$F$77),IF(Tracker!$G$78="Done",99999,Tracker!$F$78)))</f>
+        <f>IF(MIN(IF(Tracker!$G$27="Done",99999,Tracker!$F$27),IF(Tracker!$G$28="Done",99999,Tracker!$F$28),IF(Tracker!$G$33="Done",99999,Tracker!$F$33),IF(Tracker!$G$34="Done",99999,Tracker!$F$34),IF(Tracker!$G$39="Done",99999,Tracker!$F$39),IF(Tracker!$G$40="Done",99999,Tracker!$F$40),IF(Tracker!$G$45="Done",99999,Tracker!$F$45),IF(Tracker!$G$46="Done",99999,Tracker!$F$46),IF(Tracker!$G$51="Done",99999,Tracker!$F$51),IF(Tracker!$G$52="Done",99999,Tracker!$F$52),IF(Tracker!$G$57="Done",99999,Tracker!$F$57),IF(Tracker!$G$58="Done",99999,Tracker!$F$58),IF(Tracker!$G$63="Done",99999,Tracker!$F$63),IF(Tracker!$G$64="Done",99999,Tracker!$F$64),IF(Tracker!$G$69="Done",99999,Tracker!$F$69),IF(Tracker!$G$70="Done",99999,Tracker!$F$70))=99999,"—",MIN(IF(Tracker!$G$27="Done",99999,Tracker!$F$27),IF(Tracker!$G$28="Done",99999,Tracker!$F$28),IF(Tracker!$G$33="Done",99999,Tracker!$F$33),IF(Tracker!$G$34="Done",99999,Tracker!$F$34),IF(Tracker!$G$39="Done",99999,Tracker!$F$39),IF(Tracker!$G$40="Done",99999,Tracker!$F$40),IF(Tracker!$G$45="Done",99999,Tracker!$F$45),IF(Tracker!$G$46="Done",99999,Tracker!$F$46),IF(Tracker!$G$51="Done",99999,Tracker!$F$51),IF(Tracker!$G$52="Done",99999,Tracker!$F$52),IF(Tracker!$G$57="Done",99999,Tracker!$F$57),IF(Tracker!$G$58="Done",99999,Tracker!$F$58),IF(Tracker!$G$63="Done",99999,Tracker!$F$63),IF(Tracker!$G$64="Done",99999,Tracker!$F$64),IF(Tracker!$G$69="Done",99999,Tracker!$F$69),IF(Tracker!$G$70="Done",99999,Tracker!$F$70)))</f>
         <v/>
       </c>
     </row>
     <row r="51" ht="35" customHeight="1" s="31">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>Tolosa, Nenita</t>
+          <t>Manuel, Consuelo V., Dr.</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>General Education Syllabi Pool writer (item 74) — writes the course description AND the OBE syllabus for 3 courses, one set serving all 8 programmes: ART-GEC Art Appreciation; COM-GEC Purposive Communication; US-GEC Understanding the Self. 6 documents. To Chair K. Garcia: descriptions 9 Oct, syllabi 16 Oct 2026. Also Curriculum &amp; Syllabi — BEED/BSED (not allocated BEED/BSED major courses under item 79 while carrying this pool load).  [FT, 24 units, 5 preps this semester]</t>
+          <t>General Education Syllabi Pool writer (item 74) — writes the course description AND the OBE syllabus for 3 courses, one set serving all 8 programmes: ETH-GEC Ethics; MAT-GEC Mathematics in the Modern World; BL-GEC Business Logic. 6 documents. To Chair K. Garcia: descriptions 9 Oct, syllabi 16 Oct 2026. Also Curriculum &amp; Syllabi — BEED/BSED (not allocated BEED/BSED major courses under item 79 while carrying this pool load).  [FT, 24 units, 4 preps this semester]</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
@@ -5258,74 +5241,152 @@
     <row r="52" ht="23.75" customHeight="1" s="31">
       <c r="A52" s="3" t="inlineStr">
         <is>
+          <t>Mequiabas, Meah</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>General Education Syllabi Pool writer (item 74) — writes the course description AND the OBE syllabus for 3 courses, one set serving all 8 programmes: PATH-FIT 3 Dance; PATH-FIT 4 Sports; NSTP 2 Civic Welfare Training Service 2. 6 documents. To Chair K. Garcia: descriptions 9 Oct, syllabi 16 Oct 2026. Also Curriculum &amp; Syllabi — BEED/BSED (not allocated BEED/BSED major courses under item 79 while carrying this pool load).  [FT, 26 units, 4 preps this semester]</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>None — support role only</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>17 items: #19–20, 25–26, 31–32, 37–38, 43–44, 49–50, 55–56, 61–62, 74</t>
+        </is>
+      </c>
+      <c r="E52" s="4">
+        <f>IF(MIN(IF(Tracker!$G$27="Done",99999,Tracker!$F$27),IF(Tracker!$G$28="Done",99999,Tracker!$F$28),IF(Tracker!$G$33="Done",99999,Tracker!$F$33),IF(Tracker!$G$34="Done",99999,Tracker!$F$34),IF(Tracker!$G$39="Done",99999,Tracker!$F$39),IF(Tracker!$G$40="Done",99999,Tracker!$F$40),IF(Tracker!$G$45="Done",99999,Tracker!$F$45),IF(Tracker!$G$46="Done",99999,Tracker!$F$46),IF(Tracker!$G$51="Done",99999,Tracker!$F$51),IF(Tracker!$G$52="Done",99999,Tracker!$F$52),IF(Tracker!$G$57="Done",99999,Tracker!$F$57),IF(Tracker!$G$58="Done",99999,Tracker!$F$58),IF(Tracker!$G$63="Done",99999,Tracker!$F$63),IF(Tracker!$G$64="Done",99999,Tracker!$F$64),IF(Tracker!$G$69="Done",99999,Tracker!$F$69),IF(Tracker!$G$70="Done",99999,Tracker!$F$70))=99999,"—",MIN(IF(Tracker!$G$27="Done",99999,Tracker!$F$27),IF(Tracker!$G$28="Done",99999,Tracker!$F$28),IF(Tracker!$G$33="Done",99999,Tracker!$F$33),IF(Tracker!$G$34="Done",99999,Tracker!$F$34),IF(Tracker!$G$39="Done",99999,Tracker!$F$39),IF(Tracker!$G$40="Done",99999,Tracker!$F$40),IF(Tracker!$G$45="Done",99999,Tracker!$F$45),IF(Tracker!$G$46="Done",99999,Tracker!$F$46),IF(Tracker!$G$51="Done",99999,Tracker!$F$51),IF(Tracker!$G$52="Done",99999,Tracker!$F$52),IF(Tracker!$G$57="Done",99999,Tracker!$F$57),IF(Tracker!$G$58="Done",99999,Tracker!$F$58),IF(Tracker!$G$63="Done",99999,Tracker!$F$63),IF(Tracker!$G$64="Done",99999,Tracker!$F$64),IF(Tracker!$G$69="Done",99999,Tracker!$F$69),IF(Tracker!$G$70="Done",99999,Tracker!$F$70)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>Sta. Cruz, Ma. Patricia</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>Curriculum &amp; Syllabi — BEED/BSED; Library Collection  [FT, 27 units, 3 preps this semester]</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>None — support role only</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>9 items: #55–56, 61–62, 66–69, 79</t>
+        </is>
+      </c>
+      <c r="E53" s="4">
+        <f>IF(MIN(IF(Tracker!$G$63="Done",99999,Tracker!$F$63),IF(Tracker!$G$64="Done",99999,Tracker!$F$64),IF(Tracker!$G$69="Done",99999,Tracker!$F$69),IF(Tracker!$G$70="Done",99999,Tracker!$F$70),IF(Tracker!$G$75="Done",99999,Tracker!$F$75),IF(Tracker!$G$76="Done",99999,Tracker!$F$76),IF(Tracker!$G$77="Done",99999,Tracker!$F$77),IF(Tracker!$G$78="Done",99999,Tracker!$F$78))=99999,"—",MIN(IF(Tracker!$G$63="Done",99999,Tracker!$F$63),IF(Tracker!$G$64="Done",99999,Tracker!$F$64),IF(Tracker!$G$69="Done",99999,Tracker!$F$69),IF(Tracker!$G$70="Done",99999,Tracker!$F$70),IF(Tracker!$G$75="Done",99999,Tracker!$F$75),IF(Tracker!$G$76="Done",99999,Tracker!$F$76),IF(Tracker!$G$77="Done",99999,Tracker!$F$77),IF(Tracker!$G$78="Done",99999,Tracker!$F$78)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54" ht="15" customHeight="1" s="31">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>Tolosa, Nenita</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>General Education Syllabi Pool writer (item 74) — writes the course description AND the OBE syllabus for 3 courses, one set serving all 8 programmes: ART-GEC Art Appreciation; COM-GEC Purposive Communication; US-GEC Understanding the Self. 6 documents. To Chair K. Garcia: descriptions 9 Oct, syllabi 16 Oct 2026. Also Curriculum &amp; Syllabi — BEED/BSED (not allocated BEED/BSED major courses under item 79 while carrying this pool load).  [FT, 24 units, 5 preps this semester]</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>None — support role only</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>17 items: #19–20, 25–26, 31–32, 37–38, 43–44, 49–50, 55–56, 61–62, 74</t>
+        </is>
+      </c>
+      <c r="E54" s="4">
+        <f>IF(MIN(IF(Tracker!$G$27="Done",99999,Tracker!$F$27),IF(Tracker!$G$28="Done",99999,Tracker!$F$28),IF(Tracker!$G$33="Done",99999,Tracker!$F$33),IF(Tracker!$G$34="Done",99999,Tracker!$F$34),IF(Tracker!$G$39="Done",99999,Tracker!$F$39),IF(Tracker!$G$40="Done",99999,Tracker!$F$40),IF(Tracker!$G$45="Done",99999,Tracker!$F$45),IF(Tracker!$G$46="Done",99999,Tracker!$F$46),IF(Tracker!$G$51="Done",99999,Tracker!$F$51),IF(Tracker!$G$52="Done",99999,Tracker!$F$52),IF(Tracker!$G$57="Done",99999,Tracker!$F$57),IF(Tracker!$G$58="Done",99999,Tracker!$F$58),IF(Tracker!$G$63="Done",99999,Tracker!$F$63),IF(Tracker!$G$64="Done",99999,Tracker!$F$64),IF(Tracker!$G$69="Done",99999,Tracker!$F$69),IF(Tracker!$G$70="Done",99999,Tracker!$F$70))=99999,"—",MIN(IF(Tracker!$G$27="Done",99999,Tracker!$F$27),IF(Tracker!$G$28="Done",99999,Tracker!$F$28),IF(Tracker!$G$33="Done",99999,Tracker!$F$33),IF(Tracker!$G$34="Done",99999,Tracker!$F$34),IF(Tracker!$G$39="Done",99999,Tracker!$F$39),IF(Tracker!$G$40="Done",99999,Tracker!$F$40),IF(Tracker!$G$45="Done",99999,Tracker!$F$45),IF(Tracker!$G$46="Done",99999,Tracker!$F$46),IF(Tracker!$G$51="Done",99999,Tracker!$F$51),IF(Tracker!$G$52="Done",99999,Tracker!$F$52),IF(Tracker!$G$57="Done",99999,Tracker!$F$57),IF(Tracker!$G$58="Done",99999,Tracker!$F$58),IF(Tracker!$G$63="Done",99999,Tracker!$F$63),IF(Tracker!$G$64="Done",99999,Tracker!$F$64),IF(Tracker!$G$69="Done",99999,Tracker!$F$69),IF(Tracker!$G$70="Done",99999,Tracker!$F$70)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55" ht="135.75" customHeight="1" s="31">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
           <t>Villamayor, Xyrelle</t>
         </is>
       </c>
-      <c r="B52" s="3" t="inlineStr">
+      <c r="B55" s="3" t="inlineStr">
         <is>
           <t>Curriculum &amp; Syllabi — BEED/BSED  [FT, 27 units, 6 preps this semester]</t>
         </is>
       </c>
-      <c r="C52" s="3" t="inlineStr">
+      <c r="C55" s="3" t="inlineStr">
         <is>
           <t>None — support role only</t>
         </is>
       </c>
-      <c r="D52" s="3" t="inlineStr">
+      <c r="D55" s="3" t="inlineStr">
         <is>
           <t>5 items: #55–56, 61–62, 79</t>
         </is>
       </c>
-      <c r="E52" s="4">
+      <c r="E55" s="4">
         <f>IF(MIN(IF(Tracker!$G$63="Done",99999,Tracker!$F$63),IF(Tracker!$G$64="Done",99999,Tracker!$F$64),IF(Tracker!$G$69="Done",99999,Tracker!$F$69),IF(Tracker!$G$70="Done",99999,Tracker!$F$70))=99999,"—",MIN(IF(Tracker!$G$63="Done",99999,Tracker!$F$63),IF(Tracker!$G$64="Done",99999,Tracker!$F$64),IF(Tracker!$G$69="Done",99999,Tracker!$F$69),IF(Tracker!$G$70="Done",99999,Tracker!$F$70)))</f>
         <v/>
       </c>
     </row>
-    <row r="54" ht="15" customHeight="1" s="31">
-      <c r="A54" s="33" t="inlineStr">
+    <row r="57" ht="15" customHeight="1" s="31">
+      <c r="A57" s="33" t="inlineStr">
         <is>
           <t>PART-TIME FACULTY — NOT TASKED</t>
         </is>
       </c>
-      <c r="B54" s="28" t="n"/>
-      <c r="C54" s="28" t="n"/>
-      <c r="D54" s="28" t="n"/>
-      <c r="E54" s="29" t="n"/>
-    </row>
-    <row r="55" ht="135.75" customHeight="1" s="31">
-      <c r="A55" s="12" t="inlineStr">
+      <c r="B57" s="28" t="n"/>
+      <c r="C57" s="28" t="n"/>
+      <c r="D57" s="28" t="n"/>
+      <c r="E57" s="29" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="12" t="inlineStr">
         <is>
           <t>21 part-time faculty</t>
         </is>
       </c>
-      <c r="B55" s="12" t="inlineStr">
+      <c r="B58" s="12" t="inlineStr">
         <is>
           <t>Listed on the Faculty sheet because checklist item 5.1 requires every faculty member teaching general education and major courses. They carry no project tasks and sit on no committee.  Aberin, Gabriel Angelo, Adiova, Marites, Alarcon, Leuz Rafael, Cabrera, Francis, Carasco, Ryan Jay, Corpuz, Alpha Jessa, Cruz, Rommel, Empay, Jan Rhommer, Fernando, Eddyson S., Francisco, Jayson R., Francisco, Josephine Rose, Garcia, Michael Johnrein, Gomez, Donna Michelle A., Magdaong, Jennifer, Mariano, Jerick, Patiag, Glaiza Kaye, Patiag, Mark, Peralta, Ronel Evan P., Santiago, Decirae Nicole, Santos, John Vincent L., Timpac, Theodore M.</t>
         </is>
       </c>
-      <c r="C55" s="12" t="inlineStr">
+      <c r="C58" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D55" s="12" t="inlineStr">
+      <c r="D58" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E55" s="13" t="inlineStr">
+      <c r="E58" s="13" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="15" customHeight="1" s="31">
-      <c r="A57" s="35" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="35" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
       </c>
-      <c r="B57" s="15">
+      <c r="B60" s="15">
         <f>COUNT(Tracker!$A$5:$A$90)&amp;" tracker items, each with exactly one accountable owner. "&amp;COUNTIF(Faculty!$E$5:$E$59,"FT")&amp;" full-time faculty tasked; "&amp;COUNTIF(Faculty!$E$5:$E$59,"PT")&amp;" part-time faculty not tasked."</f>
         <v/>
       </c>
@@ -5333,16 +5394,16 @@
   </sheetData>
   <autoFilter ref="A4:E52"/>
   <mergeCells count="10">
-    <mergeCell ref="A21:E21"/>
-    <mergeCell ref="A34:E34"/>
-    <mergeCell ref="A26:E26"/>
+    <mergeCell ref="A30:E30"/>
+    <mergeCell ref="A57:E57"/>
     <mergeCell ref="A38:E38"/>
-    <mergeCell ref="A54:E54"/>
     <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="A42:E42"/>
     <mergeCell ref="A19:E19"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A32:E32"/>
+    <mergeCell ref="A36:E36"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" fitToHeight="0" horizontalDpi="300" verticalDpi="300"/>
@@ -6434,7 +6495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K66"/>
+  <dimension ref="A1:K65"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="31" min="1" max="1"/>
@@ -6557,7 +6618,7 @@
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>PROGRAM CHAIR (BSA and BSAIS) and VICE DEAN — owns tracker items 2, 3, 15 to 26, 71 and 72. Sole full-time author of the roughly 41 programme-specialised accountancy and AIS course descriptions and syllabi (Open Item 9); the 20 general education courses and the 13 shared business courses are lifted off this load by the two college-wide pools. Also runs the compliance audit of all eight programmes' curriculum submissions. Descriptions 9 Oct 2026, syllabi 16 Oct 2026. Records obligation on top, compulsory for all faculty: certified true copy of Transcript of Records and signed contract to HR by 30 Oct 2026 (items 12–13).</t>
+          <t>PROGRAM CHAIR (BSA and BSAIS) and VICE DEAN — owns tracker items 2, 3, 15 to 26, 71 and 72. Sole full-time author of the roughly 41 programme-specialised accountancy and AIS course descriptions and syllabi (Open Item 9); the 20 general education courses and the 13 shared business courses are lifted off this load by the two college-wide pools. Also runs the compliance audit of all eight programmes' curriculum submissions. Descriptions 9 Oct 2026, syllabi 16 Oct 2026. Records obligation on top, compulsory for all faculty: certified true copy of Transcript of Records and signed contract to HR by 30 Oct 2026 (items 12–13).  PROPOSED FIRST YEAR TRIMESTER LOADING — teaches AE11-ECO1 Managerial Economics (T1), AE15-IA1 Intermediate Accounting 1 (T2), AE22-CAC Cost Accounting and Control (T3). Writes the course description and the outcomes-based syllabus for each of those courses, for review by the Program Chair.</t>
         </is>
       </c>
       <c r="J5" s="21" t="inlineStr">
@@ -6618,7 +6679,7 @@
       </c>
       <c r="K6" s="12" t="inlineStr">
         <is>
-          <t>Part-time — not tasked.</t>
+          <t>Part-time. Not named in the First Year trimester loading — task him when the Second and Third Year loadings are drawn.</t>
         </is>
       </c>
     </row>
@@ -6654,22 +6715,22 @@
       </c>
       <c r="H7" s="12" t="inlineStr">
         <is>
-          <t>Not tasked — part-time</t>
+          <t>Curriculum &amp; Syllabi — BSA/BSAIS professional courses</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Not tasked with project work (part-time). Records obligation only, and it is compulsory: submit your certified true copy of Transcript of Records and your signed appointment / contract / letter of commitment to HR Officer Dela Cruz by 30 Oct 2026 — checklist items 5.2 and 5.3, tracker items 12 and 13.</t>
+          <t>PROPOSED FIRST YEAR TRIMESTER LOADING — teaches AE19-FINMGT Financial Management (T3). Writes the course description and the outcomes-based syllabus for each of those courses, for review by the Program Chair.</t>
         </is>
       </c>
       <c r="J7" s="23" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>#19–20, 25–26</t>
         </is>
       </c>
       <c r="K7" s="12" t="inlineStr">
         <is>
-          <t>Part-time — not tasked.</t>
+          <t>Part-time, but named in the Proposed Faculty Loading, so tasked with the courses that loading gives them.</t>
         </is>
       </c>
     </row>
@@ -6705,22 +6766,22 @@
       </c>
       <c r="H8" s="12" t="inlineStr">
         <is>
-          <t>Not tasked — part-time</t>
+          <t>Curriculum &amp; Syllabi — BSA/BSAIS professional courses</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Not tasked with project work (part-time). Records obligation only, and it is compulsory: submit your certified true copy of Transcript of Records and your signed appointment / contract / letter of commitment to HR Officer Dela Cruz by 30 Oct 2026 — checklist items 5.2 and 5.3, tracker items 12 and 13.</t>
+          <t>PROPOSED FIRST YEAR TRIMESTER LOADING — teaches CBME 1 Operations Management and TQM (T1), AE1-BL1 Law on Obligations and Contracts (T3). Writes the course description and the outcomes-based syllabus for each of those courses, for review by the Program Chair.</t>
         </is>
       </c>
       <c r="J8" s="23" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>#19–20, 25–26</t>
         </is>
       </c>
       <c r="K8" s="12" t="inlineStr">
         <is>
-          <t>Part-time — not tasked.</t>
+          <t>Part-time, but named in the Proposed Faculty Loading, so tasked with the courses that loading gives them.</t>
         </is>
       </c>
     </row>
@@ -6756,22 +6817,22 @@
       </c>
       <c r="H9" s="12" t="inlineStr">
         <is>
-          <t>Not tasked — part-time</t>
+          <t>Curriculum &amp; Syllabi — BSA/BSAIS professional courses</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Not tasked with project work (part-time). Records obligation only, and it is compulsory: submit your certified true copy of Transcript of Records and your signed appointment / contract / letter of commitment to HR Officer Dela Cruz by 30 Oct 2026 — checklist items 5.2 and 5.3, tracker items 12 and 13.</t>
+          <t>PROPOSED FIRST YEAR TRIMESTER LOADING — teaches AE13-FAR Financial Accounting and Reporting (T1), AE14-CFAS Conceptual Framework and Accounting Standards (T2). Writes the course description and the outcomes-based syllabus for each of those courses, for review by the Program Chair.</t>
         </is>
       </c>
       <c r="J9" s="23" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>#19–20, 25–26</t>
         </is>
       </c>
       <c r="K9" s="12" t="inlineStr">
         <is>
-          <t>Part-time — not tasked.</t>
+          <t>Part-time, but named in the Proposed Faculty Loading, so tasked with the courses that loading gives them.</t>
         </is>
       </c>
     </row>
@@ -6807,22 +6868,22 @@
       </c>
       <c r="H10" s="12" t="inlineStr">
         <is>
-          <t>Not tasked — part-time</t>
+          <t>Curriculum &amp; Syllabi — BSA/BSAIS professional courses</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Not tasked with project work (part-time). Records obligation only, and it is compulsory: submit your certified true copy of Transcript of Records and your signed appointment / contract / letter of commitment to HR Officer Dela Cruz by 30 Oct 2026 — checklist items 5.2 and 5.3, tracker items 12 and 13.</t>
+          <t>PROPOSED FIRST YEAR TRIMESTER LOADING — teaches AE4-MGT1 Management Science (T3). Writes the course description and the outcomes-based syllabus for each of those courses, for review by the Program Chair.</t>
         </is>
       </c>
       <c r="J10" s="23" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>#19–20, 25–26</t>
         </is>
       </c>
       <c r="K10" s="12" t="inlineStr">
         <is>
-          <t>Part-time — not tasked.</t>
+          <t>Part-time, but named in the Proposed Faculty Loading, so tasked with the courses that loading gives them.</t>
         </is>
       </c>
     </row>
@@ -7348,12 +7409,12 @@
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>PROGRAMME-SPECIALISED COURSES — BSCRIM. Write the COURSE DESCRIPTION and the OBE SYLLABUS for the BSCRIM major courses allocated to you by Chair Pisto. The allocation naming your specific courses is tracked as item 76, due 25 Sep 2026. Common syllabus template: 14-week trimester, 56 hours per 3-unit course, two examinations (midterm and final) plus one required monthly assessment and regular quizzes. Hand in to your Chair: descriptions 9 Oct 2026, syllabi 16 Oct 2026. Feeds tracker items 49 and 50. Also on the Library Collection Committee — supply BSCRIM subject title lists and accession data for items 66 and 67. Records obligation on top, compulsory for all faculty: certified true copy of Transcript of Records and signed contract to HR by 30 Oct 2026 (items 12–13).</t>
+          <t>PROGRAMME-SPECIALISED COURSES — BSCRIM. Write the COURSE DESCRIPTION and the OBE SYLLABUS for the BSCRIM major courses allocated to you by Chair Pisto. The allocation naming your specific courses is tracked as item 76, due 25 Sep 2026. Common syllabus template: 14-week trimester, 56 hours per 3-unit course, two examinations (midterm and final) plus one required monthly assessment and regular quizzes. Hand in to your Chair: descriptions 9 Oct 2026, syllabi 16 Oct 2026. Feeds tracker items 49 and 50. Also on the Library Collection Committee — supply BSCRIM subject title lists and accession data for items 66 and 67. Records obligation on top, compulsory for all faculty: certified true copy of Transcript of Records and signed contract to HR by 30 Oct 2026 (items 12–13).  PROPOSED FIRST YEAR TRIMESTER LOADING — teaches NSTP 1 (T1) and NSTP 2 (T2), Civic Welfare Training Service. Writes the course description and the outcomes-based syllabus for each of those courses, for review by the Program Chair.</t>
         </is>
       </c>
       <c r="J22" s="21" t="inlineStr">
         <is>
-          <t>#49–50, 66–67</t>
+          <t>#49–50, 66–67, #19–20, 25–26</t>
         </is>
       </c>
       <c r="K22" s="3" t="n"/>
@@ -8339,7 +8400,7 @@
       </c>
       <c r="I43" s="3" t="inlineStr">
         <is>
-          <t>GENERAL EDUCATION SYLLABI POOL (tracker item 74) — write the COURSE DESCRIPTION and the OBE SYLLABUS for 3 allocated courses, one set serving all 8 programmes: PATH-FIT 1 Movement Competency Training; PATH-FIT 2 Exercise-Based Fitness Activities; NSTP 1 Civic Welfare Training Service 1. 6 documents in total. Common syllabus template: 14-week trimester, 56 hours per 3-unit course, two examinations (midterm and final) plus one required monthly assessment and regular quizzes. Hand in to Chair Kent E. Garcia: descriptions 9 Oct 2026, syllabi 16 Oct 2026. Course codes are the BSA/BSAIS spellings — reconcile with your own programme's codes once Open Item 7 is closed. Not included in the BEED/BSED specialised allocation (item 79) while carrying this pool load. NSTP 1 is the prerequisite of NSTP 2 and the two are split between Calma and Mequiabas — agree the two syllabi between you so the sequence holds. Records obligation on top, compulsory for all faculty: certified true copy of Transcript of Records and signed contract to HR by 30 Oct 2026 (items 12–13).</t>
+          <t>GENERAL EDUCATION SYLLABI POOL (tracker item 74) — write the COURSE DESCRIPTION and the OBE SYLLABUS for 3 allocated courses, one set serving all 8 programmes: PATH-FIT 1 Movement Competency Training; PATH-FIT 2 Exercise-Based Fitness Activities; NSTP 1 Civic Welfare Training Service 1. 6 documents in total. Common syllabus template: 14-week trimester, 56 hours per 3-unit course, two examinations (midterm and final) plus one required monthly assessment and regular quizzes. Hand in to Chair Kent E. Garcia: descriptions 9 Oct 2026, syllabi 16 Oct 2026. Course codes are the BSA/BSAIS spellings — reconcile with your own programme's codes once Open Item 7 is closed. Not included in the BEED/BSED specialised allocation (item 79) while carrying this pool load. NSTP 1 is the prerequisite of NSTP 2 and the two are split between Calma and Mequiabas — agree the two syllabi between you so the sequence holds. Records obligation on top, compulsory for all faculty: certified true copy of Transcript of Records and signed contract to HR by 30 Oct 2026 (items 12–13).  PROPOSED FIRST YEAR TRIMESTER LOADING — teaches PATH-FIT 1 Movement Competency Training (T1). Writes the course description and the outcomes-based syllabus for each of those courses, for review by the Program Chair.</t>
         </is>
       </c>
       <c r="J43" s="21" t="inlineStr">
@@ -8518,17 +8579,17 @@
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>Curriculum &amp; Syllabi — BEED/BSED</t>
+          <t>Curriculum &amp; Syllabi — BEED/BSED; General Education Syllabi Pool</t>
         </is>
       </c>
       <c r="I47" s="3" t="inlineStr">
         <is>
-          <t>PROGRAMME-SPECIALISED COURSES — BEED and BSED. Write the COURSE DESCRIPTION and the OBE SYLLABUS for the BEED and BSED major courses allocated to you by Chair K. Garcia. The allocation naming your specific courses is tracked as item 79, due 25 Sep 2026. Common syllabus template: 14-week trimester, 56 hours per 3-unit course, two examinations (midterm and final) plus one required monthly assessment and regular quizzes. Hand in to your Chair: descriptions 9 Oct 2026, syllabi 16 Oct 2026. Feeds tracker items 55 and 56 (BEED) and 61 and 62 (BSED). Records obligation on top, compulsory for all faculty: certified true copy of Transcript of Records and signed contract to HR by 30 Oct 2026 (items 12–13).</t>
+          <t>PROGRAMME-SPECIALISED COURSES — BEED and BSED. Write the COURSE DESCRIPTION and the OBE SYLLABUS for the BEED and BSED major courses allocated to you by Chair K. Garcia. The allocation naming your specific courses is tracked as item 79, due 25 Sep 2026. Common syllabus template: 14-week trimester, 56 hours per 3-unit course, two examinations (midterm and final) plus one required monthly assessment and regular quizzes. Hand in to your Chair: descriptions 9 Oct 2026, syllabi 16 Oct 2026. Feeds tracker items 55 and 56 (BEED) and 61 and 62 (BSED). Records obligation on top, compulsory for all faculty: certified true copy of Transcript of Records and signed contract to HR by 30 Oct 2026 (items 12–13).  PROPOSED FIRST YEAR TRIMESTER LOADING — teaches MAT-GEC Mathematics in the Modern World and HIS-GEC Readings in Philippine History (T1). Writes the course description and the outcomes-based syllabus for each of those courses, for review by the Program Chair.  GENERAL EDUCATION SYLLABI POOL (tracker item 74) — writes the course description and the OBE syllabus for HIS-GEC Readings in Philippine History, reallocated from D. Maglalang on her resignation, 26 Oct 2026.</t>
         </is>
       </c>
       <c r="J47" s="21" t="inlineStr">
         <is>
-          <t>#55–56, 61–62</t>
+          <t>#55–56, 61–62, #19–20, 25–26, 74</t>
         </is>
       </c>
       <c r="K47" s="3" t="n"/>
@@ -8566,7 +8627,7 @@
       </c>
       <c r="I48" s="3" t="inlineStr">
         <is>
-          <t>GENERAL EDUCATION SYLLABI POOL (tracker item 74) — write the COURSE DESCRIPTION and the OBE SYLLABUS for 3 allocated courses, one set serving all 8 programmes: REL-GEC Religion, Religious Experience and Spirituality; CLE 1 Church and Salvation History; STS-GEC Science, Technology and Society. 6 documents in total. Common syllabus template: 14-week trimester, 56 hours per 3-unit course, two examinations (midterm and final) plus one required monthly assessment and regular quizzes. Hand in to Chair Kent E. Garcia: descriptions 9 Oct 2026, syllabi 16 Oct 2026. Course codes are the BSA/BSAIS spellings — reconcile with your own programme's codes once Open Item 7 is closed. Not included in the BEED/BSED specialised allocation (item 79) while carrying this pool load. Records obligation on top, compulsory for all faculty: certified true copy of Transcript of Records and signed contract to HR by 30 Oct 2026 (items 12–13).</t>
+          <t>GENERAL EDUCATION SYLLABI POOL (tracker item 74) — write the COURSE DESCRIPTION and the OBE SYLLABUS for 3 allocated courses, one set serving all 8 programmes: REL-GEC Religion, Religious Experience and Spirituality; CLE 1 Church and Salvation History; STS-GEC Science, Technology and Society. 6 documents in total. Common syllabus template: 14-week trimester, 56 hours per 3-unit course, two examinations (midterm and final) plus one required monthly assessment and regular quizzes. Hand in to Chair Kent E. Garcia: descriptions 9 Oct 2026, syllabi 16 Oct 2026. Course codes are the BSA/BSAIS spellings — reconcile with your own programme's codes once Open Item 7 is closed. Not included in the BEED/BSED specialised allocation (item 79) while carrying this pool load. Records obligation on top, compulsory for all faculty: certified true copy of Transcript of Records and signed contract to HR by 30 Oct 2026 (items 12–13).  PROPOSED FIRST YEAR TRIMESTER LOADING — teaches REL-GEC Religion, Religious Experience and Spirituality (T2), CLE 1 Church and Salvation History (T3) — CLE 1 reassigned from D. Maglalang, resigned. Writes the course description and the outcomes-based syllabus for each of those courses, for review by the Program Chair.  Also takes CLE 2 in the GE pool, reallocated from D. Maglalang, 26 Oct 2026.</t>
         </is>
       </c>
       <c r="J48" s="21" t="inlineStr">
@@ -8609,7 +8670,7 @@
       </c>
       <c r="I49" s="3" t="inlineStr">
         <is>
-          <t>GENERAL EDUCATION SYLLABI POOL (tracker item 74) — write the COURSE DESCRIPTION and the OBE SYLLABUS for 2 allocated courses, one set serving all 8 programmes: CON-GEC The Contemporary World; ITE-GEC Living in the I.T. Era. 4 documents in total. Common syllabus template: 14-week trimester, 56 hours per 3-unit course, two examinations (midterm and final) plus one required monthly assessment and regular quizzes. Hand in to Chair Kent E. Garcia: descriptions 9 Oct 2026, syllabi 16 Oct 2026. Course codes are the BSA/BSAIS spellings — reconcile with your own programme's codes once Open Item 7 is closed. Not included in the BEED/BSED specialised allocation (item 79) while carrying this pool load. Records obligation on top, compulsory for all faculty: certified true copy of Transcript of Records and signed contract to HR by 30 Oct 2026 (items 12–13).</t>
+          <t>GENERAL EDUCATION SYLLABI POOL (tracker item 74) — write the COURSE DESCRIPTION and the OBE SYLLABUS for 2 allocated courses, one set serving all 8 programmes: CON-GEC The Contemporary World; ITE-GEC Living in the I.T. Era. 4 documents in total. Common syllabus template: 14-week trimester, 56 hours per 3-unit course, two examinations (midterm and final) plus one required monthly assessment and regular quizzes. Hand in to Chair Kent E. Garcia: descriptions 9 Oct 2026, syllabi 16 Oct 2026. Course codes are the BSA/BSAIS spellings — reconcile with your own programme's codes once Open Item 7 is closed. Not included in the BEED/BSED specialised allocation (item 79) while carrying this pool load. Records obligation on top, compulsory for all faculty: certified true copy of Transcript of Records and signed contract to HR by 30 Oct 2026 (items 12–13).  PROPOSED FIRST YEAR TRIMESTER LOADING — teaches RIZ-GEC The Life and Works of Rizal (T3). Writes the course description and the outcomes-based syllabus for each of those courses, for review by the Program Chair.  Also takes RIZ-GEC in the GE pool, reallocated from D. Maglalang, 26 Oct 2026.</t>
         </is>
       </c>
       <c r="J49" s="21" t="inlineStr">
@@ -8625,10 +8686,14 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>Maglalang, Danica</t>
-        </is>
-      </c>
-      <c r="C50" s="21" t="n"/>
+          <t>Manuel, Consuelo V.</t>
+        </is>
+      </c>
+      <c r="C50" s="21" t="inlineStr">
+        <is>
+          <t>Dr.</t>
+        </is>
+      </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
           <t>Teacher Education (BEED / BSEDE / BSEDM / TEP)</t>
@@ -8643,7 +8708,7 @@
         <v>24</v>
       </c>
       <c r="G50" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H50" s="3" t="inlineStr">
         <is>
@@ -8652,7 +8717,7 @@
       </c>
       <c r="I50" s="3" t="inlineStr">
         <is>
-          <t>GENERAL EDUCATION SYLLABI POOL (tracker item 74) — write the COURSE DESCRIPTION and the OBE SYLLABUS for 3 allocated courses, one set serving all 8 programmes: CLE 2 Evangelism and Discipleship; HIS-GEC Readings in Philippine History; RIZ-GEC Rizal's Life and Works. 6 documents in total. Common syllabus template: 14-week trimester, 56 hours per 3-unit course, two examinations (midterm and final) plus one required monthly assessment and regular quizzes. Hand in to Chair Kent E. Garcia: descriptions 9 Oct 2026, syllabi 16 Oct 2026. Course codes are the BSA/BSAIS spellings — reconcile with your own programme's codes once Open Item 7 is closed. Not included in the BEED/BSED specialised allocation (item 79) while carrying this pool load. Records obligation on top, compulsory for all faculty: certified true copy of Transcript of Records and signed contract to HR by 30 Oct 2026 (items 12–13).</t>
+          <t>GENERAL EDUCATION SYLLABI POOL (tracker item 74) — write the COURSE DESCRIPTION and the OBE SYLLABUS for 3 allocated courses, one set serving all 8 programmes: ETH-GEC Ethics; MAT-GEC Mathematics in the Modern World; BL-GEC Business Logic. 6 documents in total. Common syllabus template: 14-week trimester, 56 hours per 3-unit course, two examinations (midterm and final) plus one required monthly assessment and regular quizzes. Hand in to Chair Kent E. Garcia: descriptions 9 Oct 2026, syllabi 16 Oct 2026. Course codes are the BSA/BSAIS spellings — reconcile with your own programme's codes once Open Item 7 is closed. Not included in the BEED/BSED specialised allocation (item 79) while carrying this pool load. Records obligation on top, compulsory for all faculty: certified true copy of Transcript of Records and signed contract to HR by 30 Oct 2026 (items 12–13).</t>
         </is>
       </c>
       <c r="J50" s="21" t="inlineStr">
@@ -8668,14 +8733,10 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>Manuel, Consuelo V.</t>
-        </is>
-      </c>
-      <c r="C51" s="21" t="inlineStr">
-        <is>
-          <t>Dr.</t>
-        </is>
-      </c>
+          <t>Mequiabas, Meah</t>
+        </is>
+      </c>
+      <c r="C51" s="21" t="n"/>
       <c r="D51" s="3" t="inlineStr">
         <is>
           <t>Teacher Education (BEED / BSEDE / BSEDM / TEP)</t>
@@ -8687,7 +8748,7 @@
         </is>
       </c>
       <c r="F51" s="2" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G51" s="2" t="n">
         <v>4</v>
@@ -8699,7 +8760,7 @@
       </c>
       <c r="I51" s="3" t="inlineStr">
         <is>
-          <t>GENERAL EDUCATION SYLLABI POOL (tracker item 74) — write the COURSE DESCRIPTION and the OBE SYLLABUS for 3 allocated courses, one set serving all 8 programmes: ETH-GEC Ethics; MAT-GEC Mathematics in the Modern World; BL-GEC Business Logic. 6 documents in total. Common syllabus template: 14-week trimester, 56 hours per 3-unit course, two examinations (midterm and final) plus one required monthly assessment and regular quizzes. Hand in to Chair Kent E. Garcia: descriptions 9 Oct 2026, syllabi 16 Oct 2026. Course codes are the BSA/BSAIS spellings — reconcile with your own programme's codes once Open Item 7 is closed. Not included in the BEED/BSED specialised allocation (item 79) while carrying this pool load. Records obligation on top, compulsory for all faculty: certified true copy of Transcript of Records and signed contract to HR by 30 Oct 2026 (items 12–13).</t>
+          <t>GENERAL EDUCATION SYLLABI POOL (tracker item 74) — write the COURSE DESCRIPTION and the OBE SYLLABUS for 3 allocated courses, one set serving all 8 programmes: PATH-FIT 3 Dance; PATH-FIT 4 Sports; NSTP 2 Civic Welfare Training Service 2. 6 documents in total. Common syllabus template: 14-week trimester, 56 hours per 3-unit course, two examinations (midterm and final) plus one required monthly assessment and regular quizzes. Hand in to Chair Kent E. Garcia: descriptions 9 Oct 2026, syllabi 16 Oct 2026. Course codes are the BSA/BSAIS spellings — reconcile with your own programme's codes once Open Item 7 is closed. Not included in the BEED/BSED specialised allocation (item 79) while carrying this pool load. NSTP 1 is the prerequisite of NSTP 2 and the two are split between Calma and Mequiabas — agree the two syllabi between you so the sequence holds. Records obligation on top, compulsory for all faculty: certified true copy of Transcript of Records and signed contract to HR by 30 Oct 2026 (items 12–13).  PROPOSED FIRST YEAR TRIMESTER LOADING — teaches ART-GEC Art Appreciation and PATH-FIT 2 (T2), PATH-FIT 3 Dance (T3). Writes the course description and the outcomes-based syllabus for each of those courses, for review by the Program Chair.</t>
         </is>
       </c>
       <c r="J51" s="21" t="inlineStr">
@@ -8715,7 +8776,7 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>Mequiabas, Meah</t>
+          <t>Sta. Cruz, Ma. Patricia</t>
         </is>
       </c>
       <c r="C52" s="21" t="n"/>
@@ -8730,27 +8791,31 @@
         </is>
       </c>
       <c r="F52" s="2" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G52" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H52" s="3" t="inlineStr">
         <is>
-          <t>Curriculum &amp; Syllabi — BEED/BSED; General Education Syllabi Pool (college-wide)</t>
+          <t>Curriculum &amp; Syllabi — BEED/BSED; Library Collection</t>
         </is>
       </c>
       <c r="I52" s="3" t="inlineStr">
         <is>
-          <t>GENERAL EDUCATION SYLLABI POOL (tracker item 74) — write the COURSE DESCRIPTION and the OBE SYLLABUS for 3 allocated courses, one set serving all 8 programmes: PATH-FIT 3 Dance; PATH-FIT 4 Sports; NSTP 2 Civic Welfare Training Service 2. 6 documents in total. Common syllabus template: 14-week trimester, 56 hours per 3-unit course, two examinations (midterm and final) plus one required monthly assessment and regular quizzes. Hand in to Chair Kent E. Garcia: descriptions 9 Oct 2026, syllabi 16 Oct 2026. Course codes are the BSA/BSAIS spellings — reconcile with your own programme's codes once Open Item 7 is closed. Not included in the BEED/BSED specialised allocation (item 79) while carrying this pool load. NSTP 1 is the prerequisite of NSTP 2 and the two are split between Calma and Mequiabas — agree the two syllabi between you so the sequence holds. Records obligation on top, compulsory for all faculty: certified true copy of Transcript of Records and signed contract to HR by 30 Oct 2026 (items 12–13).</t>
+          <t>PROGRAMME-SPECIALISED COURSES — BEED and BSED. Write the COURSE DESCRIPTION and the OBE SYLLABUS for the BEED and BSED major courses allocated to you by Chair K. Garcia. The allocation naming your specific courses is tracked as item 79, due 25 Sep 2026. Common syllabus template: 14-week trimester, 56 hours per 3-unit course, two examinations (midterm and final) plus one required monthly assessment and regular quizzes. Hand in to your Chair: descriptions 9 Oct 2026, syllabi 16 Oct 2026. Feeds tracker items 55 and 56 (BEED) and 61 and 62 (BSED). Also a named member of the library team — owns the working papers behind items 66 to 69 with Bernardo, on top of a 27-unit teaching load. Weight your course share accordingly with the Chair. Records obligation on top, compulsory for all faculty: certified true copy of Transcript of Records and signed contract to HR by 30 Oct 2026 (items 12–13).</t>
         </is>
       </c>
       <c r="J52" s="21" t="inlineStr">
         <is>
-          <t>#19–20, 25–26, 31–32, 37–38, 43–44, 49–50, 55–56, 61–62</t>
-        </is>
-      </c>
-      <c r="K52" s="3" t="n"/>
+          <t>#55–56, 61–62, 66–69</t>
+        </is>
+      </c>
+      <c r="K52" s="3" t="inlineStr">
+        <is>
+          <t>Also a member of the library team named in the project plan — library duty on top of a full teaching load.</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="35" customHeight="1" s="31">
       <c r="A53" s="2" t="n">
@@ -8758,7 +8823,7 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>Sta. Cruz, Ma. Patricia</t>
+          <t>Tolosa, Nenita</t>
         </is>
       </c>
       <c r="C53" s="21" t="n"/>
@@ -8773,31 +8838,27 @@
         </is>
       </c>
       <c r="F53" s="2" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="G53" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H53" s="3" t="inlineStr">
         <is>
-          <t>Curriculum &amp; Syllabi — BEED/BSED; Library Collection</t>
+          <t>Curriculum &amp; Syllabi — BEED/BSED; General Education Syllabi Pool (college-wide)</t>
         </is>
       </c>
       <c r="I53" s="3" t="inlineStr">
         <is>
-          <t>PROGRAMME-SPECIALISED COURSES — BEED and BSED. Write the COURSE DESCRIPTION and the OBE SYLLABUS for the BEED and BSED major courses allocated to you by Chair K. Garcia. The allocation naming your specific courses is tracked as item 79, due 25 Sep 2026. Common syllabus template: 14-week trimester, 56 hours per 3-unit course, two examinations (midterm and final) plus one required monthly assessment and regular quizzes. Hand in to your Chair: descriptions 9 Oct 2026, syllabi 16 Oct 2026. Feeds tracker items 55 and 56 (BEED) and 61 and 62 (BSED). Also a named member of the library team — owns the working papers behind items 66 to 69 with Bernardo, on top of a 27-unit teaching load. Weight your course share accordingly with the Chair. Records obligation on top, compulsory for all faculty: certified true copy of Transcript of Records and signed contract to HR by 30 Oct 2026 (items 12–13).</t>
+          <t>GENERAL EDUCATION SYLLABI POOL (tracker item 74) — write the COURSE DESCRIPTION and the OBE SYLLABUS for 3 allocated courses, one set serving all 8 programmes: ART-GEC Art Appreciation; COM-GEC Purposive Communication; US-GEC Understanding the Self. 6 documents in total. Common syllabus template: 14-week trimester, 56 hours per 3-unit course, two examinations (midterm and final) plus one required monthly assessment and regular quizzes. Hand in to Chair Kent E. Garcia: descriptions 9 Oct 2026, syllabi 16 Oct 2026. Course codes are the BSA/BSAIS spellings — reconcile with your own programme's codes once Open Item 7 is closed. Not included in the BEED/BSED specialised allocation (item 79) while carrying this pool load. Records obligation on top, compulsory for all faculty: certified true copy of Transcript of Records and signed contract to HR by 30 Oct 2026 (items 12–13).  PROPOSED FIRST YEAR TRIMESTER LOADING — teaches US-GEC Understanding the Self (T1). Writes the course description and the outcomes-based syllabus for each of those courses, for review by the Program Chair.</t>
         </is>
       </c>
       <c r="J53" s="21" t="inlineStr">
         <is>
-          <t>#55–56, 61–62, 66–69</t>
-        </is>
-      </c>
-      <c r="K53" s="3" t="inlineStr">
-        <is>
-          <t>Also a member of the library team named in the project plan — library duty on top of a full teaching load.</t>
-        </is>
-      </c>
+          <t>#19–20, 25–26, 31–32, 37–38, 43–44, 49–50, 55–56, 61–62</t>
+        </is>
+      </c>
+      <c r="K53" s="3" t="n"/>
     </row>
     <row r="54" ht="23.75" customHeight="1" s="31">
       <c r="A54" s="2" t="n">
@@ -8805,7 +8866,7 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>Tolosa, Nenita</t>
+          <t>Villamayor, Xyrelle</t>
         </is>
       </c>
       <c r="C54" s="21" t="n"/>
@@ -8820,70 +8881,74 @@
         </is>
       </c>
       <c r="F54" s="2" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="G54" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H54" s="3" t="inlineStr">
         <is>
-          <t>Curriculum &amp; Syllabi — BEED/BSED; General Education Syllabi Pool (college-wide)</t>
+          <t>Curriculum &amp; Syllabi — BEED/BSED</t>
         </is>
       </c>
       <c r="I54" s="3" t="inlineStr">
         <is>
-          <t>GENERAL EDUCATION SYLLABI POOL (tracker item 74) — write the COURSE DESCRIPTION and the OBE SYLLABUS for 3 allocated courses, one set serving all 8 programmes: ART-GEC Art Appreciation; COM-GEC Purposive Communication; US-GEC Understanding the Self. 6 documents in total. Common syllabus template: 14-week trimester, 56 hours per 3-unit course, two examinations (midterm and final) plus one required monthly assessment and regular quizzes. Hand in to Chair Kent E. Garcia: descriptions 9 Oct 2026, syllabi 16 Oct 2026. Course codes are the BSA/BSAIS spellings — reconcile with your own programme's codes once Open Item 7 is closed. Not included in the BEED/BSED specialised allocation (item 79) while carrying this pool load. Records obligation on top, compulsory for all faculty: certified true copy of Transcript of Records and signed contract to HR by 30 Oct 2026 (items 12–13).</t>
+          <t>PROGRAMME-SPECIALISED COURSES — BEED and BSED. Write the COURSE DESCRIPTION and the OBE SYLLABUS for the BEED and BSED major courses allocated to you by Chair K. Garcia. The allocation naming your specific courses is tracked as item 79, due 25 Sep 2026. Common syllabus template: 14-week trimester, 56 hours per 3-unit course, two examinations (midterm and final) plus one required monthly assessment and regular quizzes. Hand in to your Chair: descriptions 9 Oct 2026, syllabi 16 Oct 2026. Feeds tracker items 55 and 56 (BEED) and 61 and 62 (BSED). Records obligation on top, compulsory for all faculty: certified true copy of Transcript of Records and signed contract to HR by 30 Oct 2026 (items 12–13).  PROPOSED FIRST YEAR TRIMESTER LOADING — teaches COM-GEC Purposive Communication (T2), CON-GEC The Contemporary World (T3). Writes the course description and the outcomes-based syllabus for each of those courses, for review by the Program Chair.</t>
         </is>
       </c>
       <c r="J54" s="21" t="inlineStr">
         <is>
-          <t>#19–20, 25–26, 31–32, 37–38, 43–44, 49–50, 55–56, 61–62</t>
+          <t>#55–56, 61–62, #19–20, 25–26</t>
         </is>
       </c>
       <c r="K54" s="3" t="n"/>
     </row>
     <row r="55" ht="23.75" customHeight="1" s="31">
-      <c r="A55" s="2" t="n">
+      <c r="A55" s="22" t="n">
         <v>51</v>
       </c>
-      <c r="B55" s="3" t="inlineStr">
-        <is>
-          <t>Villamayor, Xyrelle</t>
-        </is>
-      </c>
-      <c r="C55" s="21" t="n"/>
-      <c r="D55" s="3" t="inlineStr">
+      <c r="B55" s="12" t="inlineStr">
+        <is>
+          <t>Adiova, Marites</t>
+        </is>
+      </c>
+      <c r="C55" s="23" t="n"/>
+      <c r="D55" s="12" t="inlineStr">
         <is>
           <t>Teacher Education (BEED / BSEDE / BSEDM / TEP)</t>
         </is>
       </c>
-      <c r="E55" s="2" t="inlineStr">
-        <is>
-          <t>FT</t>
-        </is>
-      </c>
-      <c r="F55" s="2" t="n">
-        <v>27</v>
-      </c>
-      <c r="G55" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="H55" s="3" t="inlineStr">
-        <is>
-          <t>Curriculum &amp; Syllabi — BEED/BSED</t>
+      <c r="E55" s="22" t="inlineStr">
+        <is>
+          <t>PT</t>
+        </is>
+      </c>
+      <c r="F55" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="G55" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="H55" s="12" t="inlineStr">
+        <is>
+          <t>Not tasked — part-time</t>
         </is>
       </c>
       <c r="I55" s="3" t="inlineStr">
         <is>
-          <t>PROGRAMME-SPECIALISED COURSES — BEED and BSED. Write the COURSE DESCRIPTION and the OBE SYLLABUS for the BEED and BSED major courses allocated to you by Chair K. Garcia. The allocation naming your specific courses is tracked as item 79, due 25 Sep 2026. Common syllabus template: 14-week trimester, 56 hours per 3-unit course, two examinations (midterm and final) plus one required monthly assessment and regular quizzes. Hand in to your Chair: descriptions 9 Oct 2026, syllabi 16 Oct 2026. Feeds tracker items 55 and 56 (BEED) and 61 and 62 (BSED). Records obligation on top, compulsory for all faculty: certified true copy of Transcript of Records and signed contract to HR by 30 Oct 2026 (items 12–13).</t>
-        </is>
-      </c>
-      <c r="J55" s="21" t="inlineStr">
-        <is>
-          <t>#55–56, 61–62</t>
-        </is>
-      </c>
-      <c r="K55" s="3" t="n"/>
+          <t>Not tasked with project work (part-time). Records obligation only, and it is compulsory: submit your certified true copy of Transcript of Records and your signed appointment / contract / letter of commitment to HR Officer Dela Cruz by 30 Oct 2026 — checklist items 5.2 and 5.3, tracker items 12 and 13.</t>
+        </is>
+      </c>
+      <c r="J55" s="23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K55" s="12" t="inlineStr">
+        <is>
+          <t>Part-time — not tasked.</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="23.75" customHeight="1" s="31">
       <c r="A56" s="22" t="n">
@@ -8891,7 +8956,7 @@
       </c>
       <c r="B56" s="12" t="inlineStr">
         <is>
-          <t>Adiova, Marites</t>
+          <t>Cabrera, Francis</t>
         </is>
       </c>
       <c r="C56" s="23" t="n"/>
@@ -8938,7 +9003,7 @@
       </c>
       <c r="B57" s="12" t="inlineStr">
         <is>
-          <t>Cabrera, Francis</t>
+          <t>Gomez, Donna Michelle A.</t>
         </is>
       </c>
       <c r="C57" s="23" t="n"/>
@@ -8953,7 +9018,7 @@
         </is>
       </c>
       <c r="F57" s="22" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="G57" s="22" t="n">
         <v>1</v>
@@ -8985,7 +9050,7 @@
       </c>
       <c r="B58" s="12" t="inlineStr">
         <is>
-          <t>Gomez, Donna Michelle A.</t>
+          <t>Magdaong, Jennifer</t>
         </is>
       </c>
       <c r="C58" s="23" t="n"/>
@@ -9000,7 +9065,7 @@
         </is>
       </c>
       <c r="F58" s="22" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="G58" s="22" t="n">
         <v>1</v>
@@ -9026,125 +9091,80 @@
         </is>
       </c>
     </row>
-    <row r="59" ht="23.75" customHeight="1" s="31">
-      <c r="A59" s="22" t="n">
-        <v>55</v>
-      </c>
-      <c r="B59" s="12" t="inlineStr">
-        <is>
-          <t>Magdaong, Jennifer</t>
-        </is>
-      </c>
-      <c r="C59" s="23" t="n"/>
-      <c r="D59" s="12" t="inlineStr">
-        <is>
-          <t>Teacher Education (BEED / BSEDE / BSEDM / TEP)</t>
-        </is>
-      </c>
-      <c r="E59" s="22" t="inlineStr">
-        <is>
-          <t>PT</t>
-        </is>
-      </c>
-      <c r="F59" s="22" t="n">
-        <v>3</v>
-      </c>
-      <c r="G59" s="22" t="n">
-        <v>1</v>
-      </c>
-      <c r="H59" s="12" t="inlineStr">
-        <is>
-          <t>Not tasked — part-time</t>
-        </is>
-      </c>
-      <c r="I59" s="3" t="inlineStr">
-        <is>
-          <t>Not tasked with project work (part-time). Records obligation only, and it is compulsory: submit your certified true copy of Transcript of Records and your signed appointment / contract / letter of commitment to HR Officer Dela Cruz by 30 Oct 2026 — checklist items 5.2 and 5.3, tracker items 12 and 13.</t>
-        </is>
-      </c>
-      <c r="J59" s="23" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K59" s="12" t="inlineStr">
-        <is>
-          <t>Part-time — not tasked.</t>
-        </is>
+    <row r="59" ht="23.75" customHeight="1" s="31"/>
+    <row r="60">
+      <c r="A60" s="35" t="inlineStr">
+        <is>
+          <t>Unique faculty</t>
+        </is>
+      </c>
+      <c r="D60" s="15">
+        <f>COUNTA($B$5:$B$59)</f>
+        <v/>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="31">
       <c r="A61" s="35" t="inlineStr">
         <is>
-          <t>Unique faculty</t>
+          <t>Full-time (tasked)</t>
         </is>
       </c>
       <c r="D61" s="15">
-        <f>COUNTA($B$5:$B$59)</f>
+        <f>COUNTIF($E$5:$E$59,"FT")</f>
         <v/>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="31">
       <c r="A62" s="35" t="inlineStr">
         <is>
-          <t>Full-time (tasked)</t>
+          <t>Part-time (not tasked)</t>
         </is>
       </c>
       <c r="D62" s="15">
-        <f>COUNTIF($E$5:$E$59,"FT")</f>
+        <f>COUNTIF($E$5:$E$59,"PT")</f>
         <v/>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="31">
       <c r="A63" s="35" t="inlineStr">
         <is>
-          <t>Part-time (not tasked)</t>
+          <t>Full-time faculty available to task (excluding the Dean, the Vice Dean and the 5 Programme Chairs; the MIS Head is on this roster as part-time)</t>
         </is>
       </c>
       <c r="D63" s="15">
-        <f>COUNTIF($E$5:$E$59,"PT")</f>
+        <f>COUNTIF($E$5:$E$59,"FT")-7</f>
         <v/>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="31">
       <c r="A64" s="35" t="inlineStr">
         <is>
-          <t>Full-time faculty available to task (excluding the Dean, the Vice Dean and the 5 Programme Chairs; the MIS Head is on this roster as part-time)</t>
+          <t>Total units carried this semester</t>
         </is>
       </c>
       <c r="D64" s="15">
-        <f>COUNTIF($E$5:$E$59,"FT")-7</f>
+        <f>SUM($F$5:$F$59)</f>
         <v/>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="31">
       <c r="A65" s="35" t="inlineStr">
         <is>
-          <t>Total units carried this semester</t>
+          <t>Average units per faculty</t>
         </is>
       </c>
       <c r="D65" s="15">
-        <f>SUM($F$5:$F$59)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="66" ht="15" customHeight="1" s="31">
-      <c r="A66" s="35" t="inlineStr">
-        <is>
-          <t>Average units per faculty</t>
-        </is>
-      </c>
-      <c r="D66" s="15">
         <f>ROUND(AVERAGE($F$5:$F$59),1)</f>
         <v/>
       </c>
     </row>
+    <row r="66" ht="15" customHeight="1" s="31"/>
   </sheetData>
   <autoFilter ref="A4:J59"/>
   <mergeCells count="8">
     <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A60:C60"/>
     <mergeCell ref="A63:C63"/>
-    <mergeCell ref="A66:C66"/>
     <mergeCell ref="A61:C61"/>
     <mergeCell ref="A62:C62"/>
     <mergeCell ref="A2:J2"/>
@@ -9162,7 +9182,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" style="31" min="1" max="1"/>
@@ -9524,7 +9544,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Feasibility study for the conversion of the BSA to a 3-year trimester delivery — description, management viability (administrator matrix), market viability (five-year enrolment projection from 30 first-year enrollees growing 10% a year), financial viability, matters to be supplied, conclusion and recommendation; cites the College's graduate survey (95% of BSA and BSAIS graduates gainfully employed in their field) and, for BSA, the first CPALE batch (4 passers of 6)</t>
+          <t>Feasibility study for the conversion of the BSA to a 3-year trimester delivery — description, management viability (administrator matrix), market viability (five-year enrolment projection from 30 first-year enrollees growing 10% a year), financial viability, matters to be supplied, conclusion and recommendation; cites the Graduate Tracer Study, Batch May 2025 (28 of 30 graduates employed in their field — 93% overall, BSA 95%, BSAIS 90%) and, for BSA, the first CPALE batch (4 passers of 6)</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -9554,7 +9574,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Feasibility study for the conversion of the BSAIS to a 3-year trimester delivery — same structure, projected from 25 first-year enrollees growing 10% a year; cites the College's graduate survey (95% of BSA and BSAIS graduates gainfully employed in their field) and, for BSA, the first CPALE batch (4 passers of 6)</t>
+          <t>Feasibility study for the conversion of the BSAIS to a 3-year trimester delivery — same structure, projected from 25 first-year enrollees growing 10% a year; cites the Graduate Tracer Study, Batch May 2025 (28 of 30 graduates employed in their field — 93% overall, BSA 95%, BSAIS 90%) and, for BSA, the first CPALE batch (4 passers of 6)</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
@@ -9638,7 +9658,7 @@
         </is>
       </c>
     </row>
-    <row r="19">
+    <row r="19" s="31">
       <c r="A19" s="4" t="n">
         <v>46288</v>
       </c>
@@ -9668,22 +9688,111 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
+    <row r="20" s="31">
+      <c r="A20" s="4" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Graduate Tracer Study, Batch of May 2025, worked into both feasibility studies — 30 graduates, 28 employed in work related to their field (93%; BSA 19 of 20, BSAIS 9 of 10), time from graduation to hiring, and the employers. Replaces the earlier 95% placeholder. Two entries in the raw file are still open: graduates recorded as employed with no employer named</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Program Chair, BSA &amp; BSAIS</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Items 4, 5; supports items 3, 6</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>For review</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>BSA &amp; BSAIS Outputs/Feasibility Study — workbook, Word and PDF</t>
+        </is>
+      </c>
+    </row>
     <row r="21">
-      <c r="A21" s="35" t="inlineStr">
+      <c r="A21" s="4" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Faculty tasking rebuilt off the Proposed Faculty Loading — the four CPAs who carry the professional courses (J.R. Francisco, J.R. Empay, D.N. Santiago, R. Cruz) now own the course descriptions and syllabi for the courses that loading gives them, and the GE, PATH-FIT, NSTP and CLE teachers are named against theirs, instead of all of it sitting on the Vice Dean. D. Maglalang removed on resignation: CLE 1 in Trimester 3 to F. Ilag, and her three GE pool courses to Ilag (CLE 2), Germino (HIS-GEC) and Jamlang (RIZ-GEC)</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Program Chair, BSA &amp; BSAIS</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Items 19–20, 25–26, 74</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>For review</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Tracker — Faculty, Assignments; Faculty Matrix &amp; Loading</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Course syllabi, outcomes-based, for all remaining BSA and BSAIS courses (64 new drafts; 73 courses covered with the existing samples) — 14-week / 56-hour basis, mapped to the programme outcomes; references blank</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Program Chair, BSA &amp; BSAIS</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Items 20, 26; supports items 74, 75</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>For review</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>BSA &amp; BSAIS Outputs/Sample Syllabus/Drafts for Review — Word</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="35" t="inlineStr">
         <is>
           <t>Outputs recorded</t>
         </is>
       </c>
-      <c r="B21" s="15">
-        <f>COUNTA($B$5:$B$19)</f>
+      <c r="B24" s="15">
+        <f>COUNTA($B$5:$B$22)</f>
         <v/>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="26" t="inlineStr">
-        <is>
-          <t>Add new rows directly beneath row 19; the count above uses a fixed range, so widen it when you do.</t>
+    <row r="25">
+      <c r="A25" s="26" t="inlineStr">
+        <is>
+          <t>Add new rows directly beneath row 22; the count above uses a fixed range, so widen it when you do.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Course teacher named on every First Year syllabus
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MfWrZ4Zkh7zsRiGVP1SDYc
</commit_message>
<xml_diff>
--- a/CHED 3-Year Trimester Application Tracker.xlsx
+++ b/CHED 3-Year Trimester Application Tracker.xlsx
@@ -24,8 +24,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="dd\-mmm\-yyyy"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -1564,7 +1565,7 @@
       </c>
       <c r="I28" s="7" t="inlineStr">
         <is>
-          <t>ASSESSMENT SCHEME confirmed by the Vice Dean, 3 Sep 2026: two examinations per term (midterm and final), one required monthly assessment, plus regular quizzes and activities. Every syllabus must carry this scheme. CAPACITY RISK: the programme-specialised courses here have no full-time author other than the Chair. 26 Oct 2026: all BSA course syllabi drafted on the OBE template (14-week / 56-hour basis, midterm Week 7, final Week 14) in BSA &amp; BSAIS Outputs/Sample Syllabus/Drafts for Review; references left blank; subject-expert review pending. AE7-INT 400-hour deployment still to be confirmed.</t>
+          <t>ASSESSMENT SCHEME confirmed by the Vice Dean, 3 Sep 2026: two examinations per term (midterm and final), one required monthly assessment, plus regular quizzes and activities. Every syllabus must carry this scheme. CAPACITY RISK: the programme-specialised courses here have no full-time author other than the Chair. 26 Oct 2026: all BSA course syllabi drafted on the OBE template (14-week / 56-hour basis, midterm Week 7, final Week 14) in BSA &amp; BSAIS Outputs/Sample Syllabus/Drafts for Review; references left blank; subject-expert review pending. AE7-INT 400-hour deployment still to be confirmed. 26 Oct 2026: the syllabus drafts now carry the course teacher. Prepared by / Subject Instructor on each of the 24 First Year courses is the faculty member the Proposed Faculty Loading assigns to it — 20 changed from the Vice Dean, 4 were already right. Reviewed by (Chair), Recommended by (Vice Dean) and Approved by (Dean) are unchanged. The 51 Second and Third Year syllabi still read Vice Dean as instructor, because no loading has been drawn for those years yet.</t>
         </is>
       </c>
     </row>
@@ -1810,7 +1811,7 @@
       </c>
       <c r="I34" s="7" t="inlineStr">
         <is>
-          <t>ASSESSMENT SCHEME confirmed by the Vice Dean, 3 Sep 2026: two examinations per term (midterm and final), one required monthly assessment, plus regular quizzes and activities. Every syllabus must carry this scheme. CAPACITY RISK: the programme-specialised courses here have no full-time author other than the Chair. 26 Oct 2026: all BSAIS course syllabi drafted on the OBE template (14-week / 56-hour basis, midterm Week 7, final Week 14) in BSA &amp; BSAIS Outputs/Sample Syllabus/Drafts for Review; references left blank; subject-expert review pending. AE7-INT 400-hour deployment still to be confirmed.</t>
+          <t>ASSESSMENT SCHEME confirmed by the Vice Dean, 3 Sep 2026: two examinations per term (midterm and final), one required monthly assessment, plus regular quizzes and activities. Every syllabus must carry this scheme. CAPACITY RISK: the programme-specialised courses here have no full-time author other than the Chair. 26 Oct 2026: all BSAIS course syllabi drafted on the OBE template (14-week / 56-hour basis, midterm Week 7, final Week 14) in BSA &amp; BSAIS Outputs/Sample Syllabus/Drafts for Review; references left blank; subject-expert review pending. AE7-INT 400-hour deployment still to be confirmed. 26 Oct 2026: the syllabus drafts now carry the course teacher. Prepared by / Subject Instructor on each of the 24 First Year courses is the faculty member the Proposed Faculty Loading assigns to it — 20 changed from the Vice Dean, 4 were already right. Reviewed by (Chair), Recommended by (Vice Dean) and Approved by (Dean) are unchanged. The 51 Second and Third Year syllabi still read Vice Dean as instructor, because no loading has been drawn for those years yet.</t>
         </is>
       </c>
     </row>
@@ -9182,7 +9183,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" style="31" min="1" max="1"/>
@@ -9778,24 +9779,60 @@
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="35" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="4" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Course teacher named on every First Year syllabus — Prepared by / Subject Instructor set from the Proposed Faculty Loading across 24 courses (J.R. Francisco: FAR, CFAS; J.R. Empay: CBME 1, BL1; D.N. Santiago: MGT1; R. Cruz: FINMGT; M. Germino: MAT-GEC, HIS-GEC; N. Tolosa: US-GEC; S.M. Calma: PATH-FIT 1; L. Ramos: NSTP 1 and 2; M. Mequiabas: ART-GEC, PATH-FIT 2 and 3; X. Villamayor: COM-GEC, CON-GEC; F. Ilag: REL-GEC, CLE 1; J. Jamlang: RIZ-GEC; Vice Dean: ECO1, IA1, CAC). Middle initials are missing for most and should be supplied before filing</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Program Chair, BSA &amp; BSAIS</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Items 20, 26</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>For review</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>BSA &amp; BSAIS Outputs/Sample Syllabus and /Drafts for Review</t>
+        </is>
+      </c>
+    </row>
+    <row r="24"/>
+    <row r="25">
+      <c r="A25" s="35" t="inlineStr">
         <is>
           <t>Outputs recorded</t>
         </is>
       </c>
-      <c r="B24" s="15">
-        <f>COUNTA($B$5:$B$22)</f>
+      <c r="B25" s="15">
+        <f>COUNTA($B$5:$B$23)</f>
         <v/>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="26" t="inlineStr">
-        <is>
-          <t>Add new rows directly beneath row 22; the count above uses a fixed range, so widen it when you do.</t>
-        </is>
-      </c>
-    </row>
+    <row r="26">
+      <c r="A26" s="26" t="inlineStr">
+        <is>
+          <t>Add new rows directly beneath row 23; the count above uses a fixed range, so widen it when you do.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>

</xml_diff>

<commit_message>
Add items 81-88 from CHED RO III letter of 7 Oct 2026; extend ranges and assignments
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WkXM4pBNvYNx8JugGmRPAy
</commit_message>
<xml_diff>
--- a/CHED 3-Year Trimester Application Tracker.xlsx
+++ b/CHED 3-Year Trimester Application Tracker.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="My Outputs" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tracker'!$A$4:$I$90</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tracker'!$A$4:$I$99</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Tracker'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Assignments'!$A$4:$E$52</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Faculty'!$A$4:$J$59</definedName>
@@ -24,9 +24,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd\-mmm\-yyyy"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -631,7 +630,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I90"/>
+  <dimension ref="A1:I99"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="31" min="1" max="1"/>
@@ -798,7 +797,7 @@
       </c>
       <c r="I7" s="7" t="inlineStr">
         <is>
-          <t>RESOLVED 3 Sep 2026: there is no prescribed CHED form. It is a compilation the college prepares against each programme's PSG. Corroborated by the CHED Region III Citizen's Charter, which requires a duly accomplished self-evaluation form per programme on submission. Each of the 8 Chairs supplies their own programme's PSG comparison; the Vice Dean consolidates. 21 Sep 2026: BSA and BSAIS self-evaluations (Official and generated copies) now use the "First Year - Trimester 1" naming convention; the builder was updated to write it. 13 Oct 2026: BSA and BSAIS drafts regenerated as v1.1 (curricular finding complete; 40 programme-outcome mappings and the Year 1 teaching-load rows filled). 11 of 17 institutional requirements per programme still outstanding: faculty roster, library, facilities, internship, admission and retention, and the Sec. 20, 22 and 23 systems. 26 Oct 2026: the BSA and BSAIS Year 1 course syllabi that the self-evaluation cites are now drafted (see item 20 and 26).</t>
+          <t>RESOLVED 3 Sep 2026: there is no prescribed CHED form. It is a compilation the college prepares against each programme's PSG. Corroborated by the CHED Region III Citizen's Charter, which requires a duly accomplished self-evaluation form per programme on submission. Each of the 8 Chairs supplies their own programme's PSG comparison; the Vice Dean consolidates. 21 Sep 2026: BSA and BSAIS self-evaluations (Official and generated copies) now use the "First Year - Trimester 1" naming convention; the builder was updated to write it. 13 Oct 2026: BSA and BSAIS drafts regenerated as v1.1 (curricular finding complete; 40 programme-outcome mappings and the Year 1 teaching-load rows filled). 11 of 17 institutional requirements per programme still outstanding: faculty roster, library, facilities, internship, admission and retention, and the Sec. 20, 22 and 23 systems. 26 Oct 2026: the BSA and BSAIS Year 1 course syllabi that the self-evaluation cites are now drafted (see item 20 and 26).  29 Oct 2026: CHED RO III letter of 7 Oct 2026 requires 17–18 contact hours per lecture unit; retest against it. The Official-folder copies still carry the superseded 54-hour, 14-to-15-week wording.</t>
         </is>
       </c>
     </row>
@@ -1059,7 +1058,7 @@
       </c>
       <c r="I14" s="7" t="inlineStr">
         <is>
-          <t>Phase 1 of the project plan calls for the trimestral fee distribution model to be initiated. 23 Sep 2026: a computation workbook is ready for the Finance Office — “BSA/BSAIS 3-Year Trimester — Tuition Computation.xlsx”. Enter the rate per unit, the miscellaneous fee per term, the expense ratios and the tax rate, and tuition, collections, expenses and net income compute for five years. Two decisions are still Finance's: the rates themselves, and whether miscellaneous fees are charged at the same amount per term under a three-term year or annualised across three terms.</t>
+          <t>Phase 1 of the project plan calls for the trimestral fee distribution model to be initiated. 23 Sep 2026: a computation workbook is ready for the Finance Office — “BSA/BSAIS 3-Year Trimester — Tuition Computation.xlsx”. Enter the rate per unit, the miscellaneous fee per term, the expense ratios and the tax rate, and tuition, collections, expenses and net income compute for five years. Two decisions are still Finance's: the rates themselves, and whether miscellaneous fees are charged at the same amount per term under a three-term year or annualised across three terms.  29 Oct 2026: overdue. The CHED RO III letter makes the fee decision the trigger for stakeholder-consultation proof (item 88).</t>
         </is>
       </c>
     </row>
@@ -1565,7 +1564,7 @@
       </c>
       <c r="I28" s="7" t="inlineStr">
         <is>
-          <t>ASSESSMENT SCHEME confirmed by the Vice Dean, 3 Sep 2026: two examinations per term (midterm and final), one required monthly assessment, plus regular quizzes and activities. Every syllabus must carry this scheme. CAPACITY RISK: the programme-specialised courses here have no full-time author other than the Chair. 26 Oct 2026: all BSA course syllabi drafted on the OBE template (14-week / 56-hour basis, midterm Week 7, final Week 14) in BSA &amp; BSAIS Outputs/Sample Syllabus/Drafts for Review; references left blank; subject-expert review pending. AE7-INT 400-hour deployment still to be confirmed. 26 Oct 2026: the syllabus drafts now carry the course teacher. Prepared by / Subject Instructor on each of the 24 First Year courses is the faculty member the Proposed Faculty Loading assigns to it — 20 changed from the Vice Dean, 4 were already right. Reviewed by (Chair), Recommended by (Vice Dean) and Approved by (Dean) are unchanged. The 51 Second and Third Year syllabi still read Vice Dean as instructor, because no loading has been drawn for those years yet.</t>
+          <t>ASSESSMENT SCHEME confirmed by the Vice Dean, 3 Sep 2026: two examinations per term (midterm and final), one required monthly assessment, plus regular quizzes and activities. Every syllabus must carry this scheme. CAPACITY RISK: the programme-specialised courses here have no full-time author other than the Chair. 26 Oct 2026: all BSA course syllabi drafted on the OBE template (14-week / 56-hour basis, midterm Week 7, final Week 14) in BSA &amp; BSAIS Outputs/Sample Syllabus/Drafts for Review; references left blank; subject-expert review pending. AE7-INT 400-hour deployment still to be confirmed. 26 Oct 2026: the syllabus drafts now carry the course teacher. Prepared by / Subject Instructor on each of the 24 First Year courses is the faculty member the Proposed Faculty Loading assigns to it — 20 changed from the Vice Dean, 4 were already right. Reviewed by (Chair), Recommended by (Vice Dean) and Approved by (Dean) are unchanged. The 51 Second and Third Year syllabi still read Vice Dean as instructor, because no loading has been drawn for those years yet.  29 Oct 2026: 64 drafts still have no references; none shows the monthly assessment; instructor sign-off to follow.</t>
         </is>
       </c>
     </row>
@@ -1811,7 +1810,7 @@
       </c>
       <c r="I34" s="7" t="inlineStr">
         <is>
-          <t>ASSESSMENT SCHEME confirmed by the Vice Dean, 3 Sep 2026: two examinations per term (midterm and final), one required monthly assessment, plus regular quizzes and activities. Every syllabus must carry this scheme. CAPACITY RISK: the programme-specialised courses here have no full-time author other than the Chair. 26 Oct 2026: all BSAIS course syllabi drafted on the OBE template (14-week / 56-hour basis, midterm Week 7, final Week 14) in BSA &amp; BSAIS Outputs/Sample Syllabus/Drafts for Review; references left blank; subject-expert review pending. AE7-INT 400-hour deployment still to be confirmed. 26 Oct 2026: the syllabus drafts now carry the course teacher. Prepared by / Subject Instructor on each of the 24 First Year courses is the faculty member the Proposed Faculty Loading assigns to it — 20 changed from the Vice Dean, 4 were already right. Reviewed by (Chair), Recommended by (Vice Dean) and Approved by (Dean) are unchanged. The 51 Second and Third Year syllabi still read Vice Dean as instructor, because no loading has been drawn for those years yet.</t>
+          <t>ASSESSMENT SCHEME confirmed by the Vice Dean, 3 Sep 2026: two examinations per term (midterm and final), one required monthly assessment, plus regular quizzes and activities. Every syllabus must carry this scheme. CAPACITY RISK: the programme-specialised courses here have no full-time author other than the Chair. 26 Oct 2026: all BSAIS course syllabi drafted on the OBE template (14-week / 56-hour basis, midterm Week 7, final Week 14) in BSA &amp; BSAIS Outputs/Sample Syllabus/Drafts for Review; references left blank; subject-expert review pending. AE7-INT 400-hour deployment still to be confirmed. 26 Oct 2026: the syllabus drafts now carry the course teacher. Prepared by / Subject Instructor on each of the 24 First Year courses is the faculty member the Proposed Faculty Loading assigns to it — 20 changed from the Vice Dean, 4 were already right. Reviewed by (Chair), Recommended by (Vice Dean) and Approved by (Dean) are unchanged. The 51 Second and Third Year syllabi still read Vice Dean as instructor, because no loading has been drawn for those years yet.  29 Oct 2026: 64 drafts still have no references; none shows the monthly assessment; instructor sign-off to follow.</t>
         </is>
       </c>
     </row>
@@ -3748,7 +3747,7 @@
       </c>
       <c r="I83" s="7" t="inlineStr">
         <is>
-          <t>Covers Open Items 2 to 5 — the questions only CHED Region III can answer. (Open Item 1, the 14-versus-15-week term length, is for the Council of Chairs, not CHED.) The questions are: which form is meant by 'CHED Program Evaluation'; which issuance governs a shift to trimestral delivery; whether the 3,000 or 5,000 book threshold applies to a conversion of existing programmes; how many hard and soft copies Region III requires; and whether syllabi are needed for every course or only new and re-sequenced ones. The syllabi question is the one that matters most — it drives the 16 October deadline on items 15 to 62, which is why this is dated 25 September.</t>
+          <t>Covers Open Items 2 to 5 — the questions only CHED Region III can answer. (Open Item 1, the 14-versus-15-week term length, is for the Council of Chairs, not CHED.) The questions are: which form is meant by 'CHED Program Evaluation'; which issuance governs a shift to trimestral delivery; whether the 3,000 or 5,000 book threshold applies to a conversion of existing programmes; how many hard and soft copies Region III requires; and whether syllabi are needed for every course or only new and re-sequenced ones. The syllabi question is the one that matters most — it drives the 16 October deadline on items 15 to 62, which is why this is dated 25 September.  29 Oct 2026: the CHED RO III letter (7 Oct) answers question 2 (governing issuances) and partly Open Item 4 (soft copy by email). Send one message to Dr. Maria Teresa S. Salta on the remaining questions; see the audit in BSA &amp; BSAIS Outputs/CHED Letter Audit.</t>
         </is>
       </c>
     </row>
@@ -4039,19 +4038,363 @@
         </is>
       </c>
     </row>
+    <row r="91" ht="15" customHeight="1" s="31">
+      <c r="A91" s="27" t="inlineStr">
+        <is>
+          <t>AREA G — CHED REGION III LETTER OF 7 OCTOBER 2026 (BSA &amp; BSAIS FIRST; other programmes follow once the pattern is approved)</t>
+        </is>
+      </c>
+      <c r="B91" s="28" t="n"/>
+      <c r="C91" s="28" t="n"/>
+      <c r="D91" s="28" t="n"/>
+      <c r="E91" s="28" t="n"/>
+      <c r="F91" s="28" t="n"/>
+      <c r="G91" s="28" t="n"/>
+      <c r="H91" s="28" t="n"/>
+      <c r="I91" s="29" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>81</v>
+      </c>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>Board Resolution approving the institutional shift to a trimester calendar system starting AY 2027–2028</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="inlineStr">
+        <is>
+          <t>CHED RO III letter, 7 Oct 2026, item 1</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="inlineStr">
+        <is>
+          <t>VPAA / VP Admin &amp; Finance Dr. Raquel T. Sta. Ines</t>
+        </is>
+      </c>
+      <c r="E92" s="3" t="inlineStr">
+        <is>
+          <t>Dean Dr. Almario B. Garcia; Vice Dean Ken Gie Anthony G. Cruel (drafts)</t>
+        </is>
+      </c>
+      <c r="F92" s="4" t="n">
+        <v>46330</v>
+      </c>
+      <c r="G92" s="5" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H92" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I92" s="7" t="inlineStr">
+        <is>
+          <t>The letter asks for a Board Resolution. The Council of Program Chairs Resolutions 2026-08-01 to 08-03 are not a Board resolution. Confirm the Letter of Intent dated 25 Aug 2026 is the same document as the item 1 transmittal letter. Council meeting date and resolution number for the 14-week decision still unrecorded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>82</v>
+      </c>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
+          <t>Comparative curriculum matrix, existing 4-year semestral to proposed 3-year trimestral, BSA</t>
+        </is>
+      </c>
+      <c r="C93" s="3" t="inlineStr">
+        <is>
+          <t>CHED RO III letter, 7 Oct 2026, item 2</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="inlineStr">
+        <is>
+          <t>Vice Dean Ken Gie Anthony G. Cruel</t>
+        </is>
+      </c>
+      <c r="E93" s="3" t="inlineStr">
+        <is>
+          <t>Registrar Laila D. Sarmiento (current semestral prospectus by 30 Oct 2026)</t>
+        </is>
+      </c>
+      <c r="F93" s="4" t="n">
+        <v>46329</v>
+      </c>
+      <c r="G93" s="5" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H93" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I93" s="7" t="inlineStr">
+        <is>
+          <t>Must show: required minimum units per PSG preserved; at least 17–18 contact hours per lecture unit over the 14-week term; prerequisite order with no enrolment bottleneck. New curriculum 191 units against the PSG minimum of 173. Blocked until the Registrar supplies the current prospectus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>83</v>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>Comparative curriculum matrix, existing 4-year semestral to proposed 3-year trimestral, BSAIS</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>CHED RO III letter, 7 Oct 2026, item 2</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="inlineStr">
+        <is>
+          <t>Vice Dean Ken Gie Anthony G. Cruel</t>
+        </is>
+      </c>
+      <c r="E94" s="3" t="inlineStr">
+        <is>
+          <t>Registrar Laila D. Sarmiento (current semestral prospectus by 30 Oct 2026)</t>
+        </is>
+      </c>
+      <c r="F94" s="4" t="n">
+        <v>46329</v>
+      </c>
+      <c r="G94" s="5" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H94" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I94" s="7" t="inlineStr">
+        <is>
+          <t>Same test as item 82. New curriculum 185 units against the PSG minimum of 167. Blocked until the Registrar supplies the current prospectus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>84</v>
+      </c>
+      <c r="B95" s="3" t="inlineStr">
+        <is>
+          <t>Academic Calendar AY 2027–2028 with class-day count, midterm and final weeks, inter-trimester breaks and a statement of compliance with annual active instructional days</t>
+        </is>
+      </c>
+      <c r="C95" s="3" t="inlineStr">
+        <is>
+          <t>CHED RO III letter, 7 Oct 2026, item 4</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="inlineStr">
+        <is>
+          <t>Vice Dean Ken Gie Anthony G. Cruel</t>
+        </is>
+      </c>
+      <c r="E95" s="3" t="inlineStr">
+        <is>
+          <t>Registrar Laila D. Sarmiento; MIS Head Jayson R. Francisco</t>
+        </is>
+      </c>
+      <c r="F95" s="4" t="n">
+        <v>46328</v>
+      </c>
+      <c r="G95" s="5" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H95" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I95" s="7" t="inlineStr">
+        <is>
+          <t>The calendar counts 70 days a trimester on a Monday–Friday basis; the adopted pattern is Monday–Thursday (48 regular + 10 exam days = 58). State which days count. The annual minimum is in CMO 1 s.2011 / CMO 40 s.2008, not yet read. Also show the monthly assessment; fix the Term 3 enrolment dates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="B96" s="3" t="inlineStr">
+        <is>
+          <t>Faculty roster and load distribution across all three trimesters with full-time adequacy statement, BSA</t>
+        </is>
+      </c>
+      <c r="C96" s="3" t="inlineStr">
+        <is>
+          <t>CHED RO III letter, 7 Oct 2026, item 5 (first part)</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="inlineStr">
+        <is>
+          <t>Vice Dean Ken Gie Anthony G. Cruel</t>
+        </is>
+      </c>
+      <c r="E96" s="3" t="inlineStr">
+        <is>
+          <t>HR Officer Ellarein Richelle Dela Cruz</t>
+        </is>
+      </c>
+      <c r="F96" s="4" t="n">
+        <v>46329</v>
+      </c>
+      <c r="G96" s="5" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H96" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I96" s="7" t="inlineStr">
+        <is>
+          <t>Current loading covers First Year only: 1 full-time and 12 part-time instructors. CMO 27 Sec 15.5 needs at least 30% full-time and three full-time CPAs. Ask CHED whether the semestral cohorts being taught out must be included.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>86</v>
+      </c>
+      <c r="B97" s="3" t="inlineStr">
+        <is>
+          <t>Faculty roster and load distribution across all three trimesters with full-time adequacy statement, BSAIS</t>
+        </is>
+      </c>
+      <c r="C97" s="3" t="inlineStr">
+        <is>
+          <t>CHED RO III letter, 7 Oct 2026, item 5 (first part)</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="inlineStr">
+        <is>
+          <t>Vice Dean Ken Gie Anthony G. Cruel</t>
+        </is>
+      </c>
+      <c r="E97" s="3" t="inlineStr">
+        <is>
+          <t>HR Officer Ellarein Richelle Dela Cruz</t>
+        </is>
+      </c>
+      <c r="F97" s="4" t="n">
+        <v>46329</v>
+      </c>
+      <c r="G97" s="5" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H97" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I97" s="7" t="inlineStr">
+        <is>
+          <t>Same as item 85. CMO 30 Sec 15.4 applies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="n">
+        <v>87</v>
+      </c>
+      <c r="B98" s="3" t="inlineStr">
+        <is>
+          <t>Room and laboratory utilisation schedule, all programmes, continuous use without conflicts</t>
+        </is>
+      </c>
+      <c r="C98" s="3" t="inlineStr">
+        <is>
+          <t>CHED RO III letter, 7 Oct 2026, item 5 (second part)</t>
+        </is>
+      </c>
+      <c r="D98" s="3" t="inlineStr">
+        <is>
+          <t>MIS Head Jayson R. Francisco</t>
+        </is>
+      </c>
+      <c r="E98" s="3" t="inlineStr">
+        <is>
+          <t>All Program Chairs (their class schedules); VPAA / VP Admin &amp; Finance Dr. Raquel T. Sta. Ines (facilities list)</t>
+        </is>
+      </c>
+      <c r="F98" s="4" t="n">
+        <v>46331</v>
+      </c>
+      <c r="G98" s="5" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H98" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I98" s="7" t="inlineStr">
+        <is>
+          <t>Only First Year BSA/BSAIS classroom assignments exist (ML 401, ML 211). No college-wide room schedule, no laboratory schedule, no facilities inventory against the programme standards.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="n">
+        <v>88</v>
+      </c>
+      <c r="B99" s="3" t="inlineStr">
+        <is>
+          <t>Fee determination and, if fees change, proof of consultation with students, faculty and alumni</t>
+        </is>
+      </c>
+      <c r="C99" s="3" t="inlineStr">
+        <is>
+          <t>CHED RO III letter, 7 Oct 2026, item 6 (CMO 3 s.2012)</t>
+        </is>
+      </c>
+      <c r="D99" s="3" t="inlineStr">
+        <is>
+          <t>VPAA / VP Admin &amp; Finance Dr. Raquel T. Sta. Ines</t>
+        </is>
+      </c>
+      <c r="E99" s="3" t="inlineStr">
+        <is>
+          <t>Finance Officer Dana Marcelo; Vice Dean Ken Gie Anthony G. Cruel (survey data)</t>
+        </is>
+      </c>
+      <c r="F99" s="4" t="n">
+        <v>46332</v>
+      </c>
+      <c r="G99" s="5" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H99" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I99" s="7" t="inlineStr">
+        <is>
+          <t>Determination by 30 Oct 2026: do per-unit tuition or annual miscellaneous fees change? Tuition workbook rates are blank (item 8). The acceptability survey (206 respondents; 6 faculty, 2 alumni) is not a consultation record. Form of proof under CMO 3 s.2012 not yet confirmed.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I90"/>
-  <mergeCells count="8">
+  <autoFilter ref="A4:I99"/>
+  <mergeCells count="9">
     <mergeCell ref="A15:I15"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="A71:I71"/>
     <mergeCell ref="A5:I5"/>
+    <mergeCell ref="A91:I91"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A79:I79"/>
     <mergeCell ref="A8:I8"/>
     <mergeCell ref="A22:I22"/>
   </mergeCells>
-  <conditionalFormatting sqref="A5:I90">
+  <conditionalFormatting sqref="A5:I99">
     <cfRule type="expression" priority="2" dxfId="7">
       <formula>AND(ISNUMBER($F5),$F5&lt;TODAY(),$G5&lt;&gt;"Done")</formula>
     </cfRule>
@@ -4059,7 +4402,7 @@
       <formula>AND(ISNUMBER($F5),$F5&gt;=TODAY(),$F5&lt;=TODAY()+7,$G5&lt;&gt;"Done")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G5:G90">
+  <conditionalFormatting sqref="G5:G99">
     <cfRule type="expression" priority="4" dxfId="2">
       <formula>$G5="Done"</formula>
     </cfRule>
@@ -4071,7 +4414,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G90" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="G5:G99" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Not started,In progress,For review,Done"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4161,16 +4504,16 @@
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>16 items: #2–3, 15–26, 71–72</t>
+          <t>21 items: #2–3, 15–26, 71–72, 82–86</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>53 items: #1, 4, 6, 8–9, 11–12, 27–62, 67, 70, 73–80</t>
+          <t>54 items: #1, 4, 6, 8–9, 11–12, 27–62, 67, 70, 73–80, 88</t>
         </is>
       </c>
       <c r="E6" s="9">
-        <f>IF(COUNTIFS(Tracker!$D$5:$D$90,$A6,Tracker!$G$5:$G$90,"&lt;&gt;Done")=0,"—",_xlfn.MINIFS(Tracker!$F$5:$F$90,Tracker!$D$5:$D$90,$A6,Tracker!$G$5:$G$90,"&lt;&gt;Done"))</f>
+        <f>IF(COUNTIFS(Tracker!$D$5:$D$99,$A6,Tracker!$G$5:$G$99,"&lt;&gt;Done")=0,"—",_xlfn.MINIFS(Tracker!$F$5:$F$99,Tracker!$D$5:$D$99,$A6,Tracker!$G$5:$G$99,"&lt;&gt;Done"))</f>
         <v/>
       </c>
     </row>
@@ -4187,16 +4530,16 @@
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>6 items: #1, 4–6, 70, 73</t>
+          <t>7 items: #1, 4–6, 70, 73, 87</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>50 items: #7, 15–62, 72</t>
+          <t>51 items: #7, 15–62, 72, 84</t>
         </is>
       </c>
       <c r="E7" s="9">
-        <f>IF(COUNTIFS(Tracker!$D$5:$D$90,$A7,Tracker!$G$5:$G$90,"&lt;&gt;Done")=0,"—",_xlfn.MINIFS(Tracker!$F$5:$F$90,Tracker!$D$5:$D$90,$A7,Tracker!$G$5:$G$90,"&lt;&gt;Done"))</f>
+        <f>IF(COUNTIFS(Tracker!$D$5:$D$99,$A7,Tracker!$G$5:$G$99,"&lt;&gt;Done")=0,"—",_xlfn.MINIFS(Tracker!$F$5:$F$99,Tracker!$D$5:$D$99,$A7,Tracker!$G$5:$G$99,"&lt;&gt;Done"))</f>
         <v/>
       </c>
     </row>
@@ -4213,16 +4556,16 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>2 items: #7, 14</t>
+          <t>4 items: #7, 14, 81, 88</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>7 items: #1, 3, 10, 13, 64–65, 71</t>
+          <t>8 items: #1, 3, 10, 13, 64–65, 71, 87</t>
         </is>
       </c>
       <c r="E8" s="4">
-        <f>IF(COUNTIFS(Tracker!$D$5:$D$90,$A8,Tracker!$G$5:$G$90,"&lt;&gt;Done")=0,"—",_xlfn.MINIFS(Tracker!$F$5:$F$90,Tracker!$D$5:$D$90,$A8,Tracker!$G$5:$G$90,"&lt;&gt;Done"))</f>
+        <f>IF(COUNTIFS(Tracker!$D$5:$D$99,$A8,Tracker!$G$5:$G$99,"&lt;&gt;Done")=0,"—",_xlfn.MINIFS(Tracker!$F$5:$F$99,Tracker!$D$5:$D$99,$A8,Tracker!$G$5:$G$99,"&lt;&gt;Done"))</f>
         <v/>
       </c>
     </row>
@@ -4244,11 +4587,11 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>1 item: #71</t>
+          <t>2 items: #71, 81</t>
         </is>
       </c>
       <c r="E9" s="4">
-        <f>IF(COUNTIFS(Tracker!$D$5:$D$90,$A9,Tracker!$G$5:$G$90,"&lt;&gt;Done")=0,"—",_xlfn.MINIFS(Tracker!$F$5:$F$90,Tracker!$D$5:$D$90,$A9,Tracker!$G$5:$G$90,"&lt;&gt;Done"))</f>
+        <f>IF(COUNTIFS(Tracker!$D$5:$D$99,$A9,Tracker!$G$5:$G$99,"&lt;&gt;Done")=0,"—",_xlfn.MINIFS(Tracker!$F$5:$F$99,Tracker!$D$5:$D$99,$A9,Tracker!$G$5:$G$99,"&lt;&gt;Done"))</f>
         <v/>
       </c>
     </row>
@@ -4270,11 +4613,11 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>2 items: #14, 63</t>
+          <t>4 items: #14, 63, 85–86</t>
         </is>
       </c>
       <c r="E10" s="4">
-        <f>IF(COUNTIFS(Tracker!$D$5:$D$90,$A10,Tracker!$G$5:$G$90,"&lt;&gt;Done")=0,"—",_xlfn.MINIFS(Tracker!$F$5:$F$90,Tracker!$D$5:$D$90,$A10,Tracker!$G$5:$G$90,"&lt;&gt;Done"))</f>
+        <f>IF(COUNTIFS(Tracker!$D$5:$D$99,$A10,Tracker!$G$5:$G$99,"&lt;&gt;Done")=0,"—",_xlfn.MINIFS(Tracker!$F$5:$F$99,Tracker!$D$5:$D$99,$A10,Tracker!$G$5:$G$99,"&lt;&gt;Done"))</f>
         <v/>
       </c>
     </row>
@@ -4300,7 +4643,7 @@
         </is>
       </c>
       <c r="E11" s="4">
-        <f>IF(COUNTIFS(Tracker!$D$5:$D$90,$A11,Tracker!$G$5:$G$90,"&lt;&gt;Done")=0,"—",_xlfn.MINIFS(Tracker!$F$5:$F$90,Tracker!$D$5:$D$90,$A11,Tracker!$G$5:$G$90,"&lt;&gt;Done"))</f>
+        <f>IF(COUNTIFS(Tracker!$D$5:$D$99,$A11,Tracker!$G$5:$G$99,"&lt;&gt;Done")=0,"—",_xlfn.MINIFS(Tracker!$F$5:$F$99,Tracker!$D$5:$D$99,$A11,Tracker!$G$5:$G$99,"&lt;&gt;Done"))</f>
         <v/>
       </c>
     </row>
@@ -4322,11 +4665,11 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>6 items: #2, 4, 6, 11–12, 67</t>
+          <t>7 items: #2, 4, 6, 11–12, 67, 87</t>
         </is>
       </c>
       <c r="E12" s="4">
-        <f>IF(COUNTIFS(Tracker!$D$5:$D$90,$A12,Tracker!$G$5:$G$90,"&lt;&gt;Done")=0,"—",_xlfn.MINIFS(Tracker!$F$5:$F$90,Tracker!$D$5:$D$90,$A12,Tracker!$G$5:$G$90,"&lt;&gt;Done"))</f>
+        <f>IF(COUNTIFS(Tracker!$D$5:$D$99,$A12,Tracker!$G$5:$G$99,"&lt;&gt;Done")=0,"—",_xlfn.MINIFS(Tracker!$F$5:$F$99,Tracker!$D$5:$D$99,$A12,Tracker!$G$5:$G$99,"&lt;&gt;Done"))</f>
         <v/>
       </c>
     </row>
@@ -4348,11 +4691,11 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>7 items: #2, 4, 6, 11–12, 67, 74</t>
+          <t>8 items: #2, 4, 6, 11–12, 67, 74, 87</t>
         </is>
       </c>
       <c r="E13" s="4">
-        <f>IF(COUNTIFS(Tracker!$D$5:$D$90,$A13,Tracker!$G$5:$G$90,"&lt;&gt;Done")=0,"—",_xlfn.MINIFS(Tracker!$F$5:$F$90,Tracker!$D$5:$D$90,$A13,Tracker!$G$5:$G$90,"&lt;&gt;Done"))</f>
+        <f>IF(COUNTIFS(Tracker!$D$5:$D$99,$A13,Tracker!$G$5:$G$99,"&lt;&gt;Done")=0,"—",_xlfn.MINIFS(Tracker!$F$5:$F$99,Tracker!$D$5:$D$99,$A13,Tracker!$G$5:$G$99,"&lt;&gt;Done"))</f>
         <v/>
       </c>
     </row>
@@ -4374,11 +4717,11 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>7 items: #2, 4, 6, 11–12, 67, 74</t>
+          <t>8 items: #2, 4, 6, 11–12, 67, 74, 87</t>
         </is>
       </c>
       <c r="E14" s="4">
-        <f>IF(COUNTIFS(Tracker!$D$5:$D$90,$A14,Tracker!$G$5:$G$90,"&lt;&gt;Done")=0,"—",_xlfn.MINIFS(Tracker!$F$5:$F$90,Tracker!$D$5:$D$90,$A14,Tracker!$G$5:$G$90,"&lt;&gt;Done"))</f>
+        <f>IF(COUNTIFS(Tracker!$D$5:$D$99,$A14,Tracker!$G$5:$G$99,"&lt;&gt;Done")=0,"—",_xlfn.MINIFS(Tracker!$F$5:$F$99,Tracker!$D$5:$D$99,$A14,Tracker!$G$5:$G$99,"&lt;&gt;Done"))</f>
         <v/>
       </c>
     </row>
@@ -4400,11 +4743,11 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>8 items: #2, 4, 6, 11–12, 67, 74–75</t>
+          <t>9 items: #2, 4, 6, 11–12, 67, 74–75, 87</t>
         </is>
       </c>
       <c r="E15" s="4">
-        <f>IF(COUNTIFS(Tracker!$D$5:$D$90,$A15,Tracker!$G$5:$G$90,"&lt;&gt;Done")=0,"—",_xlfn.MINIFS(Tracker!$F$5:$F$90,Tracker!$D$5:$D$90,$A15,Tracker!$G$5:$G$90,"&lt;&gt;Done"))</f>
+        <f>IF(COUNTIFS(Tracker!$D$5:$D$99,$A15,Tracker!$G$5:$G$99,"&lt;&gt;Done")=0,"—",_xlfn.MINIFS(Tracker!$F$5:$F$99,Tracker!$D$5:$D$99,$A15,Tracker!$G$5:$G$99,"&lt;&gt;Done"))</f>
         <v/>
       </c>
     </row>
@@ -4426,11 +4769,11 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>7 items: #2, 4, 6, 11–12, 67, 74</t>
+          <t>8 items: #2, 4, 6, 11–12, 67, 74, 87</t>
         </is>
       </c>
       <c r="E16" s="4">
-        <f>IF(COUNTIFS(Tracker!$D$5:$D$90,$A16,Tracker!$G$5:$G$90,"&lt;&gt;Done")=0,"—",_xlfn.MINIFS(Tracker!$F$5:$F$90,Tracker!$D$5:$D$90,$A16,Tracker!$G$5:$G$90,"&lt;&gt;Done"))</f>
+        <f>IF(COUNTIFS(Tracker!$D$5:$D$99,$A16,Tracker!$G$5:$G$99,"&lt;&gt;Done")=0,"—",_xlfn.MINIFS(Tracker!$F$5:$F$99,Tracker!$D$5:$D$99,$A16,Tracker!$G$5:$G$99,"&lt;&gt;Done"))</f>
         <v/>
       </c>
     </row>
@@ -4452,11 +4795,11 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1 item: #88</t>
         </is>
       </c>
       <c r="E17" s="4">
-        <f>IF(COUNTIFS(Tracker!$D$5:$D$90,$A17,Tracker!$G$5:$G$90,"&lt;&gt;Done")=0,"—",_xlfn.MINIFS(Tracker!$F$5:$F$90,Tracker!$D$5:$D$90,$A17,Tracker!$G$5:$G$90,"&lt;&gt;Done"))</f>
+        <f>IF(COUNTIFS(Tracker!$D$5:$D$99,$A17,Tracker!$G$5:$G$99,"&lt;&gt;Done")=0,"—",_xlfn.MINIFS(Tracker!$F$5:$F$99,Tracker!$D$5:$D$99,$A17,Tracker!$G$5:$G$99,"&lt;&gt;Done"))</f>
         <v/>
       </c>
     </row>
@@ -4478,11 +4821,11 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>1 item: #5</t>
+          <t>4 items: #5, 82–84</t>
         </is>
       </c>
       <c r="E18" s="4">
-        <f>IF(COUNTIFS(Tracker!$D$5:$D$90,$A18,Tracker!$G$5:$G$90,"&lt;&gt;Done")=0,"—",_xlfn.MINIFS(Tracker!$F$5:$F$90,Tracker!$D$5:$D$90,$A18,Tracker!$G$5:$G$90,"&lt;&gt;Done"))</f>
+        <f>IF(COUNTIFS(Tracker!$D$5:$D$99,$A18,Tracker!$G$5:$G$99,"&lt;&gt;Done")=0,"—",_xlfn.MINIFS(Tracker!$F$5:$F$99,Tracker!$D$5:$D$99,$A18,Tracker!$G$5:$G$99,"&lt;&gt;Done"))</f>
         <v/>
       </c>
     </row>
@@ -5388,7 +5731,7 @@
         </is>
       </c>
       <c r="B60" s="15">
-        <f>COUNT(Tracker!$A$5:$A$90)&amp;" tracker items, each with exactly one accountable owner. "&amp;COUNTIF(Faculty!$E$5:$E$59,"FT")&amp;" full-time faculty tasked; "&amp;COUNTIF(Faculty!$E$5:$E$59,"PT")&amp;" part-time faculty not tasked."</f>
+        <f>COUNT(Tracker!$A$5:$A$99)&amp;" tracker items, each with exactly one accountable owner. "&amp;COUNTIF(Faculty!$E$5:$E$59,"FT")&amp;" full-time faculty tasked; "&amp;COUNTIF(Faculty!$E$5:$E$59,"PT")&amp;" part-time faculty not tasked."</f>
         <v/>
       </c>
     </row>
@@ -5417,7 +5760,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B102"/>
+  <dimension ref="A1:B109"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" style="31" min="1" max="1"/>
@@ -6276,7 +6619,7 @@
         </is>
       </c>
       <c r="B84" s="19">
-        <f>COUNT(Tracker!$A$5:$A$90)</f>
+        <f>COUNT(Tracker!$A$5:$A$99)</f>
         <v/>
       </c>
     </row>
@@ -6287,7 +6630,7 @@
         </is>
       </c>
       <c r="B85" s="19">
-        <f>COUNTIF(Tracker!$G$5:$G$90,"Not started")</f>
+        <f>COUNTIF(Tracker!$G$5:$G$99,"Not started")</f>
         <v/>
       </c>
     </row>
@@ -6298,7 +6641,7 @@
         </is>
       </c>
       <c r="B86" s="19">
-        <f>COUNTIF(Tracker!$G$5:$G$90,"In progress")</f>
+        <f>COUNTIF(Tracker!$G$5:$G$99,"In progress")</f>
         <v/>
       </c>
     </row>
@@ -6309,7 +6652,7 @@
         </is>
       </c>
       <c r="B87" s="19">
-        <f>COUNTIF(Tracker!$G$5:$G$90,"For review")</f>
+        <f>COUNTIF(Tracker!$G$5:$G$99,"For review")</f>
         <v/>
       </c>
     </row>
@@ -6320,7 +6663,7 @@
         </is>
       </c>
       <c r="B88" s="19">
-        <f>COUNTIF(Tracker!$G$5:$G$90,"Done")</f>
+        <f>COUNTIF(Tracker!$G$5:$G$99,"Done")</f>
         <v/>
       </c>
     </row>
@@ -6331,7 +6674,7 @@
         </is>
       </c>
       <c r="B89" s="20">
-        <f>IFERROR(AVERAGE(Tracker!$H$5:$H$90),0)</f>
+        <f>IFERROR(AVERAGE(Tracker!$H$5:$H$99),0)</f>
         <v/>
       </c>
     </row>
@@ -6342,7 +6685,7 @@
         </is>
       </c>
       <c r="B90" s="19">
-        <f>COUNTIFS(Tracker!$F$5:$F$90,"&lt;"&amp;TODAY(),Tracker!$G$5:$G$90,"&lt;&gt;Done")</f>
+        <f>COUNTIFS(Tracker!$F$5:$F$99,"&lt;"&amp;TODAY(),Tracker!$G$5:$G$99,"&lt;&gt;Done")</f>
         <v/>
       </c>
     </row>
@@ -6353,7 +6696,7 @@
         </is>
       </c>
       <c r="B91" s="19">
-        <f>COUNTIFS(Tracker!$F$5:$F$90,"&gt;="&amp;TODAY(),Tracker!$F$5:$F$90,"&lt;="&amp;TODAY()+7,Tracker!$G$5:$G$90,"&lt;&gt;Done")</f>
+        <f>COUNTIFS(Tracker!$F$5:$F$99,"&gt;="&amp;TODAY(),Tracker!$F$5:$F$99,"&lt;="&amp;TODAY()+7,Tracker!$G$5:$G$99,"&lt;&gt;Done")</f>
         <v/>
       </c>
     </row>
@@ -6466,7 +6809,75 @@
       </c>
       <c r="B102" s="3" t="inlineStr">
         <is>
-          <t>Every one of the 80 items has exactly one accountable owner. Faculty and committees are support — they contribute the work, but the named owner answers for delivery. All five working bodies have a named lead: the eight Curriculum &amp; Syllabi Committees (each Programme Chair), the Library Collection Committee (Pastrana), the Feasibility &amp; Market Study Committee (Francisco) and the two college-wide pools (K. Garcia and Castillo). Since 13 September 2026 every full-time faculty member also carries a named specific task in the Specific task assigned column of the Faculty sheet — the 12 pool writers by course, the other 15 as a counted task pending their Chair's allocation under items 76 to 80.</t>
+          <t>Every one of the 88 items has exactly one accountable owner. Faculty and committees are support — they contribute the work, but the named owner answers for delivery. All five working bodies have a named lead: the eight Curriculum &amp; Syllabi Committees (each Programme Chair), the Library Collection Committee (Pastrana), the Feasibility &amp; Market Study Committee (Francisco) and the two college-wide pools (K. Garcia and Castillo). Since 13 September 2026 every full-time faculty member also carries a named specific task in the Specific task assigned column of the Faculty sheet — the 12 pool writers by course, the other 15 as a counted task pending their Chair's allocation under items 76 to 80.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="27" t="inlineStr">
+        <is>
+          <t>I. CHED REGION III LETTER OF 7 OCTOBER 2026 (Office Tracking #10-0887)</t>
+        </is>
+      </c>
+      <c r="B104" s="29" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="17" t="inlineStr">
+        <is>
+          <t>What it is</t>
+        </is>
+      </c>
+      <c r="B105" s="3" t="inlineStr">
+        <is>
+          <t>Official reply of CHED Regional Office III to the Letter of Intent dated 25 Aug 2026 (received 1 Oct 2026). Signed by Director IV Maura Consolacion D. Cristobal, Ed.D., CESO III. Images: College-Wide Outputs/CHED RO III Letter 2026-10-07. Contact: Dr. Maria Teresa S. Salta, 0964-830-2194, chedro3@ched.gov.ph.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="17" t="inlineStr">
+        <is>
+          <t>Six documents it asks for (soft copy to chedro3@ched.gov.ph)</t>
+        </is>
+      </c>
+      <c r="B106" s="3" t="inlineStr">
+        <is>
+          <t>1 Board Resolution (item 81) · 2 Comparative curriculum matrices (items 82–83 and the other six programmes) · 3 Syllabi adjusted to the 14-week term (items 20, 26 and the other programmes) · 4 Academic Calendar (item 84) · 5 Resource Capability Inventory: faculty roster and load, room and laboratory schedules (items 85–87) · 6 Proof of stakeholder consultations if fees are restructured (item 88).</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="17" t="inlineStr">
+        <is>
+          <t>Issuances it cites (texts NOT yet read)</t>
+        </is>
+      </c>
+      <c r="B107" s="3" t="inlineStr">
+        <is>
+          <t>CMO 1 s.2011 (school calendar) · CMO 40 s.2008 (Manual of Regulations, Private HEIs) · each programme’s PSG · CMO 3 s.2012 (tuition and other school fees).</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="17" t="inlineStr">
+        <is>
+          <t>Contact-hour standard it states</t>
+        </is>
+      </c>
+      <c r="B108" s="3" t="inlineStr">
+        <is>
+          <t>At least 17–18 contact hours per lecture unit across the planned 14-week term. 56 hours per 3-unit subject is 18.67 per unit. Counting only the 12 teaching weeks it is 16.0. Laboratory units need a stated convention.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="17" t="inlineStr">
+        <is>
+          <t>Effect on open items</t>
+        </is>
+      </c>
+      <c r="B109" s="3" t="inlineStr">
+        <is>
+          <t>Item 73 question 2 answered. Open Item 4 partly answered (soft copy by email; no binders mentioned). Open Item 5 reads as every course. Open Item 2 still needs CHED to confirm that the six documents are the whole list.</t>
         </is>
       </c>
     </row>
@@ -9183,7 +9594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" style="31" min="1" max="1"/>
@@ -9809,7 +10220,6 @@
         </is>
       </c>
     </row>
-    <row r="24"/>
     <row r="25">
       <c r="A25" s="35" t="inlineStr">
         <is>
@@ -9828,11 +10238,6 @@
         </is>
       </c>
     </row>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>

</xml_diff>

<commit_message>
Item 84 to For review; notes on monthly assessment
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WkXM4pBNvYNx8JugGmRPAy
</commit_message>
<xml_diff>
--- a/CHED 3-Year Trimester Application Tracker.xlsx
+++ b/CHED 3-Year Trimester Application Tracker.xlsx
@@ -1564,7 +1564,7 @@
       </c>
       <c r="I28" s="7" t="inlineStr">
         <is>
-          <t>ASSESSMENT SCHEME confirmed by the Vice Dean, 3 Sep 2026: two examinations per term (midterm and final), one required monthly assessment, plus regular quizzes and activities. Every syllabus must carry this scheme. CAPACITY RISK: the programme-specialised courses here have no full-time author other than the Chair. 26 Oct 2026: all BSA course syllabi drafted on the OBE template (14-week / 56-hour basis, midterm Week 7, final Week 14) in BSA &amp; BSAIS Outputs/Sample Syllabus/Drafts for Review; references left blank; subject-expert review pending. AE7-INT 400-hour deployment still to be confirmed. 26 Oct 2026: the syllabus drafts now carry the course teacher. Prepared by / Subject Instructor on each of the 24 First Year courses is the faculty member the Proposed Faculty Loading assigns to it — 20 changed from the Vice Dean, 4 were already right. Reviewed by (Chair), Recommended by (Vice Dean) and Approved by (Dean) are unchanged. The 51 Second and Third Year syllabi still read Vice Dean as instructor, because no loading has been drawn for those years yet.  29 Oct 2026: 64 drafts still have no references; none shows the monthly assessment; instructor sign-off to follow.</t>
+          <t>ASSESSMENT SCHEME confirmed by the Vice Dean, 3 Sep 2026: two examinations per term (midterm and final), one required monthly assessment, plus regular quizzes and activities. Every syllabus must carry this scheme. CAPACITY RISK: the programme-specialised courses here have no full-time author other than the Chair. 26 Oct 2026: all BSA course syllabi drafted on the OBE template (14-week / 56-hour basis, midterm Week 7, final Week 14) in BSA &amp; BSAIS Outputs/Sample Syllabus/Drafts for Review; references left blank; subject-expert review pending. AE7-INT 400-hour deployment still to be confirmed. 26 Oct 2026: the syllabus drafts now carry the course teacher. Prepared by / Subject Instructor on each of the 24 First Year courses is the faculty member the Proposed Faculty Loading assigns to it — 20 changed from the Vice Dean, 4 were already right. Reviewed by (Chair), Recommended by (Vice Dean) and Approved by (Dean) are unchanged. The 51 Second and Third Year syllabi still read Vice Dean as instructor, because no loading has been drawn for those years yet.  29 Oct 2026: 64 drafts still have no references; none shows the monthly assessment; instructor sign-off to follow.  Update 29 Oct 2026: monthly assessment (Weeks 4 and 11) added to all 74 syllabi. References still outstanding on 64 drafts.</t>
         </is>
       </c>
     </row>
@@ -1810,7 +1810,7 @@
       </c>
       <c r="I34" s="7" t="inlineStr">
         <is>
-          <t>ASSESSMENT SCHEME confirmed by the Vice Dean, 3 Sep 2026: two examinations per term (midterm and final), one required monthly assessment, plus regular quizzes and activities. Every syllabus must carry this scheme. CAPACITY RISK: the programme-specialised courses here have no full-time author other than the Chair. 26 Oct 2026: all BSAIS course syllabi drafted on the OBE template (14-week / 56-hour basis, midterm Week 7, final Week 14) in BSA &amp; BSAIS Outputs/Sample Syllabus/Drafts for Review; references left blank; subject-expert review pending. AE7-INT 400-hour deployment still to be confirmed. 26 Oct 2026: the syllabus drafts now carry the course teacher. Prepared by / Subject Instructor on each of the 24 First Year courses is the faculty member the Proposed Faculty Loading assigns to it — 20 changed from the Vice Dean, 4 were already right. Reviewed by (Chair), Recommended by (Vice Dean) and Approved by (Dean) are unchanged. The 51 Second and Third Year syllabi still read Vice Dean as instructor, because no loading has been drawn for those years yet.  29 Oct 2026: 64 drafts still have no references; none shows the monthly assessment; instructor sign-off to follow.</t>
+          <t>ASSESSMENT SCHEME confirmed by the Vice Dean, 3 Sep 2026: two examinations per term (midterm and final), one required monthly assessment, plus regular quizzes and activities. Every syllabus must carry this scheme. CAPACITY RISK: the programme-specialised courses here have no full-time author other than the Chair. 26 Oct 2026: all BSAIS course syllabi drafted on the OBE template (14-week / 56-hour basis, midterm Week 7, final Week 14) in BSA &amp; BSAIS Outputs/Sample Syllabus/Drafts for Review; references left blank; subject-expert review pending. AE7-INT 400-hour deployment still to be confirmed. 26 Oct 2026: the syllabus drafts now carry the course teacher. Prepared by / Subject Instructor on each of the 24 First Year courses is the faculty member the Proposed Faculty Loading assigns to it — 20 changed from the Vice Dean, 4 were already right. Reviewed by (Chair), Recommended by (Vice Dean) and Approved by (Dean) are unchanged. The 51 Second and Third Year syllabi still read Vice Dean as instructor, because no loading has been drawn for those years yet.  29 Oct 2026: 64 drafts still have no references; none shows the monthly assessment; instructor sign-off to follow.  Update 29 Oct 2026: monthly assessment (Weeks 4 and 11) added to all 74 syllabi. References still outstanding on 64 drafts.</t>
         </is>
       </c>
     </row>
@@ -4205,15 +4205,15 @@
       </c>
       <c r="G95" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>For review</t>
         </is>
       </c>
       <c r="H95" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I95" s="7" t="inlineStr">
         <is>
-          <t>The calendar counts 70 days a trimester on a Monday–Friday basis; the adopted pattern is Monday–Thursday (48 regular + 10 exam days = 58). State which days count. The annual minimum is in CMO 1 s.2011 / CMO 40 s.2008, not yet read. Also show the monthly assessment; fix the Term 3 enrolment dates.</t>
+          <t>The calendar counts 70 days a trimester on a Monday–Friday basis; the adopted pattern is Monday–Thursday (48 regular + 10 exam days = 58). State which days count. The annual minimum is in CMO 1 s.2011 / CMO 40 s.2008, not yet read. Also show the monthly assessment; fix the Term 3 enrolment dates.  29 Oct 2026: calendar revised and re-issued (HTML and PDF): Monday–Thursday count of 48 class + 10 exam = 58 days a trimester (174 a year); monthly assessment in Weeks 4 and 11; Term 3 enrolment moved to 14–16 Feb 2028. Still open: statement of compliance with the annual minimum (CMO 1 s.2011 / CMO 40 s.2008 not yet read); workbook sheet School Calendar is stale.</t>
         </is>
       </c>
     </row>

</xml_diff>